<commit_message>
Se agrega notebook de la fase 2
</commit_message>
<xml_diff>
--- a/data/raw/io_data_bimbo.xlsx
+++ b/data/raw/io_data_bimbo.xlsx
@@ -14578,84 +14578,761 @@
       </c>
     </row>
     <row r="489" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H489" s="12"/>
+      <c r="A489" s="6" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B489" s="7" t="n">
+        <v>7608</v>
+      </c>
+      <c r="C489" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D489" s="8" t="n">
+        <v>0.0833333333333333</v>
+      </c>
+      <c r="E489" s="9" t="n">
+        <v>0.708738425925926</v>
+      </c>
+      <c r="F489" s="9" t="n">
+        <v>0.7165625</v>
+      </c>
+      <c r="G489" s="9" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H489" s="0" t="n">
+        <v>136</v>
+      </c>
+      <c r="I489" s="10" t="n">
+        <v>805931</v>
+      </c>
     </row>
     <row r="490" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H490" s="12"/>
+      <c r="A490" s="6" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B490" s="7" t="n">
+        <v>7613</v>
+      </c>
+      <c r="C490" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D490" s="8" t="n">
+        <v>0.0833333333333333</v>
+      </c>
+      <c r="E490" s="9" t="n">
+        <v>0.717731481481482</v>
+      </c>
+      <c r="F490" s="9" t="n">
+        <v>0.732037037037037</v>
+      </c>
+      <c r="G490" s="9" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H490" s="10" t="n">
+        <v>632</v>
+      </c>
+      <c r="I490" s="10" t="n">
+        <v>3260364</v>
+      </c>
     </row>
     <row r="491" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H491" s="12"/>
+      <c r="A491" s="6" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B491" s="7" t="n">
+        <v>7628</v>
+      </c>
+      <c r="C491" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D491" s="8" t="n">
+        <v>0.0833333333333333</v>
+      </c>
+      <c r="E491" s="9" t="n">
+        <v>0.733506944444444</v>
+      </c>
+      <c r="F491" s="9" t="n">
+        <v>0.74150462962963</v>
+      </c>
+      <c r="G491" s="9" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H491" s="10" t="n">
+        <v>301</v>
+      </c>
+      <c r="I491" s="10" t="n">
+        <v>1486681</v>
+      </c>
     </row>
     <row r="492" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H492" s="12"/>
+      <c r="A492" s="6" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B492" s="7" t="n">
+        <v>7641</v>
+      </c>
+      <c r="C492" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D492" s="8" t="n">
+        <v>0.0833333333333333</v>
+      </c>
+      <c r="E492" s="9" t="n">
+        <v>0.742708333333333</v>
+      </c>
+      <c r="F492" s="9" t="n">
+        <v>0.752731481481482</v>
+      </c>
+      <c r="G492" s="9" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H492" s="10" t="n">
+        <v>241</v>
+      </c>
+      <c r="I492" s="10" t="n">
+        <v>1441321</v>
+      </c>
     </row>
     <row r="493" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H493" s="12"/>
+      <c r="A493" s="6" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B493" s="7" t="n">
+        <v>7648</v>
+      </c>
+      <c r="C493" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D493" s="8" t="n">
+        <v>0.0833333333333333</v>
+      </c>
+      <c r="E493" s="9" t="n">
+        <v>0.784583333333333</v>
+      </c>
+      <c r="F493" s="9" t="n">
+        <v>0.791770833333333</v>
+      </c>
+      <c r="G493" s="9" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H493" s="10" t="n">
+        <v>129</v>
+      </c>
+      <c r="I493" s="10" t="n">
+        <v>779901</v>
+      </c>
     </row>
     <row r="494" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H494" s="12"/>
+      <c r="A494" s="6" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B494" s="7" t="n">
+        <v>7653</v>
+      </c>
+      <c r="C494" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D494" s="8" t="n">
+        <v>0.0833333333333333</v>
+      </c>
+      <c r="E494" s="9" t="n">
+        <v>0.811354166666667</v>
+      </c>
+      <c r="F494" s="9" t="n">
+        <v>0.824305555555556</v>
+      </c>
+      <c r="G494" s="9" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H494" s="10" t="n">
+        <v>386</v>
+      </c>
+      <c r="I494" s="10" t="n">
+        <v>1968022</v>
+      </c>
     </row>
     <row r="495" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H495" s="12"/>
+      <c r="A495" s="6" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B495" s="7" t="n">
+        <v>7655</v>
+      </c>
+      <c r="C495" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D495" s="8" t="n">
+        <v>0.0833333333333333</v>
+      </c>
+      <c r="E495" s="9" t="n">
+        <v>0.804085648148148</v>
+      </c>
+      <c r="F495" s="9" t="n">
+        <v>0.810509259259259</v>
+      </c>
+      <c r="G495" s="9" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H495" s="10" t="n">
+        <v>108</v>
+      </c>
+      <c r="I495" s="10" t="n">
+        <v>588067</v>
+      </c>
     </row>
     <row r="496" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H496" s="12"/>
+      <c r="A496" s="6" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B496" s="7" t="n">
+        <v>7656</v>
+      </c>
+      <c r="C496" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D496" s="8" t="n">
+        <v>0.0833333333333333</v>
+      </c>
+      <c r="E496" s="9" t="n">
+        <v>0.792696759259259</v>
+      </c>
+      <c r="F496" s="9" t="n">
+        <v>0.802916666666667</v>
+      </c>
+      <c r="G496" s="9" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H496" s="10" t="n">
+        <v>318</v>
+      </c>
+      <c r="I496" s="10" t="n">
+        <v>1685607</v>
+      </c>
     </row>
     <row r="497" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H497" s="12"/>
+      <c r="A497" s="6" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B497" s="7" t="n">
+        <v>7670</v>
+      </c>
+      <c r="C497" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D497" s="8" t="n">
+        <v>0.0833333333333333</v>
+      </c>
+      <c r="E497" s="9" t="n">
+        <v>0.826041666666667</v>
+      </c>
+      <c r="F497" s="9" t="n">
+        <v>0.833148148148148</v>
+      </c>
+      <c r="G497" s="9" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H497" s="10" t="n">
+        <v>110</v>
+      </c>
+      <c r="I497" s="10" t="n">
+        <v>590962</v>
+      </c>
     </row>
     <row r="498" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H498" s="12"/>
+      <c r="A498" s="6" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B498" s="7" t="n">
+        <v>7676</v>
+      </c>
+      <c r="C498" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D498" s="8" t="n">
+        <v>0.0833333333333333</v>
+      </c>
+      <c r="E498" s="9" t="n">
+        <v>0.834085648148148</v>
+      </c>
+      <c r="F498" s="9" t="n">
+        <v>0.844641203703704</v>
+      </c>
+      <c r="G498" s="9" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H498" s="10" t="n">
+        <v>285</v>
+      </c>
+      <c r="I498" s="10" t="n">
+        <v>1658355</v>
+      </c>
     </row>
     <row r="499" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H499" s="12"/>
+      <c r="A499" s="6" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B499" s="7" t="n">
+        <v>7704</v>
+      </c>
+      <c r="C499" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D499" s="8" t="n">
+        <v>0.0833333333333333</v>
+      </c>
+      <c r="E499" s="9" t="n">
+        <v>0.84650462962963</v>
+      </c>
+      <c r="F499" s="9" t="n">
+        <v>0.851377314814815</v>
+      </c>
+      <c r="G499" s="9" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H499" s="10" t="n">
+        <v>96</v>
+      </c>
+      <c r="I499" s="10" t="n">
+        <v>399868</v>
+      </c>
     </row>
     <row r="500" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H500" s="12"/>
+      <c r="A500" s="6" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B500" s="7" t="n">
+        <v>7709</v>
+      </c>
+      <c r="C500" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D500" s="8" t="n">
+        <v>0.0833333333333333</v>
+      </c>
+      <c r="E500" s="9" t="n">
+        <v>0.852361111111111</v>
+      </c>
+      <c r="F500" s="9" t="n">
+        <v>0.860428240740741</v>
+      </c>
+      <c r="G500" s="9" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H500" s="10" t="n">
+        <v>195</v>
+      </c>
+      <c r="I500" s="10" t="n">
+        <v>950019</v>
+      </c>
     </row>
     <row r="501" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H501" s="12"/>
+      <c r="A501" s="6" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B501" s="7" t="n">
+        <v>7732</v>
+      </c>
+      <c r="C501" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D501" s="8" t="n">
+        <v>0.0833333333333333</v>
+      </c>
+      <c r="E501" s="9" t="n">
+        <v>0.862673611111111</v>
+      </c>
+      <c r="F501" s="9" t="n">
+        <v>0.871203703703704</v>
+      </c>
+      <c r="G501" s="9" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H501" s="10" t="n">
+        <v>183</v>
+      </c>
+      <c r="I501" s="10" t="n">
+        <v>929334</v>
+      </c>
     </row>
     <row r="502" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H502" s="12"/>
+      <c r="A502" s="6" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B502" s="7" t="n">
+        <v>7743</v>
+      </c>
+      <c r="C502" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D502" s="8" t="n">
+        <v>0.0833333333333333</v>
+      </c>
+      <c r="E502" s="9" t="n">
+        <v>0.872962962962963</v>
+      </c>
+      <c r="F502" s="9" t="n">
+        <v>0.881319444444444</v>
+      </c>
+      <c r="G502" s="9" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H502" s="10" t="n">
+        <v>161</v>
+      </c>
+      <c r="I502" s="10" t="n">
+        <v>895989</v>
+      </c>
     </row>
     <row r="503" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H503" s="12"/>
+      <c r="A503" s="6" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B503" s="7" t="n">
+        <v>8263</v>
+      </c>
+      <c r="C503" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D503" s="8" t="n">
+        <v>0.0833333333333333</v>
+      </c>
+      <c r="E503" s="9" t="n">
+        <v>0.644328703703704</v>
+      </c>
+      <c r="F503" s="9" t="n">
+        <v>0.705613425925926</v>
+      </c>
+      <c r="G503" s="9" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H503" s="10" t="n">
+        <v>3801</v>
+      </c>
+      <c r="I503" s="10" t="n">
+        <v>15028070</v>
+      </c>
     </row>
     <row r="504" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H504" s="12"/>
+      <c r="A504" s="6" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B504" s="7" t="n">
+        <v>9304</v>
+      </c>
+      <c r="C504" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D504" s="8" t="n">
+        <v>0.0833333333333333</v>
+      </c>
+      <c r="E504" s="9" t="n">
+        <v>0.882372685185185</v>
+      </c>
+      <c r="F504" s="9" t="n">
+        <v>0.883622685185185</v>
+      </c>
+      <c r="G504" s="9" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H504" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="I504" s="10" t="n">
+        <v>437500</v>
+      </c>
     </row>
     <row r="505" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H505" s="12"/>
+      <c r="A505" s="6" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B505" s="7" t="n">
+        <v>9327</v>
+      </c>
+      <c r="C505" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D505" s="8" t="n">
+        <v>0.0833333333333333</v>
+      </c>
+      <c r="E505" s="9" t="n">
+        <v>0.884479166666667</v>
+      </c>
+      <c r="F505" s="9" t="n">
+        <v>0.887199074074074</v>
+      </c>
+      <c r="G505" s="9" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H505" s="10" t="n">
+        <v>67</v>
+      </c>
+      <c r="I505" s="10" t="n">
+        <v>622834</v>
+      </c>
     </row>
     <row r="506" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H506" s="12"/>
+      <c r="A506" s="6" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B506" s="7" t="n">
+        <v>9352</v>
+      </c>
+      <c r="C506" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D506" s="8" t="n">
+        <v>0.0833333333333333</v>
+      </c>
+      <c r="E506" s="9" t="n">
+        <v>0.888229166666667</v>
+      </c>
+      <c r="F506" s="9" t="n">
+        <v>0.891111111111111</v>
+      </c>
+      <c r="G506" s="9" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H506" s="10" t="n">
+        <v>33</v>
+      </c>
+      <c r="I506" s="10" t="n">
+        <v>311436</v>
+      </c>
     </row>
     <row r="507" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H507" s="12"/>
+      <c r="A507" s="6" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B507" s="7" t="n">
+        <v>9413</v>
+      </c>
+      <c r="C507" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D507" s="8" t="n">
+        <v>0.0833333333333333</v>
+      </c>
+      <c r="E507" s="9" t="n">
+        <v>0.891898148148148</v>
+      </c>
+      <c r="F507" s="9" t="n">
+        <v>0.892581018518519</v>
+      </c>
+      <c r="G507" s="9" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H507" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I507" s="10" t="n">
+        <v>6917</v>
+      </c>
     </row>
     <row r="508" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H508" s="12"/>
+      <c r="A508" s="6" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B508" s="7" t="n">
+        <v>304</v>
+      </c>
+      <c r="C508" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D508" s="8" t="n">
+        <v>0.0833333333333333</v>
+      </c>
+      <c r="E508" s="9" t="n">
+        <v>0.894143518518519</v>
+      </c>
+      <c r="F508" s="9" t="n">
+        <v>0.914791666666667</v>
+      </c>
+      <c r="G508" s="9" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H508" s="10" t="n">
+        <v>1364</v>
+      </c>
+      <c r="I508" s="10" t="n">
+        <v>3458081</v>
+      </c>
     </row>
     <row r="509" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H509" s="12"/>
+      <c r="A509" s="6" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B509" s="7" t="n">
+        <v>311</v>
+      </c>
+      <c r="C509" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D509" s="8" t="n">
+        <v>0.0833333333333333</v>
+      </c>
+      <c r="E509" s="9" t="n">
+        <v>0.916805555555556</v>
+      </c>
+      <c r="F509" s="9" t="n">
+        <v>0.936782407407407</v>
+      </c>
+      <c r="G509" s="9" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H509" s="10" t="n">
+        <v>1232</v>
+      </c>
+      <c r="I509" s="10" t="n">
+        <v>2928073</v>
+      </c>
     </row>
     <row r="510" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H510" s="12"/>
+      <c r="A510" s="6" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B510" s="7" t="n">
+        <v>207</v>
+      </c>
+      <c r="C510" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D510" s="8" t="n">
+        <v>0.0833333333333333</v>
+      </c>
+      <c r="E510" s="9" t="n">
+        <v>0.938148148148148</v>
+      </c>
+      <c r="F510" s="9" t="n">
+        <v>0.955277777777778</v>
+      </c>
+      <c r="G510" s="9" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H510" s="10" t="n">
+        <v>712</v>
+      </c>
+      <c r="I510" s="10" t="n">
+        <v>1904628</v>
+      </c>
     </row>
     <row r="511" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H511" s="12"/>
+      <c r="A511" s="6" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B511" s="7" t="n">
+        <v>210</v>
+      </c>
+      <c r="C511" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D511" s="8" t="n">
+        <v>0.0833333333333333</v>
+      </c>
+      <c r="E511" s="9" t="n">
+        <v>0.956574074074074</v>
+      </c>
+      <c r="F511" s="9" t="n">
+        <v>0.972002314814815</v>
+      </c>
+      <c r="G511" s="9" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H511" s="10" t="n">
+        <v>710</v>
+      </c>
+      <c r="I511" s="10" t="n">
+        <v>2168596</v>
+      </c>
     </row>
     <row r="512" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H512" s="12"/>
+      <c r="A512" s="6" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B512" s="7" t="n">
+        <v>213</v>
+      </c>
+      <c r="C512" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D512" s="8" t="n">
+        <v>0.0833333333333333</v>
+      </c>
+      <c r="E512" s="9" t="n">
+        <v>0.974502314814815</v>
+      </c>
+      <c r="F512" s="9" t="n">
+        <v>0.990520833333333</v>
+      </c>
+      <c r="G512" s="9" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H512" s="10" t="n">
+        <v>759</v>
+      </c>
+      <c r="I512" s="10" t="n">
+        <v>6682736</v>
+      </c>
     </row>
     <row r="513" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H513" s="12"/>
+      <c r="A513" s="6" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B513" s="7" t="n">
+        <v>257</v>
+      </c>
+      <c r="C513" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D513" s="8" t="n">
+        <v>0.0833333333333333</v>
+      </c>
+      <c r="E513" s="9" t="n">
+        <v>0.992511574074074</v>
+      </c>
+      <c r="F513" s="9" t="n">
+        <v>0.00809027777777778</v>
+      </c>
+      <c r="G513" s="9" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H513" s="10" t="n">
+        <v>966</v>
+      </c>
+      <c r="I513" s="10" t="n">
+        <v>2414078</v>
+      </c>
     </row>
     <row r="514" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H514" s="12"/>
+      <c r="A514" s="6" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B514" s="7" t="n">
+        <v>261</v>
+      </c>
+      <c r="C514" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D514" s="8" t="n">
+        <v>0.0833333333333333</v>
+      </c>
+      <c r="E514" s="9" t="n">
+        <v>0.00958333333333333</v>
+      </c>
+      <c r="F514" s="9" t="n">
+        <v>0.0315625</v>
+      </c>
+      <c r="G514" s="9" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H514" s="10" t="n">
+        <v>1121</v>
+      </c>
+      <c r="I514" s="10" t="n">
+        <v>3314810</v>
+      </c>
     </row>
     <row r="515" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C515" s="8"/>
       <c r="H515" s="12"/>
     </row>
     <row r="516" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16073,15 +16750,15 @@
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="C2:D488" type="custom">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="C2:D514 C515" type="custom">
       <formula1>OR(TIMEVALUE(TEXT(C2, "hh:mm:ss"))=C2, AND(ISNUMBER(C2), LEFT(CELL("format", C2))="D"))</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="A2:A488" type="custom">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="A2:A514" type="custom">
       <formula1>OR(NOT(ISERROR(DATEVALUE(A2))), AND(ISNUMBER(A2), LEFT(CELL("format", A2))="D"))</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="B2:B488 H2:I488" type="custom">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="B2:B514 H2:I488 I489:I514 H490:H514" type="custom">
       <formula1>AND(ISNUMBER(B2),(NOT(OR(NOT(ISERROR(DATEVALUE(B2))), AND(ISNUMBER(B2), LEFT(CELL("format", B2))="D")))))</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Se agrega borrador de la Fase 3
</commit_message>
<xml_diff>
--- a/data/raw/io_data_bimbo.xlsx
+++ b/data/raw/io_data_bimbo.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I986"/>
+  <dimension ref="A1:I1048576"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.88"/>
@@ -14599,7 +14599,7 @@
       <c r="G489" s="9" t="n">
         <v>0.32</v>
       </c>
-      <c r="H489" s="0" t="n">
+      <c r="H489" s="1" t="n">
         <v>136</v>
       </c>
       <c r="I489" s="10" t="n">
@@ -15332,97 +15332,877 @@
       </c>
     </row>
     <row r="515" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C515" s="8"/>
-      <c r="H515" s="12"/>
+      <c r="A515" s="6" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B515" s="7" t="n">
+        <v>9382</v>
+      </c>
+      <c r="C515" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D515" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E515" s="9" t="n">
+        <v>0.636053240740741</v>
+      </c>
+      <c r="F515" s="9" t="n">
+        <v>0.644652777777778</v>
+      </c>
+      <c r="G515" s="9" t="n">
+        <v>0.257581018518519</v>
+      </c>
+      <c r="H515" s="10" t="n">
+        <v>134</v>
+      </c>
+      <c r="I515" s="10" t="n">
+        <v>358301</v>
+      </c>
     </row>
     <row r="516" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H516" s="12"/>
+      <c r="A516" s="6" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B516" s="7" t="n">
+        <v>9384</v>
+      </c>
+      <c r="C516" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D516" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E516" s="9" t="n">
+        <v>0.646481481481481</v>
+      </c>
+      <c r="F516" s="9" t="n">
+        <v>0.653240740740741</v>
+      </c>
+      <c r="G516" s="9" t="n">
+        <v>0.257581018518519</v>
+      </c>
+      <c r="H516" s="10" t="n">
+        <v>93</v>
+      </c>
+      <c r="I516" s="10" t="n">
+        <v>288615</v>
+      </c>
     </row>
     <row r="517" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H517" s="12"/>
+      <c r="A517" s="6" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B517" s="7" t="n">
+        <v>9389</v>
+      </c>
+      <c r="C517" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D517" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E517" s="9" t="n">
+        <v>0.653842592592593</v>
+      </c>
+      <c r="F517" s="9" t="n">
+        <v>0.656041666666667</v>
+      </c>
+      <c r="G517" s="9" t="n">
+        <v>0.257581018518519</v>
+      </c>
+      <c r="H517" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="I517" s="10" t="n">
+        <v>37990</v>
+      </c>
     </row>
     <row r="518" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H518" s="12"/>
+      <c r="A518" s="6" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B518" s="7" t="n">
+        <v>7604</v>
+      </c>
+      <c r="C518" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D518" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E518" s="9" t="n">
+        <v>0.657002314814815</v>
+      </c>
+      <c r="F518" s="9" t="n">
+        <v>0.662083333333333</v>
+      </c>
+      <c r="G518" s="9" t="n">
+        <v>0.257581018518519</v>
+      </c>
+      <c r="H518" s="10" t="n">
+        <v>310</v>
+      </c>
+      <c r="I518" s="10" t="n">
+        <v>1801292</v>
+      </c>
     </row>
     <row r="519" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H519" s="12"/>
+      <c r="A519" s="6" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B519" s="7" t="n">
+        <v>7624</v>
+      </c>
+      <c r="C519" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D519" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E519" s="9" t="n">
+        <v>0.677592592592593</v>
+      </c>
+      <c r="F519" s="9" t="n">
+        <v>0.686423611111111</v>
+      </c>
+      <c r="G519" s="9" t="n">
+        <v>0.257581018518519</v>
+      </c>
+      <c r="H519" s="10" t="n">
+        <v>259</v>
+      </c>
+      <c r="I519" s="10" t="n">
+        <v>1535017</v>
+      </c>
     </row>
     <row r="520" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H520" s="12"/>
+      <c r="A520" s="6" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B520" s="7" t="n">
+        <v>7632</v>
+      </c>
+      <c r="C520" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D520" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E520" s="9" t="n">
+        <v>0.687638888888889</v>
+      </c>
+      <c r="F520" s="9" t="n">
+        <v>0.69875</v>
+      </c>
+      <c r="G520" s="9" t="n">
+        <v>0.257581018518519</v>
+      </c>
+      <c r="H520" s="10" t="n">
+        <v>323</v>
+      </c>
+      <c r="I520" s="10" t="n">
+        <v>1650688</v>
+      </c>
     </row>
     <row r="521" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H521" s="12"/>
+      <c r="A521" s="6" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B521" s="7" t="n">
+        <v>7645</v>
+      </c>
+      <c r="C521" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D521" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E521" s="9" t="n">
+        <v>0.700625</v>
+      </c>
+      <c r="F521" s="9" t="n">
+        <v>0.713969907407407</v>
+      </c>
+      <c r="G521" s="9" t="n">
+        <v>0.257581018518519</v>
+      </c>
+      <c r="H521" s="10" t="n">
+        <v>406</v>
+      </c>
+      <c r="I521" s="10" t="n">
+        <v>2241163</v>
+      </c>
     </row>
     <row r="522" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H522" s="12"/>
+      <c r="A522" s="6" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B522" s="7" t="n">
+        <v>7701</v>
+      </c>
+      <c r="C522" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D522" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E522" s="9" t="n">
+        <v>0.715706018518519</v>
+      </c>
+      <c r="F522" s="9" t="n">
+        <v>0.719421296296296</v>
+      </c>
+      <c r="G522" s="9" t="n">
+        <v>0.257581018518519</v>
+      </c>
+      <c r="H522" s="10" t="n">
+        <v>52</v>
+      </c>
+      <c r="I522" s="10" t="n">
+        <v>227396</v>
+      </c>
     </row>
     <row r="523" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H523" s="12"/>
+      <c r="A523" s="6" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B523" s="7" t="n">
+        <v>7711</v>
+      </c>
+      <c r="C523" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D523" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E523" s="9" t="n">
+        <v>0.72037037037037</v>
+      </c>
+      <c r="F523" s="9" t="n">
+        <v>0.723738425925926</v>
+      </c>
+      <c r="G523" s="9" t="n">
+        <v>0.257581018518519</v>
+      </c>
+      <c r="H523" s="10" t="n">
+        <v>96</v>
+      </c>
+      <c r="I523" s="10" t="n">
+        <v>364937</v>
+      </c>
     </row>
     <row r="524" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H524" s="12"/>
+      <c r="A524" s="6" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B524" s="7" t="n">
+        <v>7715</v>
+      </c>
+      <c r="C524" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D524" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E524" s="9" t="n">
+        <v>0.724722222222222</v>
+      </c>
+      <c r="F524" s="9" t="n">
+        <v>0.727893518518519</v>
+      </c>
+      <c r="G524" s="9" t="n">
+        <v>0.257581018518519</v>
+      </c>
+      <c r="H524" s="10" t="n">
+        <v>61</v>
+      </c>
+      <c r="I524" s="10" t="n">
+        <v>242162</v>
+      </c>
     </row>
     <row r="525" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H525" s="12"/>
+      <c r="A525" s="6" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B525" s="7" t="n">
+        <v>7719</v>
+      </c>
+      <c r="C525" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D525" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E525" s="9" t="n">
+        <v>0.728865740740741</v>
+      </c>
+      <c r="F525" s="9" t="n">
+        <v>0.732164351851852</v>
+      </c>
+      <c r="G525" s="9" t="n">
+        <v>0.257581018518519</v>
+      </c>
+      <c r="H525" s="10" t="n">
+        <v>112</v>
+      </c>
+      <c r="I525" s="10" t="n">
+        <v>515164</v>
+      </c>
     </row>
     <row r="526" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H526" s="12"/>
+      <c r="A526" s="6" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B526" s="7" t="n">
+        <v>7727</v>
+      </c>
+      <c r="C526" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D526" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E526" s="9" t="n">
+        <v>0.73287037037037</v>
+      </c>
+      <c r="F526" s="9" t="n">
+        <v>0.74005787037037</v>
+      </c>
+      <c r="G526" s="9" t="n">
+        <v>0.257581018518519</v>
+      </c>
+      <c r="H526" s="10" t="n">
+        <v>184</v>
+      </c>
+      <c r="I526" s="10" t="n">
+        <v>676180</v>
+      </c>
     </row>
     <row r="527" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H527" s="12"/>
+      <c r="A527" s="6" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B527" s="7" t="n">
+        <v>7728</v>
+      </c>
+      <c r="C527" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D527" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E527" s="9" t="n">
+        <v>0.742453703703704</v>
+      </c>
+      <c r="F527" s="9" t="n">
+        <v>0.749618055555556</v>
+      </c>
+      <c r="G527" s="9" t="n">
+        <v>0.257581018518519</v>
+      </c>
+      <c r="H527" s="10" t="n">
+        <v>151</v>
+      </c>
+      <c r="I527" s="10" t="n">
+        <v>658713</v>
+      </c>
     </row>
     <row r="528" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H528" s="12"/>
+      <c r="A528" s="6" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B528" s="7" t="n">
+        <v>7742</v>
+      </c>
+      <c r="C528" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D528" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E528" s="9" t="n">
+        <v>0.750509259259259</v>
+      </c>
+      <c r="F528" s="9" t="n">
+        <v>0.756076388888889</v>
+      </c>
+      <c r="G528" s="9" t="n">
+        <v>0.257581018518519</v>
+      </c>
+      <c r="H528" s="10" t="n">
+        <v>114</v>
+      </c>
+      <c r="I528" s="10" t="n">
+        <v>404809</v>
+      </c>
     </row>
     <row r="529" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H529" s="12"/>
+      <c r="A529" s="6" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B529" s="7" t="n">
+        <v>9326</v>
+      </c>
+      <c r="C529" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D529" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E529" s="9" t="n">
+        <v>0.757164351851852</v>
+      </c>
+      <c r="F529" s="9" t="n">
+        <v>0.759548611111111</v>
+      </c>
+      <c r="G529" s="9" t="n">
+        <v>0.257581018518519</v>
+      </c>
+      <c r="H529" s="10" t="n">
+        <v>106</v>
+      </c>
+      <c r="I529" s="10" t="n">
+        <v>958182</v>
+      </c>
     </row>
     <row r="530" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H530" s="12"/>
+      <c r="A530" s="6" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B530" s="7" t="n">
+        <v>9345</v>
+      </c>
+      <c r="C530" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D530" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E530" s="9" t="n">
+        <v>0.762361111111111</v>
+      </c>
+      <c r="F530" s="9" t="n">
+        <v>0.764733796296296</v>
+      </c>
+      <c r="G530" s="9" t="n">
+        <v>0.257581018518519</v>
+      </c>
+      <c r="H530" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="I530" s="10" t="n">
+        <v>249921</v>
+      </c>
     </row>
     <row r="531" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H531" s="12"/>
+      <c r="A531" s="6" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B531" s="7" t="n">
+        <v>9370</v>
+      </c>
+      <c r="C531" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D531" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E531" s="9" t="n">
+        <v>0.7671875</v>
+      </c>
+      <c r="F531" s="9" t="n">
+        <v>0.768796296296296</v>
+      </c>
+      <c r="G531" s="9" t="n">
+        <v>0.257581018518519</v>
+      </c>
+      <c r="H531" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="I531" s="10" t="n">
+        <v>40910</v>
+      </c>
     </row>
     <row r="532" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H532" s="12"/>
+      <c r="A532" s="6" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B532" s="7" t="n">
+        <v>9371</v>
+      </c>
+      <c r="C532" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D532" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E532" s="9" t="n">
+        <v>0.765844907407407</v>
+      </c>
+      <c r="F532" s="9" t="n">
+        <v>0.766747685185185</v>
+      </c>
+      <c r="G532" s="9" t="n">
+        <v>0.257581018518519</v>
+      </c>
+      <c r="H532" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="I532" s="10" t="n">
+        <v>24546</v>
+      </c>
     </row>
     <row r="533" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H533" s="12"/>
+      <c r="A533" s="6" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B533" s="7" t="n">
+        <v>9419</v>
+      </c>
+      <c r="C533" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D533" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E533" s="9" t="n">
+        <v>0.768877314814815</v>
+      </c>
+      <c r="F533" s="9" t="n">
+        <v>0.774722222222222</v>
+      </c>
+      <c r="G533" s="9" t="n">
+        <v>0.257581018518519</v>
+      </c>
+      <c r="H533" s="10" t="n">
+        <v>104</v>
+      </c>
+      <c r="I533" s="10" t="n">
+        <v>926802</v>
+      </c>
     </row>
     <row r="534" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H534" s="12"/>
+      <c r="A534" s="6" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B534" s="7" t="n">
+        <v>257</v>
+      </c>
+      <c r="C534" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D534" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E534" s="9" t="n">
+        <v>0.825578703703704</v>
+      </c>
+      <c r="F534" s="9" t="n">
+        <v>0.837604166666667</v>
+      </c>
+      <c r="G534" s="9" t="n">
+        <v>0.257581018518519</v>
+      </c>
+      <c r="H534" s="10" t="n">
+        <v>1133</v>
+      </c>
+      <c r="I534" s="10" t="n">
+        <v>3171387</v>
+      </c>
     </row>
     <row r="535" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H535" s="12"/>
+      <c r="A535" s="6" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B535" s="7" t="n">
+        <v>261</v>
+      </c>
+      <c r="C535" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D535" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E535" s="9" t="n">
+        <v>0.922766203703704</v>
+      </c>
+      <c r="F535" s="9" t="n">
+        <v>0.941238425925926</v>
+      </c>
+      <c r="G535" s="9" t="n">
+        <v>0.257581018518519</v>
+      </c>
+      <c r="H535" s="10" t="n">
+        <v>1408</v>
+      </c>
+      <c r="I535" s="10" t="n">
+        <v>3846778</v>
+      </c>
     </row>
     <row r="536" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H536" s="12"/>
+      <c r="A536" s="6" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B536" s="7" t="n">
+        <v>212</v>
+      </c>
+      <c r="C536" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D536" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E536" s="9" t="n">
+        <v>0.83875</v>
+      </c>
+      <c r="F536" s="9" t="n">
+        <v>0.858946759259259</v>
+      </c>
+      <c r="G536" s="9" t="n">
+        <v>0.257581018518519</v>
+      </c>
+      <c r="H536" s="10" t="n">
+        <v>961</v>
+      </c>
+      <c r="I536" s="10" t="n">
+        <v>3495182</v>
+      </c>
     </row>
     <row r="537" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H537" s="12"/>
+      <c r="A537" s="6" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B537" s="7" t="n">
+        <v>213</v>
+      </c>
+      <c r="C537" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D537" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E537" s="9" t="n">
+        <v>0.942488425925926</v>
+      </c>
+      <c r="F537" s="9" t="n">
+        <v>0.953101851851852</v>
+      </c>
+      <c r="G537" s="9" t="n">
+        <v>0.257581018518519</v>
+      </c>
+      <c r="H537" s="10" t="n">
+        <v>582</v>
+      </c>
+      <c r="I537" s="10" t="n">
+        <v>5140453</v>
+      </c>
     </row>
     <row r="538" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H538" s="12"/>
+      <c r="A538" s="6" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B538" s="7" t="n">
+        <v>260</v>
+      </c>
+      <c r="C538" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D538" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E538" s="9" t="n">
+        <v>0.955416666666667</v>
+      </c>
+      <c r="F538" s="9" t="n">
+        <v>0.972060185185185</v>
+      </c>
+      <c r="G538" s="9" t="n">
+        <v>0.257581018518519</v>
+      </c>
+      <c r="H538" s="10" t="n">
+        <v>870</v>
+      </c>
+      <c r="I538" s="10" t="n">
+        <v>2794399</v>
+      </c>
     </row>
     <row r="539" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H539" s="12"/>
+      <c r="A539" s="6" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B539" s="7" t="n">
+        <v>301</v>
+      </c>
+      <c r="C539" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D539" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E539" s="9" t="n">
+        <v>0.776331018518519</v>
+      </c>
+      <c r="F539" s="9" t="n">
+        <v>0.795590277777778</v>
+      </c>
+      <c r="G539" s="9" t="n">
+        <v>0.257581018518519</v>
+      </c>
+      <c r="H539" s="10" t="n">
+        <v>1009</v>
+      </c>
+      <c r="I539" s="10" t="n">
+        <v>2915400</v>
+      </c>
     </row>
     <row r="540" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H540" s="12"/>
+      <c r="A540" s="6" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B540" s="7" t="n">
+        <v>305</v>
+      </c>
+      <c r="C540" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D540" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E540" s="9" t="n">
+        <v>0.821956018518519</v>
+      </c>
+      <c r="F540" s="9" t="n">
+        <v>0.824641203703704</v>
+      </c>
+      <c r="G540" s="9" t="n">
+        <v>0.257581018518519</v>
+      </c>
+      <c r="H540" s="10" t="n">
+        <v>120</v>
+      </c>
+      <c r="I540" s="10" t="n">
+        <v>563070</v>
+      </c>
     </row>
     <row r="541" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H541" s="12"/>
+      <c r="A541" s="6" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B541" s="7" t="n">
+        <v>1259</v>
+      </c>
+      <c r="C541" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D541" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E541" s="9" t="n">
+        <v>0.861053240740741</v>
+      </c>
+      <c r="F541" s="9" t="n">
+        <v>0.871423611111111</v>
+      </c>
+      <c r="G541" s="9" t="n">
+        <v>0.257581018518519</v>
+      </c>
+      <c r="H541" s="10" t="n">
+        <v>336</v>
+      </c>
+      <c r="I541" s="10" t="n">
+        <v>2046199</v>
+      </c>
     </row>
     <row r="542" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H542" s="12"/>
+      <c r="A542" s="6" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B542" s="7" t="n">
+        <v>207</v>
+      </c>
+      <c r="C542" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D542" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E542" s="9" t="n">
+        <v>0.890474537037037</v>
+      </c>
+      <c r="F542" s="9" t="n">
+        <v>0.907465277777778</v>
+      </c>
+      <c r="G542" s="9" t="n">
+        <v>0.257581018518519</v>
+      </c>
+      <c r="H542" s="10" t="n">
+        <v>769</v>
+      </c>
+      <c r="I542" s="10" t="n">
+        <v>2618954</v>
+      </c>
     </row>
     <row r="543" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H543" s="12"/>
+      <c r="A543" s="6" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B543" s="7" t="n">
+        <v>210</v>
+      </c>
+      <c r="C543" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D543" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E543" s="9" t="n">
+        <v>0.873229166666667</v>
+      </c>
+      <c r="F543" s="9" t="n">
+        <v>0.889155092592593</v>
+      </c>
+      <c r="G543" s="9" t="n">
+        <v>0.257581018518519</v>
+      </c>
+      <c r="H543" s="10" t="n">
+        <v>745</v>
+      </c>
+      <c r="I543" s="10" t="n">
+        <v>2276295</v>
+      </c>
     </row>
     <row r="544" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H544" s="12"/>
+      <c r="A544" s="6" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B544" s="7" t="n">
+        <v>258</v>
+      </c>
+      <c r="C544" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D544" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E544" s="9" t="n">
+        <v>0.909074074074074</v>
+      </c>
+      <c r="F544" s="9" t="n">
+        <v>0.920810185185185</v>
+      </c>
+      <c r="G544" s="9" t="n">
+        <v>0.257581018518519</v>
+      </c>
+      <c r="H544" s="10" t="n">
+        <v>916</v>
+      </c>
+      <c r="I544" s="10" t="n">
+        <v>1982025</v>
+      </c>
     </row>
     <row r="545" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B545" s="7"/>
       <c r="H545" s="12"/>
     </row>
     <row r="546" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16745,20 +17525,18 @@
     <row r="985" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H985" s="12"/>
     </row>
-    <row r="986" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H986" s="12"/>
-    </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="C2:D514 C515" type="custom">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="C2:D544" type="custom">
       <formula1>OR(TIMEVALUE(TEXT(C2, "hh:mm:ss"))=C2, AND(ISNUMBER(C2), LEFT(CELL("format", C2))="D"))</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="A2:A514" type="custom">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="A2:A544" type="custom">
       <formula1>OR(NOT(ISERROR(DATEVALUE(A2))), AND(ISNUMBER(A2), LEFT(CELL("format", A2))="D"))</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="B2:B514 H2:I488 I489:I514 H490:H514" type="custom">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="B2:B545 H2:I488 I489:I544 H490:H544" type="custom">
       <formula1>AND(ISNUMBER(B2),(NOT(OR(NOT(ISERROR(DATEVALUE(B2))), AND(ISNUMBER(B2), LEFT(CELL("format", B2))="D")))))</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Se hace ajuste a la Fase 3
</commit_message>
<xml_diff>
--- a/data/raw/io_data_bimbo.xlsx
+++ b/data/raw/io_data_bimbo.xlsx
@@ -16202,65 +16202,584 @@
       </c>
     </row>
     <row r="545" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B545" s="7"/>
-      <c r="H545" s="12"/>
+      <c r="A545" s="6" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B545" s="7" t="n">
+        <v>7603</v>
+      </c>
+      <c r="C545" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D545" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E545" s="9" t="n">
+        <v>0.644050925925926</v>
+      </c>
+      <c r="F545" s="9" t="n">
+        <v>0.656608796296296</v>
+      </c>
+      <c r="G545" s="9" t="n">
+        <v>0.289548611111111</v>
+      </c>
+      <c r="H545" s="10" t="n">
+        <v>370</v>
+      </c>
+      <c r="I545" s="10" t="n">
+        <v>2071246</v>
+      </c>
     </row>
     <row r="546" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H546" s="12"/>
+      <c r="A546" s="6" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B546" s="7" t="n">
+        <v>7606</v>
+      </c>
+      <c r="C546" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D546" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E546" s="9" t="n">
+        <v>0.657673611111111</v>
+      </c>
+      <c r="F546" s="9" t="n">
+        <v>0.666608796296296</v>
+      </c>
+      <c r="G546" s="9" t="n">
+        <v>0.289548611111111</v>
+      </c>
+      <c r="H546" s="10" t="n">
+        <v>239</v>
+      </c>
+      <c r="I546" s="10" t="n">
+        <v>1047776</v>
+      </c>
     </row>
     <row r="547" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H547" s="12"/>
+      <c r="A547" s="6" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B547" s="7" t="n">
+        <v>7607</v>
+      </c>
+      <c r="C547" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D547" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E547" s="9" t="n">
+        <v>0.667615740740741</v>
+      </c>
+      <c r="F547" s="9" t="n">
+        <v>0.675011574074074</v>
+      </c>
+      <c r="G547" s="9" t="n">
+        <v>0.289548611111111</v>
+      </c>
+      <c r="H547" s="10" t="n">
+        <v>223</v>
+      </c>
+      <c r="I547" s="10" t="n">
+        <v>1254594</v>
+      </c>
     </row>
     <row r="548" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H548" s="12"/>
+      <c r="A548" s="6" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B548" s="7" t="n">
+        <v>7611</v>
+      </c>
+      <c r="C548" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D548" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E548" s="9" t="n">
+        <v>0.676400462962963</v>
+      </c>
+      <c r="F548" s="9" t="n">
+        <v>0.689502314814815</v>
+      </c>
+      <c r="G548" s="9" t="n">
+        <v>0.289548611111111</v>
+      </c>
+      <c r="H548" s="10" t="n">
+        <v>211</v>
+      </c>
+      <c r="I548" s="10" t="n">
+        <v>1313417</v>
+      </c>
     </row>
     <row r="549" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H549" s="12"/>
+      <c r="A549" s="6" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B549" s="7" t="n">
+        <v>7621</v>
+      </c>
+      <c r="C549" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D549" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E549" s="9" t="n">
+        <v>0.690763888888889</v>
+      </c>
+      <c r="F549" s="9" t="n">
+        <v>0.707534722222222</v>
+      </c>
+      <c r="G549" s="9" t="n">
+        <v>0.289548611111111</v>
+      </c>
+      <c r="H549" s="10" t="n">
+        <v>992</v>
+      </c>
+      <c r="I549" s="10" t="n">
+        <v>5988388</v>
+      </c>
     </row>
     <row r="550" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H550" s="12"/>
+      <c r="A550" s="6" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B550" s="7" t="n">
+        <v>7646</v>
+      </c>
+      <c r="C550" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D550" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E550" s="9" t="n">
+        <v>0.709895833333333</v>
+      </c>
+      <c r="F550" s="9" t="n">
+        <v>0.726041666666667</v>
+      </c>
+      <c r="G550" s="9" t="n">
+        <v>0.289548611111111</v>
+      </c>
+      <c r="H550" s="10" t="n">
+        <v>891</v>
+      </c>
+      <c r="I550" s="10" t="n">
+        <v>4923640</v>
+      </c>
     </row>
     <row r="551" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H551" s="12"/>
+      <c r="A551" s="6" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B551" s="7" t="n">
+        <v>7653</v>
+      </c>
+      <c r="C551" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D551" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E551" s="9" t="n">
+        <v>0.728784722222222</v>
+      </c>
+      <c r="F551" s="9" t="n">
+        <v>0.739664351851852</v>
+      </c>
+      <c r="G551" s="9" t="n">
+        <v>0.289548611111111</v>
+      </c>
+      <c r="H551" s="10" t="n">
+        <v>503</v>
+      </c>
+      <c r="I551" s="10" t="n">
+        <v>3029953</v>
+      </c>
     </row>
     <row r="552" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H552" s="12"/>
+      <c r="A552" s="6" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B552" s="7" t="n">
+        <v>7664</v>
+      </c>
+      <c r="C552" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D552" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E552" s="9" t="n">
+        <v>0.741585648148148</v>
+      </c>
+      <c r="F552" s="9" t="n">
+        <v>0.758159722222222</v>
+      </c>
+      <c r="G552" s="9" t="n">
+        <v>0.289548611111111</v>
+      </c>
+      <c r="H552" s="10" t="n">
+        <v>832</v>
+      </c>
+      <c r="I552" s="10" t="n">
+        <v>4518380</v>
+      </c>
     </row>
     <row r="553" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H553" s="12"/>
+      <c r="A553" s="6" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B553" s="7" t="n">
+        <v>7674</v>
+      </c>
+      <c r="C553" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D553" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E553" s="9" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="F553" s="9" t="n">
+        <v>0.762152777777778</v>
+      </c>
+      <c r="G553" s="9" t="n">
+        <v>0.289548611111111</v>
+      </c>
+      <c r="H553" s="10" t="n">
+        <v>417</v>
+      </c>
+      <c r="I553" s="10" t="n">
+        <v>5086702</v>
+      </c>
     </row>
     <row r="554" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H554" s="12"/>
+      <c r="A554" s="6" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B554" s="7" t="n">
+        <v>7676</v>
+      </c>
+      <c r="C554" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D554" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E554" s="9" t="n">
+        <v>0.76693287037037</v>
+      </c>
+      <c r="F554" s="9" t="n">
+        <v>0.78537037037037</v>
+      </c>
+      <c r="G554" s="9" t="n">
+        <v>0.289548611111111</v>
+      </c>
+      <c r="H554" s="10" t="n">
+        <v>744</v>
+      </c>
+      <c r="I554" s="10" t="n">
+        <v>3990336</v>
+      </c>
     </row>
     <row r="555" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H555" s="12"/>
+      <c r="A555" s="6" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B555" s="7" t="n">
+        <v>7725</v>
+      </c>
+      <c r="C555" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D555" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E555" s="9" t="n">
+        <v>0.817916666666667</v>
+      </c>
+      <c r="F555" s="9" t="n">
+        <v>0.827581018518519</v>
+      </c>
+      <c r="G555" s="9" t="n">
+        <v>0.289548611111111</v>
+      </c>
+      <c r="H555" s="10" t="n">
+        <v>308</v>
+      </c>
+      <c r="I555" s="10" t="n">
+        <v>1482595</v>
+      </c>
     </row>
     <row r="556" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H556" s="12"/>
+      <c r="A556" s="6" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B556" s="7" t="n">
+        <v>7735</v>
+      </c>
+      <c r="C556" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D556" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E556" s="9" t="n">
+        <v>0.828668981481482</v>
+      </c>
+      <c r="F556" s="9" t="n">
+        <v>0.834814814814815</v>
+      </c>
+      <c r="G556" s="9" t="n">
+        <v>0.289548611111111</v>
+      </c>
+      <c r="H556" s="10" t="n">
+        <v>152</v>
+      </c>
+      <c r="I556" s="10" t="n">
+        <v>817954</v>
+      </c>
     </row>
     <row r="557" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H557" s="12"/>
+      <c r="A557" s="6" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B557" s="7" t="n">
+        <v>8002</v>
+      </c>
+      <c r="C557" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D557" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E557" s="9" t="n">
+        <v>0.837002314814815</v>
+      </c>
+      <c r="F557" s="9" t="n">
+        <v>0.853993055555556</v>
+      </c>
+      <c r="G557" s="9" t="n">
+        <v>0.289548611111111</v>
+      </c>
+      <c r="H557" s="10" t="n">
+        <v>904</v>
+      </c>
+      <c r="I557" s="10" t="n">
+        <v>2593634</v>
+      </c>
     </row>
     <row r="558" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H558" s="12"/>
+      <c r="A558" s="6" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B558" s="7" t="n">
+        <v>304</v>
+      </c>
+      <c r="C558" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D558" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E558" s="9" t="n">
+        <v>0.923368055555556</v>
+      </c>
+      <c r="F558" s="9" t="n">
+        <v>0.937256944444444</v>
+      </c>
+      <c r="G558" s="9" t="n">
+        <v>0.289548611111111</v>
+      </c>
+      <c r="H558" s="10" t="n">
+        <v>1046</v>
+      </c>
+      <c r="I558" s="10" t="n">
+        <v>2556410</v>
+      </c>
     </row>
     <row r="559" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H559" s="12"/>
+      <c r="A559" s="6" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B559" s="7" t="n">
+        <v>1259</v>
+      </c>
+      <c r="C559" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D559" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E559" s="9" t="n">
+        <v>0.881550925925926</v>
+      </c>
+      <c r="F559" s="9" t="n">
+        <v>0.919849537037037</v>
+      </c>
+      <c r="G559" s="9" t="n">
+        <v>0.289548611111111</v>
+      </c>
+      <c r="H559" s="10" t="n">
+        <v>2033</v>
+      </c>
+      <c r="I559" s="10" t="n">
+        <v>8674617</v>
+      </c>
     </row>
     <row r="560" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H560" s="12"/>
+      <c r="A560" s="6" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B560" s="7" t="n">
+        <v>209</v>
+      </c>
+      <c r="C560" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D560" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E560" s="9" t="n">
+        <v>0.858217592592593</v>
+      </c>
+      <c r="F560" s="9" t="n">
+        <v>0.878263888888889</v>
+      </c>
+      <c r="G560" s="9" t="n">
+        <v>0.289548611111111</v>
+      </c>
+      <c r="H560" s="10" t="n">
+        <v>1860</v>
+      </c>
+      <c r="I560" s="10" t="n">
+        <v>4906510</v>
+      </c>
     </row>
     <row r="561" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H561" s="12"/>
+      <c r="A561" s="6" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B561" s="7" t="n">
+        <v>213</v>
+      </c>
+      <c r="C561" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D561" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E561" s="9" t="n">
+        <v>0.941875</v>
+      </c>
+      <c r="F561" s="9" t="n">
+        <v>0.955659722222222</v>
+      </c>
+      <c r="G561" s="9" t="n">
+        <v>0.289548611111111</v>
+      </c>
+      <c r="H561" s="10" t="n">
+        <v>548</v>
+      </c>
+      <c r="I561" s="10" t="n">
+        <v>4086775</v>
+      </c>
     </row>
     <row r="562" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H562" s="12"/>
+      <c r="A562" s="6" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B562" s="7" t="n">
+        <v>253</v>
+      </c>
+      <c r="C562" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D562" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E562" s="9" t="n">
+        <v>0.958344907407407</v>
+      </c>
+      <c r="F562" s="9" t="n">
+        <v>0.969594907407407</v>
+      </c>
+      <c r="G562" s="9" t="n">
+        <v>0.289548611111111</v>
+      </c>
+      <c r="H562" s="10" t="n">
+        <v>819</v>
+      </c>
+      <c r="I562" s="10" t="n">
+        <v>1471919</v>
+      </c>
     </row>
     <row r="563" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H563" s="12"/>
+      <c r="A563" s="6" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B563" s="7" t="n">
+        <v>256</v>
+      </c>
+      <c r="C563" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D563" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E563" s="9" t="n">
+        <v>0.972650462962963</v>
+      </c>
+      <c r="F563" s="9" t="n">
+        <v>0.990428240740741</v>
+      </c>
+      <c r="G563" s="9" t="n">
+        <v>0.289548611111111</v>
+      </c>
+      <c r="H563" s="10" t="n">
+        <v>1837</v>
+      </c>
+      <c r="I563" s="10" t="n">
+        <v>3769828</v>
+      </c>
     </row>
     <row r="564" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H564" s="12"/>
+      <c r="A564" s="6" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B564" s="7" t="n">
+        <v>260</v>
+      </c>
+      <c r="C564" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D564" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E564" s="9" t="n">
+        <v>0.992569444444444</v>
+      </c>
+      <c r="F564" s="9" t="n">
+        <v>0.0113194444444444</v>
+      </c>
+      <c r="G564" s="9" t="n">
+        <v>0.289548611111111</v>
+      </c>
+      <c r="H564" s="10" t="n">
+        <v>1414</v>
+      </c>
+      <c r="I564" s="10" t="n">
+        <v>3427321</v>
+      </c>
     </row>
     <row r="565" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H565" s="12"/>
@@ -17528,15 +18047,15 @@
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="C2:D544" type="custom">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="C2:D564" type="custom">
       <formula1>OR(TIMEVALUE(TEXT(C2, "hh:mm:ss"))=C2, AND(ISNUMBER(C2), LEFT(CELL("format", C2))="D"))</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="A2:A544" type="custom">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="A2:A564" type="custom">
       <formula1>OR(NOT(ISERROR(DATEVALUE(A2))), AND(ISNUMBER(A2), LEFT(CELL("format", A2))="D"))</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="B2:B545 H2:I488 I489:I544 H490:H544" type="custom">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="B2:B564 H2:I488 I489:I564 H490:H564" type="custom">
       <formula1>AND(ISNUMBER(B2),(NOT(OR(NOT(ISERROR(DATEVALUE(B2))), AND(ISNUMBER(B2), LEFT(CELL("format", B2))="D")))))</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Modificación e implementación enfoque de la Fase 3
</commit_message>
<xml_diff>
--- a/data/raw/io_data_bimbo.xlsx
+++ b/data/raw/io_data_bimbo.xlsx
@@ -16782,70 +16782,618 @@
       </c>
     </row>
     <row r="565" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H565" s="12"/>
+      <c r="A565" s="6" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B565" s="7" t="n">
+        <v>9383</v>
+      </c>
+      <c r="C565" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D565" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E565" s="9" t="n">
+        <v>0.653611111111111</v>
+      </c>
+      <c r="F565" s="9" t="n">
+        <v>0.65599537037037</v>
+      </c>
+      <c r="G565" s="9" t="n">
+        <v>0.285300925925926</v>
+      </c>
+      <c r="H565" s="12" t="n">
+        <v>17</v>
+      </c>
+      <c r="I565" s="10" t="n">
+        <v>119421</v>
+      </c>
     </row>
     <row r="566" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H566" s="12"/>
+      <c r="A566" s="6" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B566" s="7" t="n">
+        <v>7601</v>
+      </c>
+      <c r="C566" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D566" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E566" s="9" t="n">
+        <v>0.656828703703704</v>
+      </c>
+      <c r="F566" s="9" t="n">
+        <v>0.662037037037037</v>
+      </c>
+      <c r="G566" s="9" t="n">
+        <v>0.285300925925926</v>
+      </c>
+      <c r="H566" s="12" t="n">
+        <v>84</v>
+      </c>
+      <c r="I566" s="10" t="n">
+        <v>490140</v>
+      </c>
     </row>
     <row r="567" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H567" s="12"/>
+      <c r="A567" s="6" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B567" s="7" t="n">
+        <v>7624</v>
+      </c>
+      <c r="C567" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D567" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E567" s="9" t="n">
+        <v>0.664675925925926</v>
+      </c>
+      <c r="F567" s="9" t="n">
+        <v>0.680011574074074</v>
+      </c>
+      <c r="G567" s="9" t="n">
+        <v>0.285300925925926</v>
+      </c>
+      <c r="H567" s="12" t="n">
+        <v>412</v>
+      </c>
+      <c r="I567" s="10" t="n">
+        <v>1998459</v>
+      </c>
     </row>
     <row r="568" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H568" s="12"/>
+      <c r="A568" s="6" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B568" s="7" t="n">
+        <v>7627</v>
+      </c>
+      <c r="C568" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D568" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E568" s="9" t="n">
+        <v>0.681377314814815</v>
+      </c>
+      <c r="F568" s="9" t="n">
+        <v>0.692604166666667</v>
+      </c>
+      <c r="G568" s="9" t="n">
+        <v>0.285300925925926</v>
+      </c>
+      <c r="H568" s="12" t="n">
+        <v>383</v>
+      </c>
+      <c r="I568" s="10" t="n">
+        <v>2028033</v>
+      </c>
     </row>
     <row r="569" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H569" s="12"/>
+      <c r="A569" s="6" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B569" s="7" t="n">
+        <v>7634</v>
+      </c>
+      <c r="C569" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D569" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E569" s="9" t="n">
+        <v>0.693645833333333</v>
+      </c>
+      <c r="F569" s="9" t="n">
+        <v>0.705023148148148</v>
+      </c>
+      <c r="G569" s="9" t="n">
+        <v>0.285300925925926</v>
+      </c>
+      <c r="H569" s="12" t="n">
+        <v>272</v>
+      </c>
+      <c r="I569" s="10" t="n">
+        <v>1333224</v>
+      </c>
     </row>
     <row r="570" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H570" s="12"/>
+      <c r="A570" s="6" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B570" s="7" t="n">
+        <v>7637</v>
+      </c>
+      <c r="C570" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D570" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E570" s="9" t="n">
+        <v>0.706412037037037</v>
+      </c>
+      <c r="F570" s="9" t="n">
+        <v>0.723101851851852</v>
+      </c>
+      <c r="G570" s="9" t="n">
+        <v>0.285300925925926</v>
+      </c>
+      <c r="H570" s="12" t="n">
+        <v>508</v>
+      </c>
+      <c r="I570" s="10" t="n">
+        <v>2841372</v>
+      </c>
     </row>
     <row r="571" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H571" s="12"/>
+      <c r="A571" s="6" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B571" s="7" t="n">
+        <v>7649</v>
+      </c>
+      <c r="C571" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D571" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E571" s="9" t="n">
+        <v>0.726469907407407</v>
+      </c>
+      <c r="F571" s="9" t="n">
+        <v>0.740104166666667</v>
+      </c>
+      <c r="G571" s="9" t="n">
+        <v>0.285300925925926</v>
+      </c>
+      <c r="H571" s="12" t="n">
+        <v>288</v>
+      </c>
+      <c r="I571" s="10" t="n">
+        <v>1762488</v>
+      </c>
     </row>
     <row r="572" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H572" s="12"/>
+      <c r="A572" s="6" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B572" s="7" t="n">
+        <v>7675</v>
+      </c>
+      <c r="C572" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D572" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E572" s="9" t="n">
+        <v>0.741423611111111</v>
+      </c>
+      <c r="F572" s="9" t="n">
+        <v>0.750844907407407</v>
+      </c>
+      <c r="G572" s="9" t="n">
+        <v>0.285300925925926</v>
+      </c>
+      <c r="H572" s="12" t="n">
+        <v>225</v>
+      </c>
+      <c r="I572" s="10" t="n">
+        <v>1074317</v>
+      </c>
     </row>
     <row r="573" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H573" s="12"/>
+      <c r="A573" s="6" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B573" s="7" t="n">
+        <v>7677</v>
+      </c>
+      <c r="C573" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D573" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E573" s="9" t="n">
+        <v>0.752465277777778</v>
+      </c>
+      <c r="F573" s="9" t="n">
+        <v>0.760231481481482</v>
+      </c>
+      <c r="G573" s="9" t="n">
+        <v>0.285300925925926</v>
+      </c>
+      <c r="H573" s="12" t="n">
+        <v>226</v>
+      </c>
+      <c r="I573" s="10" t="n">
+        <v>1245988</v>
+      </c>
     </row>
     <row r="574" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H574" s="12"/>
+      <c r="A574" s="6" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B574" s="7" t="n">
+        <v>7681</v>
+      </c>
+      <c r="C574" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D574" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E574" s="9" t="n">
+        <v>0.761273148148148</v>
+      </c>
+      <c r="F574" s="9" t="n">
+        <v>0.775844907407407</v>
+      </c>
+      <c r="G574" s="9" t="n">
+        <v>0.285300925925926</v>
+      </c>
+      <c r="H574" s="12" t="n">
+        <v>532</v>
+      </c>
+      <c r="I574" s="10" t="n">
+        <v>2722707</v>
+      </c>
     </row>
     <row r="575" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H575" s="12"/>
+      <c r="A575" s="6" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B575" s="7" t="n">
+        <v>7692</v>
+      </c>
+      <c r="C575" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D575" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E575" s="9" t="n">
+        <v>0.7778125</v>
+      </c>
+      <c r="F575" s="9" t="n">
+        <v>0.794513888888889</v>
+      </c>
+      <c r="G575" s="9" t="n">
+        <v>0.285300925925926</v>
+      </c>
+      <c r="H575" s="12" t="n">
+        <v>415</v>
+      </c>
+      <c r="I575" s="10" t="n">
+        <v>2091337</v>
+      </c>
     </row>
     <row r="576" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H576" s="12"/>
+      <c r="A576" s="6" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B576" s="7" t="n">
+        <v>7729</v>
+      </c>
+      <c r="C576" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D576" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E576" s="9" t="n">
+        <v>0.795810185185185</v>
+      </c>
+      <c r="F576" s="9" t="n">
+        <v>0.805474537037037</v>
+      </c>
+      <c r="G576" s="9" t="n">
+        <v>0.285300925925926</v>
+      </c>
+      <c r="H576" s="12" t="n">
+        <v>263</v>
+      </c>
+      <c r="I576" s="10" t="n">
+        <v>1313091</v>
+      </c>
     </row>
     <row r="577" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H577" s="12"/>
+      <c r="A577" s="6" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B577" s="7" t="n">
+        <v>304</v>
+      </c>
+      <c r="C577" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D577" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E577" s="9" t="n">
+        <v>0.832824074074074</v>
+      </c>
+      <c r="F577" s="9" t="n">
+        <v>0.850138888888889</v>
+      </c>
+      <c r="G577" s="9" t="n">
+        <v>0.285300925925926</v>
+      </c>
+      <c r="H577" s="12" t="n">
+        <v>1286</v>
+      </c>
+      <c r="I577" s="10" t="n">
+        <v>3063869</v>
+      </c>
     </row>
     <row r="578" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H578" s="12"/>
+      <c r="A578" s="6" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B578" s="7" t="n">
+        <v>307</v>
+      </c>
+      <c r="C578" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D578" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E578" s="9" t="n">
+        <v>0.851851851851852</v>
+      </c>
+      <c r="F578" s="9" t="n">
+        <v>0.865671296296296</v>
+      </c>
+      <c r="G578" s="9" t="n">
+        <v>0.285300925925926</v>
+      </c>
+      <c r="H578" s="12" t="n">
+        <v>1048</v>
+      </c>
+      <c r="I578" s="10" t="n">
+        <v>2355209</v>
+      </c>
     </row>
     <row r="579" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H579" s="12"/>
+      <c r="A579" s="6" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B579" s="7" t="n">
+        <v>309</v>
+      </c>
+      <c r="C579" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D579" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E579" s="9" t="n">
+        <v>0.867199074074074</v>
+      </c>
+      <c r="F579" s="9" t="n">
+        <v>0.882534722222222</v>
+      </c>
+      <c r="G579" s="9" t="n">
+        <v>0.285300925925926</v>
+      </c>
+      <c r="H579" s="12" t="n">
+        <v>1091</v>
+      </c>
+      <c r="I579" s="10" t="n">
+        <v>2478938</v>
+      </c>
     </row>
     <row r="580" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H580" s="12"/>
+      <c r="A580" s="6" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B580" s="7" t="n">
+        <v>312</v>
+      </c>
+      <c r="C580" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D580" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E580" s="9" t="n">
+        <v>0.884016203703704</v>
+      </c>
+      <c r="F580" s="9" t="n">
+        <v>0.903414351851852</v>
+      </c>
+      <c r="G580" s="9" t="n">
+        <v>0.285300925925926</v>
+      </c>
+      <c r="H580" s="12" t="n">
+        <v>1130</v>
+      </c>
+      <c r="I580" s="10" t="n">
+        <v>2802889</v>
+      </c>
     </row>
     <row r="581" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H581" s="12"/>
+      <c r="A581" s="6" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B581" s="7" t="n">
+        <v>315</v>
+      </c>
+      <c r="C581" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D581" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E581" s="9" t="n">
+        <v>0.905335648148148</v>
+      </c>
+      <c r="F581" s="9" t="n">
+        <v>0.918321759259259</v>
+      </c>
+      <c r="G581" s="9" t="n">
+        <v>0.285300925925926</v>
+      </c>
+      <c r="H581" s="12" t="n">
+        <v>494</v>
+      </c>
+      <c r="I581" s="10" t="n">
+        <v>3972162</v>
+      </c>
     </row>
     <row r="582" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H582" s="12"/>
+      <c r="A582" s="6" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B582" s="7" t="n">
+        <v>201</v>
+      </c>
+      <c r="C582" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D582" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E582" s="9" t="n">
+        <v>0.920162037037037</v>
+      </c>
+      <c r="F582" s="9" t="n">
+        <v>0.938449074074074</v>
+      </c>
+      <c r="G582" s="9" t="n">
+        <v>0.285300925925926</v>
+      </c>
+      <c r="H582" s="12" t="n">
+        <v>1408</v>
+      </c>
+      <c r="I582" s="10" t="n">
+        <v>3213641</v>
+      </c>
     </row>
     <row r="583" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H583" s="12"/>
+      <c r="A583" s="6" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B583" s="7" t="n">
+        <v>209</v>
+      </c>
+      <c r="C583" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D583" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E583" s="9" t="n">
+        <v>0.94005787037037</v>
+      </c>
+      <c r="F583" s="9" t="n">
+        <v>0.966400462962963</v>
+      </c>
+      <c r="G583" s="9" t="n">
+        <v>0.285300925925926</v>
+      </c>
+      <c r="H583" s="12" t="n">
+        <v>1535</v>
+      </c>
+      <c r="I583" s="10" t="n">
+        <v>4295208</v>
+      </c>
     </row>
     <row r="584" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H584" s="12"/>
+      <c r="A584" s="6" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B584" s="7" t="n">
+        <v>252</v>
+      </c>
+      <c r="C584" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D584" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E584" s="9" t="n">
+        <v>0.969340277777778</v>
+      </c>
+      <c r="F584" s="9" t="n">
+        <v>0.985092592592593</v>
+      </c>
+      <c r="G584" s="9" t="n">
+        <v>0.285300925925926</v>
+      </c>
+      <c r="H584" s="12" t="n">
+        <v>916</v>
+      </c>
+      <c r="I584" s="10" t="n">
+        <v>1987151</v>
+      </c>
     </row>
     <row r="585" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H585" s="12"/>
+      <c r="A585" s="6" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B585" s="7" t="n">
+        <v>256</v>
+      </c>
+      <c r="C585" s="8" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D585" s="8" t="n">
+        <v>0.0416666666666667</v>
+      </c>
+      <c r="E585" s="9" t="n">
+        <v>0.986134259259259</v>
+      </c>
+      <c r="F585" s="9" t="n">
+        <v>0.998217592592593</v>
+      </c>
+      <c r="G585" s="9" t="n">
+        <v>0.285300925925926</v>
+      </c>
+      <c r="H585" s="12" t="n">
+        <v>1300</v>
+      </c>
+      <c r="I585" s="10" t="n">
+        <v>2733794</v>
+      </c>
     </row>
     <row r="586" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A586" s="6"/>
       <c r="H586" s="12"/>
+      <c r="I586" s="10"/>
     </row>
     <row r="587" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H587" s="12"/>
@@ -18047,15 +18595,15 @@
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="C2:D564" type="custom">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="C2:D585" type="custom">
       <formula1>OR(TIMEVALUE(TEXT(C2, "hh:mm:ss"))=C2, AND(ISNUMBER(C2), LEFT(CELL("format", C2))="D"))</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="A2:A564" type="custom">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="A2:A586" type="custom">
       <formula1>OR(NOT(ISERROR(DATEVALUE(A2))), AND(ISNUMBER(A2), LEFT(CELL("format", A2))="D"))</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="B2:B564 H2:I488 I489:I564 H490:H564" type="custom">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="B2:B565 H2:I488 I489:I586 H490:H564 B566:B585" type="custom">
       <formula1>AND(ISNUMBER(B2),(NOT(OR(NOT(ISERROR(DATEVALUE(B2))), AND(ISNUMBER(B2), LEFT(CELL("format", B2))="D")))))</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Se agregan datos a la fecha
</commit_message>
<xml_diff>
--- a/data/raw/io_data_bimbo.xlsx
+++ b/data/raw/io_data_bimbo.xlsx
@@ -145,7 +145,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -202,6 +202,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="21" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="46" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
@@ -23340,235 +23343,613 @@
       </c>
     </row>
     <row r="791" ht="15.75" customHeight="1">
-      <c r="A791" s="3"/>
-      <c r="B791" s="4"/>
-      <c r="C791" s="8"/>
-      <c r="D791" s="8"/>
-      <c r="E791" s="5"/>
-      <c r="F791" s="5"/>
-      <c r="G791" s="19"/>
-      <c r="H791" s="12"/>
-      <c r="I791" s="19"/>
+      <c r="A791" s="13">
+        <v>46239.0</v>
+      </c>
+      <c r="B791" s="14">
+        <v>9378.0</v>
+      </c>
+      <c r="C791" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D791" s="15">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="E791" s="16">
+        <v>0.638900462962963</v>
+      </c>
+      <c r="F791" s="16">
+        <v>0.6465972222222223</v>
+      </c>
+      <c r="G791" s="19">
+        <v>0.24149305555555678</v>
+      </c>
+      <c r="H791" s="17">
+        <v>136.0</v>
+      </c>
+      <c r="I791" s="11">
+        <v>424280.0</v>
+      </c>
     </row>
     <row r="792" ht="15.75" customHeight="1">
-      <c r="A792" s="3"/>
-      <c r="B792" s="4"/>
-      <c r="C792" s="8"/>
-      <c r="D792" s="8"/>
-      <c r="E792" s="5"/>
-      <c r="F792" s="5"/>
-      <c r="G792" s="19"/>
-      <c r="H792" s="12"/>
-      <c r="I792" s="19"/>
+      <c r="A792" s="13">
+        <v>46239.0</v>
+      </c>
+      <c r="B792" s="14">
+        <v>9379.0</v>
+      </c>
+      <c r="C792" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D792" s="15">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="E792" s="16">
+        <v>0.6473842592592592</v>
+      </c>
+      <c r="F792" s="16">
+        <v>0.6530439814814815</v>
+      </c>
+      <c r="G792" s="19">
+        <v>0.24149305555555678</v>
+      </c>
+      <c r="H792" s="17">
+        <v>145.0</v>
+      </c>
+      <c r="I792" s="11">
+        <v>570712.0</v>
+      </c>
     </row>
     <row r="793" ht="15.75" customHeight="1">
-      <c r="A793" s="3"/>
-      <c r="B793" s="4"/>
-      <c r="C793" s="8"/>
-      <c r="D793" s="8"/>
-      <c r="E793" s="5"/>
-      <c r="F793" s="5"/>
-      <c r="G793" s="19"/>
-      <c r="H793" s="12"/>
-      <c r="I793" s="19"/>
+      <c r="A793" s="13">
+        <v>46239.0</v>
+      </c>
+      <c r="B793" s="14">
+        <v>9382.0</v>
+      </c>
+      <c r="C793" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D793" s="15">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="E793" s="16">
+        <v>0.6540625</v>
+      </c>
+      <c r="F793" s="16">
+        <v>0.6585069444444445</v>
+      </c>
+      <c r="G793" s="19">
+        <v>0.24149305555555678</v>
+      </c>
+      <c r="H793" s="17">
+        <v>112.0</v>
+      </c>
+      <c r="I793" s="11">
+        <v>398206.0</v>
+      </c>
     </row>
     <row r="794" ht="15.75" customHeight="1">
-      <c r="A794" s="3"/>
-      <c r="B794" s="4"/>
-      <c r="C794" s="8"/>
-      <c r="D794" s="8"/>
-      <c r="E794" s="5"/>
-      <c r="F794" s="5"/>
-      <c r="G794" s="19"/>
-      <c r="H794" s="12"/>
-      <c r="I794" s="19"/>
+      <c r="A794" s="13">
+        <v>46239.0</v>
+      </c>
+      <c r="B794" s="14">
+        <v>9386.0</v>
+      </c>
+      <c r="C794" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D794" s="15">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="E794" s="16">
+        <v>0.6604050925925926</v>
+      </c>
+      <c r="F794" s="16">
+        <v>0.6657523148148148</v>
+      </c>
+      <c r="G794" s="19">
+        <v>0.24149305555555678</v>
+      </c>
+      <c r="H794" s="17">
+        <v>136.0</v>
+      </c>
+      <c r="I794" s="11">
+        <v>490346.0</v>
+      </c>
     </row>
     <row r="795" ht="15.75" customHeight="1">
-      <c r="A795" s="3"/>
-      <c r="B795" s="4"/>
-      <c r="C795" s="8"/>
-      <c r="D795" s="8"/>
-      <c r="E795" s="5"/>
-      <c r="F795" s="5"/>
-      <c r="G795" s="19"/>
-      <c r="H795" s="12"/>
-      <c r="I795" s="19"/>
+      <c r="A795" s="13">
+        <v>46239.0</v>
+      </c>
+      <c r="B795" s="14">
+        <v>7623.0</v>
+      </c>
+      <c r="C795" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D795" s="15">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="E795" s="16">
+        <v>0.6666319444444444</v>
+      </c>
+      <c r="F795" s="16">
+        <v>0.6738310185185186</v>
+      </c>
+      <c r="G795" s="19">
+        <v>0.24149305555555678</v>
+      </c>
+      <c r="H795" s="17">
+        <v>155.0</v>
+      </c>
+      <c r="I795" s="11">
+        <v>830379.0</v>
+      </c>
     </row>
     <row r="796" ht="15.75" customHeight="1">
-      <c r="A796" s="3"/>
-      <c r="B796" s="4"/>
-      <c r="C796" s="8"/>
-      <c r="D796" s="8"/>
-      <c r="E796" s="5"/>
-      <c r="F796" s="5"/>
-      <c r="G796" s="19"/>
-      <c r="H796" s="12"/>
-      <c r="I796" s="19"/>
+      <c r="A796" s="13">
+        <v>46239.0</v>
+      </c>
+      <c r="B796" s="14">
+        <v>7620.0</v>
+      </c>
+      <c r="C796" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D796" s="15">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="E796" s="16">
+        <v>0.6748611111111111</v>
+      </c>
+      <c r="F796" s="16">
+        <v>0.6816550925925926</v>
+      </c>
+      <c r="G796" s="19">
+        <v>0.24149305555555678</v>
+      </c>
+      <c r="H796" s="17">
+        <v>99.0</v>
+      </c>
+      <c r="I796" s="11">
+        <v>527780.0</v>
+      </c>
     </row>
     <row r="797" ht="15.75" customHeight="1">
-      <c r="A797" s="3"/>
-      <c r="B797" s="4"/>
-      <c r="C797" s="8"/>
-      <c r="D797" s="8"/>
-      <c r="E797" s="5"/>
-      <c r="F797" s="5"/>
-      <c r="G797" s="19"/>
-      <c r="H797" s="12"/>
-      <c r="I797" s="19"/>
+      <c r="A797" s="13">
+        <v>46239.0</v>
+      </c>
+      <c r="B797" s="14">
+        <v>7624.0</v>
+      </c>
+      <c r="C797" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D797" s="15">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="E797" s="16">
+        <v>0.6830787037037037</v>
+      </c>
+      <c r="F797" s="16">
+        <v>0.690150462962963</v>
+      </c>
+      <c r="G797" s="19">
+        <v>0.24149305555555678</v>
+      </c>
+      <c r="H797" s="17">
+        <v>186.0</v>
+      </c>
+      <c r="I797" s="11">
+        <v>1017917.0</v>
+      </c>
     </row>
     <row r="798" ht="15.75" customHeight="1">
-      <c r="A798" s="3"/>
-      <c r="B798" s="4"/>
-      <c r="C798" s="8"/>
-      <c r="D798" s="8"/>
-      <c r="E798" s="5"/>
-      <c r="F798" s="5"/>
-      <c r="G798" s="19"/>
-      <c r="H798" s="12"/>
-      <c r="I798" s="19"/>
+      <c r="A798" s="13">
+        <v>46239.0</v>
+      </c>
+      <c r="B798" s="14">
+        <v>7627.0</v>
+      </c>
+      <c r="C798" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D798" s="15">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="E798" s="16">
+        <v>0.6916203703703704</v>
+      </c>
+      <c r="F798" s="16">
+        <v>0.6972569444444444</v>
+      </c>
+      <c r="G798" s="19">
+        <v>0.24149305555555678</v>
+      </c>
+      <c r="H798" s="17">
+        <v>152.0</v>
+      </c>
+      <c r="I798" s="11">
+        <v>784038.0</v>
+      </c>
     </row>
     <row r="799" ht="15.75" customHeight="1">
-      <c r="A799" s="3"/>
-      <c r="B799" s="4"/>
-      <c r="C799" s="8"/>
-      <c r="D799" s="8"/>
-      <c r="E799" s="5"/>
-      <c r="F799" s="5"/>
-      <c r="G799" s="19"/>
-      <c r="H799" s="12"/>
-      <c r="I799" s="19"/>
+      <c r="A799" s="13">
+        <v>46239.0</v>
+      </c>
+      <c r="B799" s="14">
+        <v>7640.0</v>
+      </c>
+      <c r="C799" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D799" s="15">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="E799" s="16">
+        <v>0.6980902777777778</v>
+      </c>
+      <c r="F799" s="16">
+        <v>0.7048611111111112</v>
+      </c>
+      <c r="G799" s="19">
+        <v>0.24149305555555678</v>
+      </c>
+      <c r="H799" s="17">
+        <v>133.0</v>
+      </c>
+      <c r="I799" s="11">
+        <v>667269.0</v>
+      </c>
     </row>
     <row r="800" ht="15.75" customHeight="1">
-      <c r="A800" s="3"/>
-      <c r="B800" s="4"/>
-      <c r="C800" s="8"/>
-      <c r="D800" s="8"/>
-      <c r="E800" s="5"/>
-      <c r="F800" s="5"/>
-      <c r="G800" s="19"/>
-      <c r="H800" s="12"/>
-      <c r="I800" s="19"/>
+      <c r="A800" s="13">
+        <v>46239.0</v>
+      </c>
+      <c r="B800" s="14">
+        <v>7663.0</v>
+      </c>
+      <c r="C800" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D800" s="15">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="E800" s="16">
+        <v>0.7067708333333333</v>
+      </c>
+      <c r="F800" s="16">
+        <v>0.7156018518518519</v>
+      </c>
+      <c r="G800" s="19">
+        <v>0.24149305555555678</v>
+      </c>
+      <c r="H800" s="17">
+        <v>313.0</v>
+      </c>
+      <c r="I800" s="11">
+        <v>1438947.0</v>
+      </c>
     </row>
     <row r="801" ht="15.75" customHeight="1">
-      <c r="A801" s="3"/>
-      <c r="B801" s="4"/>
-      <c r="C801" s="8"/>
-      <c r="D801" s="8"/>
-      <c r="E801" s="5"/>
-      <c r="F801" s="5"/>
-      <c r="G801" s="19"/>
-      <c r="H801" s="12"/>
-      <c r="I801" s="19"/>
+      <c r="A801" s="13">
+        <v>46239.0</v>
+      </c>
+      <c r="B801" s="14">
+        <v>7706.0</v>
+      </c>
+      <c r="C801" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D801" s="15">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="E801" s="16">
+        <v>0.7166898148148149</v>
+      </c>
+      <c r="F801" s="16">
+        <v>0.724212962962963</v>
+      </c>
+      <c r="G801" s="19">
+        <v>0.24149305555555678</v>
+      </c>
+      <c r="H801" s="17">
+        <v>94.0</v>
+      </c>
+      <c r="I801" s="11">
+        <v>413581.0</v>
+      </c>
     </row>
     <row r="802" ht="15.75" customHeight="1">
-      <c r="A802" s="3"/>
-      <c r="B802" s="4"/>
-      <c r="C802" s="8"/>
-      <c r="D802" s="8"/>
-      <c r="E802" s="5"/>
-      <c r="F802" s="5"/>
-      <c r="G802" s="19"/>
-      <c r="H802" s="12"/>
-      <c r="I802" s="19"/>
+      <c r="A802" s="13">
+        <v>46239.0</v>
+      </c>
+      <c r="B802" s="14">
+        <v>7719.0</v>
+      </c>
+      <c r="C802" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D802" s="15">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="E802" s="16">
+        <v>0.7253587962962963</v>
+      </c>
+      <c r="F802" s="16">
+        <v>0.729375</v>
+      </c>
+      <c r="G802" s="19">
+        <v>0.24149305555555678</v>
+      </c>
+      <c r="H802" s="17">
+        <v>155.0</v>
+      </c>
+      <c r="I802" s="11">
+        <v>723969.0</v>
+      </c>
     </row>
     <row r="803" ht="15.75" customHeight="1">
-      <c r="A803" s="3"/>
-      <c r="B803" s="4"/>
-      <c r="C803" s="8"/>
-      <c r="D803" s="8"/>
-      <c r="E803" s="5"/>
-      <c r="F803" s="5"/>
-      <c r="G803" s="19"/>
-      <c r="H803" s="12"/>
-      <c r="I803" s="19"/>
+      <c r="A803" s="13">
+        <v>46239.0</v>
+      </c>
+      <c r="B803" s="14">
+        <v>7728.0</v>
+      </c>
+      <c r="C803" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D803" s="15">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="E803" s="16">
+        <v>0.7301620370370371</v>
+      </c>
+      <c r="F803" s="16">
+        <v>0.7392592592592593</v>
+      </c>
+      <c r="G803" s="19">
+        <v>0.24149305555555678</v>
+      </c>
+      <c r="H803" s="17">
+        <v>198.0</v>
+      </c>
+      <c r="I803" s="11">
+        <v>811930.0</v>
+      </c>
     </row>
     <row r="804" ht="15.75" customHeight="1">
-      <c r="A804" s="3"/>
-      <c r="B804" s="4"/>
-      <c r="C804" s="8"/>
-      <c r="D804" s="8"/>
-      <c r="E804" s="5"/>
-      <c r="F804" s="5"/>
-      <c r="G804" s="19"/>
-      <c r="H804" s="12"/>
-      <c r="I804" s="19"/>
+      <c r="A804" s="13">
+        <v>46239.0</v>
+      </c>
+      <c r="B804" s="14">
+        <v>7742.0</v>
+      </c>
+      <c r="C804" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D804" s="15">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="E804" s="16">
+        <v>0.7419907407407408</v>
+      </c>
+      <c r="F804" s="16">
+        <v>0.7477083333333333</v>
+      </c>
+      <c r="G804" s="19">
+        <v>0.24149305555555678</v>
+      </c>
+      <c r="H804" s="17">
+        <v>194.0</v>
+      </c>
+      <c r="I804" s="11">
+        <v>615805.0</v>
+      </c>
     </row>
     <row r="805" ht="15.75" customHeight="1">
-      <c r="A805" s="3"/>
-      <c r="B805" s="4"/>
-      <c r="C805" s="8"/>
-      <c r="D805" s="8"/>
-      <c r="E805" s="5"/>
-      <c r="F805" s="5"/>
-      <c r="G805" s="19"/>
-      <c r="H805" s="12"/>
-      <c r="I805" s="19"/>
+      <c r="A805" s="13">
+        <v>46239.0</v>
+      </c>
+      <c r="B805" s="14">
+        <v>306.0</v>
+      </c>
+      <c r="C805" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D805" s="15">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="E805" s="16">
+        <v>0.7731712962962963</v>
+      </c>
+      <c r="F805" s="16">
+        <v>0.7921759259259259</v>
+      </c>
+      <c r="G805" s="19">
+        <v>0.24149305555555678</v>
+      </c>
+      <c r="H805" s="17">
+        <v>954.0</v>
+      </c>
+      <c r="I805" s="11">
+        <v>2375290.0</v>
+      </c>
     </row>
     <row r="806" ht="15.75" customHeight="1">
-      <c r="A806" s="3"/>
-      <c r="B806" s="4"/>
-      <c r="C806" s="8"/>
-      <c r="D806" s="8"/>
-      <c r="E806" s="5"/>
-      <c r="F806" s="5"/>
-      <c r="G806" s="19"/>
-      <c r="H806" s="12"/>
-      <c r="I806" s="19"/>
+      <c r="A806" s="13">
+        <v>46239.0</v>
+      </c>
+      <c r="B806" s="14">
+        <v>308.0</v>
+      </c>
+      <c r="C806" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D806" s="15">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="E806" s="16">
+        <v>0.7937152777777777</v>
+      </c>
+      <c r="F806" s="16">
+        <v>0.8050462962962963</v>
+      </c>
+      <c r="G806" s="19">
+        <v>0.24149305555555678</v>
+      </c>
+      <c r="H806" s="17">
+        <v>721.0</v>
+      </c>
+      <c r="I806" s="11">
+        <v>1543771.0</v>
+      </c>
     </row>
     <row r="807" ht="15.75" customHeight="1">
-      <c r="A807" s="3"/>
-      <c r="B807" s="4"/>
-      <c r="C807" s="8"/>
-      <c r="D807" s="8"/>
-      <c r="E807" s="5"/>
-      <c r="F807" s="5"/>
-      <c r="G807" s="19"/>
-      <c r="H807" s="12"/>
-      <c r="I807" s="19"/>
+      <c r="A807" s="13">
+        <v>46239.0</v>
+      </c>
+      <c r="B807" s="14">
+        <v>312.0</v>
+      </c>
+      <c r="C807" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D807" s="15">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="E807" s="16">
+        <v>0.8062962962962963</v>
+      </c>
+      <c r="F807" s="16">
+        <v>0.8328819444444444</v>
+      </c>
+      <c r="G807" s="19">
+        <v>0.24149305555555678</v>
+      </c>
+      <c r="H807" s="17">
+        <v>1059.0</v>
+      </c>
+      <c r="I807" s="11">
+        <v>2834399.0</v>
+      </c>
     </row>
     <row r="808" ht="15.75" customHeight="1">
-      <c r="A808" s="3"/>
-      <c r="B808" s="4"/>
-      <c r="C808" s="8"/>
-      <c r="D808" s="8"/>
-      <c r="E808" s="5"/>
-      <c r="F808" s="5"/>
-      <c r="G808" s="19"/>
-      <c r="H808" s="12"/>
-      <c r="I808" s="19"/>
+      <c r="A808" s="13">
+        <v>46239.0</v>
+      </c>
+      <c r="B808" s="14">
+        <v>1259.0</v>
+      </c>
+      <c r="C808" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D808" s="15">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="E808" s="16">
+        <v>0.834837962962963</v>
+      </c>
+      <c r="F808" s="16">
+        <v>0.8709143518518518</v>
+      </c>
+      <c r="G808" s="19">
+        <v>0.24149305555555678</v>
+      </c>
+      <c r="H808" s="17">
+        <v>1908.0</v>
+      </c>
+      <c r="I808" s="11">
+        <v>8919716.0</v>
+      </c>
     </row>
     <row r="809" ht="15.75" customHeight="1">
-      <c r="A809" s="3"/>
-      <c r="B809" s="4"/>
-      <c r="C809" s="8"/>
-      <c r="D809" s="8"/>
-      <c r="E809" s="5"/>
-      <c r="F809" s="5"/>
-      <c r="G809" s="19"/>
-      <c r="H809" s="12"/>
-      <c r="I809" s="19"/>
+      <c r="A809" s="13">
+        <v>46239.0</v>
+      </c>
+      <c r="B809" s="14">
+        <v>212.0</v>
+      </c>
+      <c r="C809" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D809" s="15">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="E809" s="16">
+        <v>0.8746990740740741</v>
+      </c>
+      <c r="F809" s="16">
+        <v>0.9003935185185186</v>
+      </c>
+      <c r="G809" s="19">
+        <v>0.24149305555555678</v>
+      </c>
+      <c r="H809" s="17">
+        <v>1287.0</v>
+      </c>
+      <c r="I809" s="11">
+        <v>4050639.0</v>
+      </c>
     </row>
     <row r="810" ht="15.75" customHeight="1">
-      <c r="A810" s="3"/>
-      <c r="B810" s="4"/>
-      <c r="C810" s="8"/>
-      <c r="D810" s="8"/>
-      <c r="E810" s="5"/>
-      <c r="F810" s="5"/>
-      <c r="G810" s="19"/>
-      <c r="H810" s="12"/>
-      <c r="I810" s="19"/>
+      <c r="A810" s="13">
+        <v>46239.0</v>
+      </c>
+      <c r="B810" s="14">
+        <v>256.0</v>
+      </c>
+      <c r="C810" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D810" s="15">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="E810" s="16">
+        <v>0.9028356481481481</v>
+      </c>
+      <c r="F810" s="16">
+        <v>0.9190046296296296</v>
+      </c>
+      <c r="G810" s="19">
+        <v>0.24149305555555678</v>
+      </c>
+      <c r="H810" s="17">
+        <v>1100.0</v>
+      </c>
+      <c r="I810" s="11">
+        <v>2379253.0</v>
+      </c>
     </row>
     <row r="811" ht="15.75" customHeight="1">
-      <c r="A811" s="3"/>
-      <c r="B811" s="4"/>
-      <c r="C811" s="8"/>
-      <c r="D811" s="8"/>
-      <c r="E811" s="5"/>
-      <c r="F811" s="5"/>
-      <c r="G811" s="19"/>
-      <c r="H811" s="12"/>
-      <c r="I811" s="19"/>
+      <c r="A811" s="13">
+        <v>46239.0</v>
+      </c>
+      <c r="B811" s="14">
+        <v>261.0</v>
+      </c>
+      <c r="C811" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D811" s="15">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="E811" s="16">
+        <v>0.9206944444444445</v>
+      </c>
+      <c r="F811" s="16">
+        <v>0.9355208333333334</v>
+      </c>
+      <c r="G811" s="19">
+        <v>0.24149305555555678</v>
+      </c>
+      <c r="H811" s="17">
+        <v>983.0</v>
+      </c>
+      <c r="I811" s="11">
+        <v>2169470.0</v>
+      </c>
     </row>
     <row r="812" ht="15.75" customHeight="1">
       <c r="A812" s="3"/>
@@ -23577,9 +23958,9 @@
       <c r="D812" s="8"/>
       <c r="E812" s="5"/>
       <c r="F812" s="5"/>
-      <c r="G812" s="19"/>
+      <c r="G812" s="20"/>
       <c r="H812" s="12"/>
-      <c r="I812" s="19"/>
+      <c r="I812" s="20"/>
     </row>
     <row r="813" ht="15.75" customHeight="1">
       <c r="A813" s="3"/>
@@ -23588,9 +23969,9 @@
       <c r="D813" s="8"/>
       <c r="E813" s="5"/>
       <c r="F813" s="5"/>
-      <c r="G813" s="19"/>
+      <c r="G813" s="20"/>
       <c r="H813" s="12"/>
-      <c r="I813" s="19"/>
+      <c r="I813" s="20"/>
     </row>
     <row r="814" ht="15.75" customHeight="1">
       <c r="A814" s="3"/>
@@ -23599,9 +23980,9 @@
       <c r="D814" s="8"/>
       <c r="E814" s="5"/>
       <c r="F814" s="5"/>
-      <c r="G814" s="19"/>
+      <c r="G814" s="20"/>
       <c r="H814" s="12"/>
-      <c r="I814" s="19"/>
+      <c r="I814" s="20"/>
     </row>
     <row r="815" ht="15.75" customHeight="1">
       <c r="A815" s="3"/>
@@ -23610,9 +23991,9 @@
       <c r="D815" s="8"/>
       <c r="E815" s="5"/>
       <c r="F815" s="5"/>
-      <c r="G815" s="19"/>
+      <c r="G815" s="20"/>
       <c r="H815" s="12"/>
-      <c r="I815" s="19"/>
+      <c r="I815" s="20"/>
     </row>
     <row r="816" ht="15.75" customHeight="1">
       <c r="A816" s="3"/>
@@ -23621,9 +24002,9 @@
       <c r="D816" s="8"/>
       <c r="E816" s="5"/>
       <c r="F816" s="5"/>
-      <c r="G816" s="19"/>
+      <c r="G816" s="20"/>
       <c r="H816" s="12"/>
-      <c r="I816" s="19"/>
+      <c r="I816" s="20"/>
     </row>
     <row r="817" ht="15.75" customHeight="1">
       <c r="A817" s="3"/>
@@ -23632,9 +24013,9 @@
       <c r="D817" s="8"/>
       <c r="E817" s="5"/>
       <c r="F817" s="5"/>
-      <c r="G817" s="19"/>
+      <c r="G817" s="20"/>
       <c r="H817" s="12"/>
-      <c r="I817" s="19"/>
+      <c r="I817" s="20"/>
     </row>
     <row r="818" ht="15.75" customHeight="1">
       <c r="A818" s="3"/>
@@ -23643,9 +24024,9 @@
       <c r="D818" s="8"/>
       <c r="E818" s="5"/>
       <c r="F818" s="5"/>
-      <c r="G818" s="19"/>
+      <c r="G818" s="20"/>
       <c r="H818" s="12"/>
-      <c r="I818" s="19"/>
+      <c r="I818" s="20"/>
     </row>
     <row r="819" ht="15.75" customHeight="1">
       <c r="A819" s="3"/>
@@ -23654,9 +24035,9 @@
       <c r="D819" s="8"/>
       <c r="E819" s="5"/>
       <c r="F819" s="5"/>
-      <c r="G819" s="19"/>
+      <c r="G819" s="20"/>
       <c r="H819" s="12"/>
-      <c r="I819" s="19"/>
+      <c r="I819" s="20"/>
     </row>
     <row r="820" ht="15.75" customHeight="1">
       <c r="A820" s="3"/>
@@ -23665,9 +24046,9 @@
       <c r="D820" s="8"/>
       <c r="E820" s="5"/>
       <c r="F820" s="5"/>
-      <c r="G820" s="19"/>
+      <c r="G820" s="20"/>
       <c r="H820" s="12"/>
-      <c r="I820" s="19"/>
+      <c r="I820" s="20"/>
     </row>
     <row r="821" ht="15.75" customHeight="1">
       <c r="A821" s="3"/>
@@ -23676,9 +24057,9 @@
       <c r="D821" s="8"/>
       <c r="E821" s="5"/>
       <c r="F821" s="5"/>
-      <c r="G821" s="19"/>
+      <c r="G821" s="20"/>
       <c r="H821" s="12"/>
-      <c r="I821" s="19"/>
+      <c r="I821" s="20"/>
     </row>
     <row r="822" ht="15.75" customHeight="1">
       <c r="A822" s="3"/>
@@ -23687,9 +24068,9 @@
       <c r="D822" s="8"/>
       <c r="E822" s="5"/>
       <c r="F822" s="5"/>
-      <c r="G822" s="19"/>
+      <c r="G822" s="20"/>
       <c r="H822" s="12"/>
-      <c r="I822" s="19"/>
+      <c r="I822" s="20"/>
     </row>
     <row r="823" ht="15.75" customHeight="1">
       <c r="A823" s="3"/>
@@ -23698,9 +24079,9 @@
       <c r="D823" s="8"/>
       <c r="E823" s="5"/>
       <c r="F823" s="5"/>
-      <c r="G823" s="19"/>
+      <c r="G823" s="20"/>
       <c r="H823" s="12"/>
-      <c r="I823" s="19"/>
+      <c r="I823" s="20"/>
     </row>
     <row r="824" ht="15.75" customHeight="1">
       <c r="A824" s="3"/>
@@ -23709,9 +24090,9 @@
       <c r="D824" s="8"/>
       <c r="E824" s="5"/>
       <c r="F824" s="5"/>
-      <c r="G824" s="19"/>
+      <c r="G824" s="20"/>
       <c r="H824" s="12"/>
-      <c r="I824" s="19"/>
+      <c r="I824" s="20"/>
     </row>
     <row r="825" ht="15.75" customHeight="1">
       <c r="A825" s="3"/>
@@ -23720,9 +24101,9 @@
       <c r="D825" s="8"/>
       <c r="E825" s="5"/>
       <c r="F825" s="5"/>
-      <c r="G825" s="19"/>
+      <c r="G825" s="20"/>
       <c r="H825" s="12"/>
-      <c r="I825" s="19"/>
+      <c r="I825" s="20"/>
     </row>
     <row r="826" ht="15.75" customHeight="1">
       <c r="A826" s="3"/>
@@ -23731,9 +24112,9 @@
       <c r="D826" s="8"/>
       <c r="E826" s="5"/>
       <c r="F826" s="5"/>
-      <c r="G826" s="19"/>
+      <c r="G826" s="20"/>
       <c r="H826" s="12"/>
-      <c r="I826" s="19"/>
+      <c r="I826" s="20"/>
     </row>
     <row r="827" ht="15.75" customHeight="1">
       <c r="A827" s="3"/>
@@ -23742,9 +24123,9 @@
       <c r="D827" s="8"/>
       <c r="E827" s="5"/>
       <c r="F827" s="5"/>
-      <c r="G827" s="19"/>
+      <c r="G827" s="20"/>
       <c r="H827" s="12"/>
-      <c r="I827" s="19"/>
+      <c r="I827" s="20"/>
     </row>
     <row r="828" ht="15.75" customHeight="1">
       <c r="A828" s="3"/>
@@ -23753,9 +24134,9 @@
       <c r="D828" s="8"/>
       <c r="E828" s="5"/>
       <c r="F828" s="5"/>
-      <c r="G828" s="19"/>
+      <c r="G828" s="20"/>
       <c r="H828" s="12"/>
-      <c r="I828" s="19"/>
+      <c r="I828" s="20"/>
     </row>
     <row r="829" ht="15.75" customHeight="1">
       <c r="A829" s="3"/>
@@ -23764,9 +24145,9 @@
       <c r="D829" s="8"/>
       <c r="E829" s="5"/>
       <c r="F829" s="5"/>
-      <c r="G829" s="19"/>
+      <c r="G829" s="20"/>
       <c r="H829" s="12"/>
-      <c r="I829" s="19"/>
+      <c r="I829" s="20"/>
     </row>
     <row r="830" ht="15.75" customHeight="1">
       <c r="A830" s="3"/>
@@ -23775,9 +24156,9 @@
       <c r="D830" s="8"/>
       <c r="E830" s="5"/>
       <c r="F830" s="5"/>
-      <c r="G830" s="19"/>
+      <c r="G830" s="20"/>
       <c r="H830" s="12"/>
-      <c r="I830" s="19"/>
+      <c r="I830" s="20"/>
     </row>
     <row r="831" ht="15.75" customHeight="1">
       <c r="A831" s="3"/>
@@ -23786,9 +24167,9 @@
       <c r="D831" s="8"/>
       <c r="E831" s="5"/>
       <c r="F831" s="5"/>
-      <c r="G831" s="19"/>
+      <c r="G831" s="20"/>
       <c r="H831" s="12"/>
-      <c r="I831" s="19"/>
+      <c r="I831" s="20"/>
     </row>
     <row r="832" ht="15.75" customHeight="1">
       <c r="A832" s="3"/>
@@ -23797,9 +24178,9 @@
       <c r="D832" s="8"/>
       <c r="E832" s="5"/>
       <c r="F832" s="5"/>
-      <c r="G832" s="19"/>
+      <c r="G832" s="20"/>
       <c r="H832" s="12"/>
-      <c r="I832" s="19"/>
+      <c r="I832" s="20"/>
     </row>
     <row r="833" ht="15.75" customHeight="1">
       <c r="A833" s="3"/>
@@ -23808,9 +24189,9 @@
       <c r="D833" s="8"/>
       <c r="E833" s="5"/>
       <c r="F833" s="5"/>
-      <c r="G833" s="19"/>
+      <c r="G833" s="20"/>
       <c r="H833" s="12"/>
-      <c r="I833" s="19"/>
+      <c r="I833" s="20"/>
     </row>
     <row r="834" ht="15.75" customHeight="1">
       <c r="A834" s="3"/>
@@ -23819,9 +24200,9 @@
       <c r="D834" s="8"/>
       <c r="E834" s="5"/>
       <c r="F834" s="5"/>
-      <c r="G834" s="19"/>
+      <c r="G834" s="20"/>
       <c r="H834" s="12"/>
-      <c r="I834" s="19"/>
+      <c r="I834" s="20"/>
     </row>
     <row r="835" ht="15.75" customHeight="1">
       <c r="A835" s="3"/>
@@ -23830,9 +24211,9 @@
       <c r="D835" s="8"/>
       <c r="E835" s="5"/>
       <c r="F835" s="5"/>
-      <c r="G835" s="19"/>
+      <c r="G835" s="20"/>
       <c r="H835" s="12"/>
-      <c r="I835" s="19"/>
+      <c r="I835" s="20"/>
     </row>
     <row r="836" ht="15.75" customHeight="1">
       <c r="A836" s="3"/>
@@ -23841,9 +24222,9 @@
       <c r="D836" s="8"/>
       <c r="E836" s="5"/>
       <c r="F836" s="5"/>
-      <c r="G836" s="19"/>
+      <c r="G836" s="20"/>
       <c r="H836" s="12"/>
-      <c r="I836" s="19"/>
+      <c r="I836" s="20"/>
     </row>
     <row r="837" ht="15.75" customHeight="1">
       <c r="A837" s="3"/>
@@ -23852,9 +24233,9 @@
       <c r="D837" s="8"/>
       <c r="E837" s="5"/>
       <c r="F837" s="5"/>
-      <c r="G837" s="19"/>
+      <c r="G837" s="20"/>
       <c r="H837" s="12"/>
-      <c r="I837" s="19"/>
+      <c r="I837" s="20"/>
     </row>
     <row r="838" ht="15.75" customHeight="1">
       <c r="A838" s="3"/>
@@ -23863,9 +24244,9 @@
       <c r="D838" s="8"/>
       <c r="E838" s="5"/>
       <c r="F838" s="5"/>
-      <c r="G838" s="19"/>
+      <c r="G838" s="20"/>
       <c r="H838" s="12"/>
-      <c r="I838" s="19"/>
+      <c r="I838" s="20"/>
     </row>
     <row r="839" ht="15.75" customHeight="1">
       <c r="A839" s="3"/>
@@ -23874,9 +24255,9 @@
       <c r="D839" s="8"/>
       <c r="E839" s="5"/>
       <c r="F839" s="5"/>
-      <c r="G839" s="19"/>
+      <c r="G839" s="20"/>
       <c r="H839" s="12"/>
-      <c r="I839" s="19"/>
+      <c r="I839" s="20"/>
     </row>
     <row r="840" ht="15.75" customHeight="1">
       <c r="A840" s="3"/>
@@ -23885,9 +24266,9 @@
       <c r="D840" s="8"/>
       <c r="E840" s="5"/>
       <c r="F840" s="5"/>
-      <c r="G840" s="19"/>
+      <c r="G840" s="20"/>
       <c r="H840" s="12"/>
-      <c r="I840" s="19"/>
+      <c r="I840" s="20"/>
     </row>
     <row r="841" ht="15.75" customHeight="1">
       <c r="A841" s="3"/>
@@ -23896,9 +24277,9 @@
       <c r="D841" s="8"/>
       <c r="E841" s="5"/>
       <c r="F841" s="5"/>
-      <c r="G841" s="19"/>
+      <c r="G841" s="20"/>
       <c r="H841" s="12"/>
-      <c r="I841" s="19"/>
+      <c r="I841" s="20"/>
     </row>
     <row r="842" ht="15.75" customHeight="1">
       <c r="A842" s="3"/>
@@ -23907,9 +24288,9 @@
       <c r="D842" s="8"/>
       <c r="E842" s="5"/>
       <c r="F842" s="5"/>
-      <c r="G842" s="19"/>
+      <c r="G842" s="20"/>
       <c r="H842" s="12"/>
-      <c r="I842" s="19"/>
+      <c r="I842" s="20"/>
     </row>
     <row r="843" ht="15.75" customHeight="1">
       <c r="A843" s="3"/>
@@ -23918,9 +24299,9 @@
       <c r="D843" s="8"/>
       <c r="E843" s="5"/>
       <c r="F843" s="5"/>
-      <c r="G843" s="19"/>
+      <c r="G843" s="20"/>
       <c r="H843" s="12"/>
-      <c r="I843" s="19"/>
+      <c r="I843" s="20"/>
     </row>
     <row r="844" ht="15.75" customHeight="1">
       <c r="A844" s="3"/>
@@ -23929,9 +24310,9 @@
       <c r="D844" s="8"/>
       <c r="E844" s="5"/>
       <c r="F844" s="5"/>
-      <c r="G844" s="19"/>
+      <c r="G844" s="20"/>
       <c r="H844" s="12"/>
-      <c r="I844" s="19"/>
+      <c r="I844" s="20"/>
     </row>
     <row r="845" ht="15.75" customHeight="1">
       <c r="A845" s="3"/>
@@ -23940,9 +24321,9 @@
       <c r="D845" s="8"/>
       <c r="E845" s="5"/>
       <c r="F845" s="5"/>
-      <c r="G845" s="19"/>
+      <c r="G845" s="20"/>
       <c r="H845" s="12"/>
-      <c r="I845" s="19"/>
+      <c r="I845" s="20"/>
     </row>
     <row r="846" ht="15.75" customHeight="1">
       <c r="A846" s="3"/>
@@ -23951,9 +24332,9 @@
       <c r="D846" s="8"/>
       <c r="E846" s="5"/>
       <c r="F846" s="5"/>
-      <c r="G846" s="19"/>
+      <c r="G846" s="20"/>
       <c r="H846" s="12"/>
-      <c r="I846" s="19"/>
+      <c r="I846" s="20"/>
     </row>
     <row r="847" ht="15.75" customHeight="1">
       <c r="A847" s="3"/>
@@ -23962,9 +24343,9 @@
       <c r="D847" s="8"/>
       <c r="E847" s="5"/>
       <c r="F847" s="5"/>
-      <c r="G847" s="19"/>
+      <c r="G847" s="20"/>
       <c r="H847" s="12"/>
-      <c r="I847" s="19"/>
+      <c r="I847" s="20"/>
     </row>
     <row r="848" ht="15.75" customHeight="1">
       <c r="A848" s="3"/>
@@ -23973,9 +24354,9 @@
       <c r="D848" s="8"/>
       <c r="E848" s="5"/>
       <c r="F848" s="5"/>
-      <c r="G848" s="19"/>
+      <c r="G848" s="20"/>
       <c r="H848" s="12"/>
-      <c r="I848" s="19"/>
+      <c r="I848" s="20"/>
     </row>
     <row r="849" ht="15.75" customHeight="1">
       <c r="A849" s="3"/>
@@ -23984,9 +24365,9 @@
       <c r="D849" s="8"/>
       <c r="E849" s="5"/>
       <c r="F849" s="5"/>
-      <c r="G849" s="19"/>
+      <c r="G849" s="20"/>
       <c r="H849" s="12"/>
-      <c r="I849" s="19"/>
+      <c r="I849" s="20"/>
     </row>
     <row r="850" ht="15.75" customHeight="1">
       <c r="A850" s="3"/>
@@ -23995,9 +24376,9 @@
       <c r="D850" s="8"/>
       <c r="E850" s="5"/>
       <c r="F850" s="5"/>
-      <c r="G850" s="19"/>
+      <c r="G850" s="20"/>
       <c r="H850" s="12"/>
-      <c r="I850" s="19"/>
+      <c r="I850" s="20"/>
     </row>
     <row r="851" ht="15.75" customHeight="1">
       <c r="A851" s="3"/>
@@ -24006,9 +24387,9 @@
       <c r="D851" s="8"/>
       <c r="E851" s="5"/>
       <c r="F851" s="5"/>
-      <c r="G851" s="19"/>
+      <c r="G851" s="20"/>
       <c r="H851" s="12"/>
-      <c r="I851" s="19"/>
+      <c r="I851" s="20"/>
     </row>
     <row r="852" ht="15.75" customHeight="1">
       <c r="A852" s="3"/>
@@ -24017,9 +24398,9 @@
       <c r="D852" s="8"/>
       <c r="E852" s="5"/>
       <c r="F852" s="5"/>
-      <c r="G852" s="19"/>
+      <c r="G852" s="20"/>
       <c r="H852" s="12"/>
-      <c r="I852" s="19"/>
+      <c r="I852" s="20"/>
     </row>
     <row r="853" ht="15.75" customHeight="1">
       <c r="A853" s="3"/>
@@ -24028,9 +24409,9 @@
       <c r="D853" s="8"/>
       <c r="E853" s="5"/>
       <c r="F853" s="5"/>
-      <c r="G853" s="19"/>
+      <c r="G853" s="20"/>
       <c r="H853" s="12"/>
-      <c r="I853" s="19"/>
+      <c r="I853" s="20"/>
     </row>
     <row r="854" ht="15.75" customHeight="1">
       <c r="A854" s="3"/>
@@ -24039,9 +24420,9 @@
       <c r="D854" s="8"/>
       <c r="E854" s="5"/>
       <c r="F854" s="5"/>
-      <c r="G854" s="19"/>
+      <c r="G854" s="20"/>
       <c r="H854" s="12"/>
-      <c r="I854" s="19"/>
+      <c r="I854" s="20"/>
     </row>
     <row r="855" ht="15.75" customHeight="1">
       <c r="A855" s="3"/>
@@ -24050,9 +24431,9 @@
       <c r="D855" s="8"/>
       <c r="E855" s="5"/>
       <c r="F855" s="5"/>
-      <c r="G855" s="19"/>
+      <c r="G855" s="20"/>
       <c r="H855" s="12"/>
-      <c r="I855" s="19"/>
+      <c r="I855" s="20"/>
     </row>
     <row r="856" ht="15.75" customHeight="1">
       <c r="A856" s="3"/>
@@ -24061,9 +24442,9 @@
       <c r="D856" s="8"/>
       <c r="E856" s="5"/>
       <c r="F856" s="5"/>
-      <c r="G856" s="19"/>
+      <c r="G856" s="20"/>
       <c r="H856" s="12"/>
-      <c r="I856" s="19"/>
+      <c r="I856" s="20"/>
     </row>
     <row r="857" ht="15.75" customHeight="1">
       <c r="A857" s="3"/>
@@ -24072,9 +24453,9 @@
       <c r="D857" s="8"/>
       <c r="E857" s="5"/>
       <c r="F857" s="5"/>
-      <c r="G857" s="19"/>
+      <c r="G857" s="20"/>
       <c r="H857" s="12"/>
-      <c r="I857" s="19"/>
+      <c r="I857" s="20"/>
     </row>
     <row r="858" ht="15.75" customHeight="1">
       <c r="A858" s="3"/>
@@ -24083,9 +24464,9 @@
       <c r="D858" s="8"/>
       <c r="E858" s="5"/>
       <c r="F858" s="5"/>
-      <c r="G858" s="19"/>
+      <c r="G858" s="20"/>
       <c r="H858" s="12"/>
-      <c r="I858" s="19"/>
+      <c r="I858" s="20"/>
     </row>
     <row r="859" ht="15.75" customHeight="1">
       <c r="A859" s="3"/>
@@ -24094,9 +24475,9 @@
       <c r="D859" s="8"/>
       <c r="E859" s="5"/>
       <c r="F859" s="5"/>
-      <c r="G859" s="19"/>
+      <c r="G859" s="20"/>
       <c r="H859" s="12"/>
-      <c r="I859" s="19"/>
+      <c r="I859" s="20"/>
     </row>
     <row r="860" ht="15.75" customHeight="1">
       <c r="A860" s="3"/>
@@ -24105,9 +24486,9 @@
       <c r="D860" s="8"/>
       <c r="E860" s="5"/>
       <c r="F860" s="5"/>
-      <c r="G860" s="19"/>
+      <c r="G860" s="20"/>
       <c r="H860" s="12"/>
-      <c r="I860" s="19"/>
+      <c r="I860" s="20"/>
     </row>
     <row r="861" ht="15.75" customHeight="1">
       <c r="A861" s="3"/>
@@ -24116,9 +24497,9 @@
       <c r="D861" s="8"/>
       <c r="E861" s="5"/>
       <c r="F861" s="5"/>
-      <c r="G861" s="19"/>
+      <c r="G861" s="20"/>
       <c r="H861" s="12"/>
-      <c r="I861" s="19"/>
+      <c r="I861" s="20"/>
     </row>
     <row r="862" ht="15.75" customHeight="1">
       <c r="A862" s="3"/>
@@ -24127,9 +24508,9 @@
       <c r="D862" s="8"/>
       <c r="E862" s="5"/>
       <c r="F862" s="5"/>
-      <c r="G862" s="19"/>
+      <c r="G862" s="20"/>
       <c r="H862" s="12"/>
-      <c r="I862" s="19"/>
+      <c r="I862" s="20"/>
     </row>
     <row r="863" ht="15.75" customHeight="1">
       <c r="A863" s="3"/>
@@ -24138,9 +24519,9 @@
       <c r="D863" s="8"/>
       <c r="E863" s="5"/>
       <c r="F863" s="5"/>
-      <c r="G863" s="19"/>
+      <c r="G863" s="20"/>
       <c r="H863" s="12"/>
-      <c r="I863" s="19"/>
+      <c r="I863" s="20"/>
     </row>
     <row r="864" ht="15.75" customHeight="1">
       <c r="A864" s="3"/>
@@ -24149,9 +24530,9 @@
       <c r="D864" s="8"/>
       <c r="E864" s="5"/>
       <c r="F864" s="5"/>
-      <c r="G864" s="19"/>
+      <c r="G864" s="20"/>
       <c r="H864" s="12"/>
-      <c r="I864" s="19"/>
+      <c r="I864" s="20"/>
     </row>
     <row r="865" ht="15.75" customHeight="1">
       <c r="A865" s="3"/>
@@ -24160,9 +24541,9 @@
       <c r="D865" s="8"/>
       <c r="E865" s="5"/>
       <c r="F865" s="5"/>
-      <c r="G865" s="19"/>
+      <c r="G865" s="20"/>
       <c r="H865" s="12"/>
-      <c r="I865" s="19"/>
+      <c r="I865" s="20"/>
     </row>
     <row r="866" ht="15.75" customHeight="1">
       <c r="A866" s="3"/>
@@ -24171,9 +24552,9 @@
       <c r="D866" s="8"/>
       <c r="E866" s="5"/>
       <c r="F866" s="5"/>
-      <c r="G866" s="19"/>
+      <c r="G866" s="20"/>
       <c r="H866" s="12"/>
-      <c r="I866" s="19"/>
+      <c r="I866" s="20"/>
     </row>
     <row r="867" ht="15.75" customHeight="1">
       <c r="A867" s="3"/>
@@ -24182,9 +24563,9 @@
       <c r="D867" s="8"/>
       <c r="E867" s="5"/>
       <c r="F867" s="5"/>
-      <c r="G867" s="19"/>
+      <c r="G867" s="20"/>
       <c r="H867" s="12"/>
-      <c r="I867" s="19"/>
+      <c r="I867" s="20"/>
     </row>
     <row r="868" ht="15.75" customHeight="1">
       <c r="A868" s="3"/>
@@ -24193,9 +24574,9 @@
       <c r="D868" s="8"/>
       <c r="E868" s="5"/>
       <c r="F868" s="5"/>
-      <c r="G868" s="19"/>
+      <c r="G868" s="20"/>
       <c r="H868" s="12"/>
-      <c r="I868" s="19"/>
+      <c r="I868" s="20"/>
     </row>
     <row r="869" ht="15.75" customHeight="1">
       <c r="A869" s="3"/>
@@ -24204,9 +24585,9 @@
       <c r="D869" s="8"/>
       <c r="E869" s="5"/>
       <c r="F869" s="5"/>
-      <c r="G869" s="19"/>
+      <c r="G869" s="20"/>
       <c r="H869" s="12"/>
-      <c r="I869" s="19"/>
+      <c r="I869" s="20"/>
     </row>
     <row r="870" ht="15.75" customHeight="1">
       <c r="A870" s="3"/>
@@ -24215,9 +24596,9 @@
       <c r="D870" s="8"/>
       <c r="E870" s="5"/>
       <c r="F870" s="5"/>
-      <c r="G870" s="19"/>
+      <c r="G870" s="20"/>
       <c r="H870" s="12"/>
-      <c r="I870" s="19"/>
+      <c r="I870" s="20"/>
     </row>
     <row r="871" ht="15.75" customHeight="1">
       <c r="A871" s="3"/>
@@ -24226,9 +24607,9 @@
       <c r="D871" s="8"/>
       <c r="E871" s="5"/>
       <c r="F871" s="5"/>
-      <c r="G871" s="19"/>
+      <c r="G871" s="20"/>
       <c r="H871" s="12"/>
-      <c r="I871" s="19"/>
+      <c r="I871" s="20"/>
     </row>
     <row r="872" ht="15.75" customHeight="1">
       <c r="A872" s="3"/>
@@ -24237,1417 +24618,1417 @@
       <c r="D872" s="8"/>
       <c r="E872" s="5"/>
       <c r="F872" s="5"/>
-      <c r="G872" s="19"/>
+      <c r="G872" s="20"/>
       <c r="H872" s="12"/>
-      <c r="I872" s="19"/>
+      <c r="I872" s="20"/>
     </row>
     <row r="873" ht="15.75" customHeight="1">
-      <c r="A873" s="19"/>
-      <c r="B873" s="19"/>
-      <c r="C873" s="19"/>
-      <c r="D873" s="19"/>
-      <c r="E873" s="19"/>
-      <c r="F873" s="19"/>
-      <c r="G873" s="19"/>
-      <c r="H873" s="19"/>
-      <c r="I873" s="19"/>
+      <c r="A873" s="20"/>
+      <c r="B873" s="20"/>
+      <c r="C873" s="20"/>
+      <c r="D873" s="20"/>
+      <c r="E873" s="20"/>
+      <c r="F873" s="20"/>
+      <c r="G873" s="20"/>
+      <c r="H873" s="20"/>
+      <c r="I873" s="20"/>
     </row>
     <row r="874" ht="15.75" customHeight="1">
-      <c r="A874" s="19"/>
-      <c r="B874" s="19"/>
-      <c r="C874" s="19"/>
-      <c r="D874" s="19"/>
-      <c r="E874" s="19"/>
-      <c r="F874" s="19"/>
-      <c r="G874" s="19"/>
-      <c r="H874" s="19"/>
-      <c r="I874" s="19"/>
+      <c r="A874" s="20"/>
+      <c r="B874" s="20"/>
+      <c r="C874" s="20"/>
+      <c r="D874" s="20"/>
+      <c r="E874" s="20"/>
+      <c r="F874" s="20"/>
+      <c r="G874" s="20"/>
+      <c r="H874" s="20"/>
+      <c r="I874" s="20"/>
     </row>
     <row r="875" ht="15.75" customHeight="1">
-      <c r="A875" s="19"/>
-      <c r="B875" s="19"/>
-      <c r="C875" s="19"/>
-      <c r="D875" s="19"/>
-      <c r="E875" s="19"/>
-      <c r="F875" s="19"/>
-      <c r="G875" s="19"/>
-      <c r="H875" s="19"/>
-      <c r="I875" s="19"/>
+      <c r="A875" s="20"/>
+      <c r="B875" s="20"/>
+      <c r="C875" s="20"/>
+      <c r="D875" s="20"/>
+      <c r="E875" s="20"/>
+      <c r="F875" s="20"/>
+      <c r="G875" s="20"/>
+      <c r="H875" s="20"/>
+      <c r="I875" s="20"/>
     </row>
     <row r="876" ht="15.75" customHeight="1">
-      <c r="A876" s="19"/>
-      <c r="B876" s="19"/>
-      <c r="C876" s="19"/>
-      <c r="D876" s="19"/>
-      <c r="E876" s="19"/>
-      <c r="F876" s="19"/>
-      <c r="G876" s="19"/>
-      <c r="H876" s="19"/>
-      <c r="I876" s="19"/>
+      <c r="A876" s="20"/>
+      <c r="B876" s="20"/>
+      <c r="C876" s="20"/>
+      <c r="D876" s="20"/>
+      <c r="E876" s="20"/>
+      <c r="F876" s="20"/>
+      <c r="G876" s="20"/>
+      <c r="H876" s="20"/>
+      <c r="I876" s="20"/>
     </row>
     <row r="877" ht="15.75" customHeight="1">
-      <c r="A877" s="19"/>
-      <c r="B877" s="19"/>
-      <c r="C877" s="19"/>
-      <c r="D877" s="19"/>
-      <c r="E877" s="19"/>
-      <c r="F877" s="19"/>
-      <c r="G877" s="19"/>
-      <c r="H877" s="19"/>
-      <c r="I877" s="19"/>
+      <c r="A877" s="20"/>
+      <c r="B877" s="20"/>
+      <c r="C877" s="20"/>
+      <c r="D877" s="20"/>
+      <c r="E877" s="20"/>
+      <c r="F877" s="20"/>
+      <c r="G877" s="20"/>
+      <c r="H877" s="20"/>
+      <c r="I877" s="20"/>
     </row>
     <row r="878" ht="15.75" customHeight="1">
-      <c r="A878" s="19"/>
-      <c r="B878" s="19"/>
-      <c r="C878" s="19"/>
-      <c r="D878" s="19"/>
-      <c r="E878" s="19"/>
-      <c r="F878" s="19"/>
-      <c r="G878" s="19"/>
-      <c r="H878" s="19"/>
-      <c r="I878" s="19"/>
+      <c r="A878" s="20"/>
+      <c r="B878" s="20"/>
+      <c r="C878" s="20"/>
+      <c r="D878" s="20"/>
+      <c r="E878" s="20"/>
+      <c r="F878" s="20"/>
+      <c r="G878" s="20"/>
+      <c r="H878" s="20"/>
+      <c r="I878" s="20"/>
     </row>
     <row r="879" ht="15.75" customHeight="1">
-      <c r="A879" s="19"/>
-      <c r="B879" s="19"/>
-      <c r="C879" s="19"/>
-      <c r="D879" s="19"/>
-      <c r="E879" s="19"/>
-      <c r="F879" s="19"/>
-      <c r="G879" s="19"/>
-      <c r="H879" s="19"/>
-      <c r="I879" s="19"/>
+      <c r="A879" s="20"/>
+      <c r="B879" s="20"/>
+      <c r="C879" s="20"/>
+      <c r="D879" s="20"/>
+      <c r="E879" s="20"/>
+      <c r="F879" s="20"/>
+      <c r="G879" s="20"/>
+      <c r="H879" s="20"/>
+      <c r="I879" s="20"/>
     </row>
     <row r="880" ht="15.75" customHeight="1">
-      <c r="A880" s="19"/>
-      <c r="B880" s="19"/>
-      <c r="C880" s="19"/>
-      <c r="D880" s="19"/>
-      <c r="E880" s="19"/>
-      <c r="F880" s="19"/>
-      <c r="G880" s="19"/>
-      <c r="H880" s="19"/>
-      <c r="I880" s="19"/>
+      <c r="A880" s="20"/>
+      <c r="B880" s="20"/>
+      <c r="C880" s="20"/>
+      <c r="D880" s="20"/>
+      <c r="E880" s="20"/>
+      <c r="F880" s="20"/>
+      <c r="G880" s="20"/>
+      <c r="H880" s="20"/>
+      <c r="I880" s="20"/>
     </row>
     <row r="881" ht="15.75" customHeight="1">
-      <c r="A881" s="19"/>
-      <c r="B881" s="19"/>
-      <c r="C881" s="19"/>
-      <c r="D881" s="19"/>
-      <c r="E881" s="19"/>
-      <c r="F881" s="19"/>
-      <c r="G881" s="19"/>
-      <c r="H881" s="19"/>
-      <c r="I881" s="19"/>
+      <c r="A881" s="20"/>
+      <c r="B881" s="20"/>
+      <c r="C881" s="20"/>
+      <c r="D881" s="20"/>
+      <c r="E881" s="20"/>
+      <c r="F881" s="20"/>
+      <c r="G881" s="20"/>
+      <c r="H881" s="20"/>
+      <c r="I881" s="20"/>
     </row>
     <row r="882" ht="15.75" customHeight="1">
-      <c r="A882" s="19"/>
-      <c r="B882" s="19"/>
-      <c r="C882" s="19"/>
-      <c r="D882" s="19"/>
-      <c r="E882" s="19"/>
-      <c r="F882" s="19"/>
-      <c r="G882" s="19"/>
-      <c r="H882" s="19"/>
-      <c r="I882" s="19"/>
+      <c r="A882" s="20"/>
+      <c r="B882" s="20"/>
+      <c r="C882" s="20"/>
+      <c r="D882" s="20"/>
+      <c r="E882" s="20"/>
+      <c r="F882" s="20"/>
+      <c r="G882" s="20"/>
+      <c r="H882" s="20"/>
+      <c r="I882" s="20"/>
     </row>
     <row r="883" ht="15.75" customHeight="1">
-      <c r="A883" s="19"/>
-      <c r="B883" s="19"/>
-      <c r="C883" s="19"/>
-      <c r="D883" s="19"/>
-      <c r="E883" s="19"/>
-      <c r="F883" s="19"/>
-      <c r="G883" s="19"/>
-      <c r="H883" s="19"/>
-      <c r="I883" s="19"/>
+      <c r="A883" s="20"/>
+      <c r="B883" s="20"/>
+      <c r="C883" s="20"/>
+      <c r="D883" s="20"/>
+      <c r="E883" s="20"/>
+      <c r="F883" s="20"/>
+      <c r="G883" s="20"/>
+      <c r="H883" s="20"/>
+      <c r="I883" s="20"/>
     </row>
     <row r="884" ht="15.75" customHeight="1">
-      <c r="A884" s="19"/>
-      <c r="B884" s="19"/>
-      <c r="C884" s="19"/>
-      <c r="D884" s="19"/>
-      <c r="E884" s="19"/>
-      <c r="F884" s="19"/>
-      <c r="G884" s="19"/>
-      <c r="H884" s="19"/>
-      <c r="I884" s="19"/>
+      <c r="A884" s="20"/>
+      <c r="B884" s="20"/>
+      <c r="C884" s="20"/>
+      <c r="D884" s="20"/>
+      <c r="E884" s="20"/>
+      <c r="F884" s="20"/>
+      <c r="G884" s="20"/>
+      <c r="H884" s="20"/>
+      <c r="I884" s="20"/>
     </row>
     <row r="885" ht="15.75" customHeight="1">
-      <c r="A885" s="19"/>
-      <c r="B885" s="19"/>
-      <c r="C885" s="19"/>
-      <c r="D885" s="19"/>
-      <c r="E885" s="19"/>
-      <c r="F885" s="19"/>
-      <c r="G885" s="19"/>
-      <c r="H885" s="19"/>
-      <c r="I885" s="19"/>
+      <c r="A885" s="20"/>
+      <c r="B885" s="20"/>
+      <c r="C885" s="20"/>
+      <c r="D885" s="20"/>
+      <c r="E885" s="20"/>
+      <c r="F885" s="20"/>
+      <c r="G885" s="20"/>
+      <c r="H885" s="20"/>
+      <c r="I885" s="20"/>
     </row>
     <row r="886" ht="15.75" customHeight="1">
-      <c r="A886" s="19"/>
-      <c r="B886" s="19"/>
-      <c r="C886" s="19"/>
-      <c r="D886" s="19"/>
-      <c r="E886" s="19"/>
-      <c r="F886" s="19"/>
-      <c r="G886" s="19"/>
-      <c r="H886" s="19"/>
-      <c r="I886" s="19"/>
+      <c r="A886" s="20"/>
+      <c r="B886" s="20"/>
+      <c r="C886" s="20"/>
+      <c r="D886" s="20"/>
+      <c r="E886" s="20"/>
+      <c r="F886" s="20"/>
+      <c r="G886" s="20"/>
+      <c r="H886" s="20"/>
+      <c r="I886" s="20"/>
     </row>
     <row r="887" ht="15.75" customHeight="1">
-      <c r="A887" s="19"/>
-      <c r="B887" s="19"/>
-      <c r="C887" s="19"/>
-      <c r="D887" s="19"/>
-      <c r="E887" s="19"/>
-      <c r="F887" s="19"/>
-      <c r="G887" s="19"/>
-      <c r="H887" s="19"/>
-      <c r="I887" s="19"/>
+      <c r="A887" s="20"/>
+      <c r="B887" s="20"/>
+      <c r="C887" s="20"/>
+      <c r="D887" s="20"/>
+      <c r="E887" s="20"/>
+      <c r="F887" s="20"/>
+      <c r="G887" s="20"/>
+      <c r="H887" s="20"/>
+      <c r="I887" s="20"/>
     </row>
     <row r="888" ht="15.75" customHeight="1">
-      <c r="A888" s="19"/>
-      <c r="B888" s="19"/>
-      <c r="C888" s="19"/>
-      <c r="D888" s="19"/>
-      <c r="E888" s="19"/>
-      <c r="F888" s="19"/>
-      <c r="G888" s="19"/>
-      <c r="H888" s="19"/>
-      <c r="I888" s="19"/>
+      <c r="A888" s="20"/>
+      <c r="B888" s="20"/>
+      <c r="C888" s="20"/>
+      <c r="D888" s="20"/>
+      <c r="E888" s="20"/>
+      <c r="F888" s="20"/>
+      <c r="G888" s="20"/>
+      <c r="H888" s="20"/>
+      <c r="I888" s="20"/>
     </row>
     <row r="889" ht="15.75" customHeight="1">
-      <c r="A889" s="19"/>
-      <c r="B889" s="19"/>
-      <c r="C889" s="19"/>
-      <c r="D889" s="19"/>
-      <c r="E889" s="19"/>
-      <c r="F889" s="19"/>
-      <c r="G889" s="19"/>
-      <c r="H889" s="19"/>
-      <c r="I889" s="19"/>
+      <c r="A889" s="20"/>
+      <c r="B889" s="20"/>
+      <c r="C889" s="20"/>
+      <c r="D889" s="20"/>
+      <c r="E889" s="20"/>
+      <c r="F889" s="20"/>
+      <c r="G889" s="20"/>
+      <c r="H889" s="20"/>
+      <c r="I889" s="20"/>
     </row>
     <row r="890" ht="15.75" customHeight="1">
-      <c r="A890" s="19"/>
-      <c r="B890" s="19"/>
-      <c r="C890" s="19"/>
-      <c r="D890" s="19"/>
-      <c r="E890" s="19"/>
-      <c r="F890" s="19"/>
-      <c r="G890" s="19"/>
-      <c r="H890" s="19"/>
-      <c r="I890" s="19"/>
+      <c r="A890" s="20"/>
+      <c r="B890" s="20"/>
+      <c r="C890" s="20"/>
+      <c r="D890" s="20"/>
+      <c r="E890" s="20"/>
+      <c r="F890" s="20"/>
+      <c r="G890" s="20"/>
+      <c r="H890" s="20"/>
+      <c r="I890" s="20"/>
     </row>
     <row r="891" ht="15.75" customHeight="1">
-      <c r="A891" s="19"/>
-      <c r="B891" s="19"/>
-      <c r="C891" s="19"/>
-      <c r="D891" s="19"/>
-      <c r="E891" s="19"/>
-      <c r="F891" s="19"/>
-      <c r="G891" s="19"/>
-      <c r="H891" s="19"/>
-      <c r="I891" s="19"/>
+      <c r="A891" s="20"/>
+      <c r="B891" s="20"/>
+      <c r="C891" s="20"/>
+      <c r="D891" s="20"/>
+      <c r="E891" s="20"/>
+      <c r="F891" s="20"/>
+      <c r="G891" s="20"/>
+      <c r="H891" s="20"/>
+      <c r="I891" s="20"/>
     </row>
     <row r="892" ht="15.75" customHeight="1">
-      <c r="A892" s="19"/>
-      <c r="B892" s="19"/>
-      <c r="C892" s="19"/>
-      <c r="D892" s="19"/>
-      <c r="E892" s="19"/>
-      <c r="F892" s="19"/>
-      <c r="G892" s="19"/>
-      <c r="H892" s="19"/>
-      <c r="I892" s="19"/>
+      <c r="A892" s="20"/>
+      <c r="B892" s="20"/>
+      <c r="C892" s="20"/>
+      <c r="D892" s="20"/>
+      <c r="E892" s="20"/>
+      <c r="F892" s="20"/>
+      <c r="G892" s="20"/>
+      <c r="H892" s="20"/>
+      <c r="I892" s="20"/>
     </row>
     <row r="893" ht="15.75" customHeight="1">
-      <c r="A893" s="19"/>
-      <c r="B893" s="19"/>
-      <c r="C893" s="19"/>
-      <c r="D893" s="19"/>
-      <c r="E893" s="19"/>
-      <c r="F893" s="19"/>
-      <c r="G893" s="19"/>
-      <c r="H893" s="19"/>
-      <c r="I893" s="19"/>
+      <c r="A893" s="20"/>
+      <c r="B893" s="20"/>
+      <c r="C893" s="20"/>
+      <c r="D893" s="20"/>
+      <c r="E893" s="20"/>
+      <c r="F893" s="20"/>
+      <c r="G893" s="20"/>
+      <c r="H893" s="20"/>
+      <c r="I893" s="20"/>
     </row>
     <row r="894" ht="15.75" customHeight="1">
-      <c r="A894" s="19"/>
-      <c r="B894" s="19"/>
-      <c r="C894" s="19"/>
-      <c r="D894" s="19"/>
-      <c r="E894" s="19"/>
-      <c r="F894" s="19"/>
-      <c r="G894" s="19"/>
-      <c r="H894" s="19"/>
-      <c r="I894" s="19"/>
+      <c r="A894" s="20"/>
+      <c r="B894" s="20"/>
+      <c r="C894" s="20"/>
+      <c r="D894" s="20"/>
+      <c r="E894" s="20"/>
+      <c r="F894" s="20"/>
+      <c r="G894" s="20"/>
+      <c r="H894" s="20"/>
+      <c r="I894" s="20"/>
     </row>
     <row r="895" ht="15.75" customHeight="1">
-      <c r="A895" s="19"/>
-      <c r="B895" s="19"/>
-      <c r="C895" s="19"/>
-      <c r="D895" s="19"/>
-      <c r="E895" s="19"/>
-      <c r="F895" s="19"/>
-      <c r="G895" s="19"/>
-      <c r="H895" s="19"/>
-      <c r="I895" s="19"/>
+      <c r="A895" s="20"/>
+      <c r="B895" s="20"/>
+      <c r="C895" s="20"/>
+      <c r="D895" s="20"/>
+      <c r="E895" s="20"/>
+      <c r="F895" s="20"/>
+      <c r="G895" s="20"/>
+      <c r="H895" s="20"/>
+      <c r="I895" s="20"/>
     </row>
     <row r="896" ht="15.75" customHeight="1">
-      <c r="A896" s="19"/>
-      <c r="B896" s="19"/>
-      <c r="C896" s="19"/>
-      <c r="D896" s="19"/>
-      <c r="E896" s="19"/>
-      <c r="F896" s="19"/>
-      <c r="G896" s="19"/>
-      <c r="H896" s="19"/>
-      <c r="I896" s="19"/>
+      <c r="A896" s="20"/>
+      <c r="B896" s="20"/>
+      <c r="C896" s="20"/>
+      <c r="D896" s="20"/>
+      <c r="E896" s="20"/>
+      <c r="F896" s="20"/>
+      <c r="G896" s="20"/>
+      <c r="H896" s="20"/>
+      <c r="I896" s="20"/>
     </row>
     <row r="897" ht="15.75" customHeight="1">
-      <c r="A897" s="19"/>
-      <c r="B897" s="19"/>
-      <c r="C897" s="19"/>
-      <c r="D897" s="19"/>
-      <c r="E897" s="19"/>
-      <c r="F897" s="19"/>
-      <c r="G897" s="19"/>
-      <c r="H897" s="19"/>
-      <c r="I897" s="19"/>
+      <c r="A897" s="20"/>
+      <c r="B897" s="20"/>
+      <c r="C897" s="20"/>
+      <c r="D897" s="20"/>
+      <c r="E897" s="20"/>
+      <c r="F897" s="20"/>
+      <c r="G897" s="20"/>
+      <c r="H897" s="20"/>
+      <c r="I897" s="20"/>
     </row>
     <row r="898" ht="15.75" customHeight="1">
-      <c r="A898" s="19"/>
-      <c r="B898" s="19"/>
-      <c r="C898" s="19"/>
-      <c r="D898" s="19"/>
-      <c r="E898" s="19"/>
-      <c r="F898" s="19"/>
-      <c r="G898" s="19"/>
-      <c r="H898" s="19"/>
-      <c r="I898" s="19"/>
+      <c r="A898" s="20"/>
+      <c r="B898" s="20"/>
+      <c r="C898" s="20"/>
+      <c r="D898" s="20"/>
+      <c r="E898" s="20"/>
+      <c r="F898" s="20"/>
+      <c r="G898" s="20"/>
+      <c r="H898" s="20"/>
+      <c r="I898" s="20"/>
     </row>
     <row r="899" ht="15.75" customHeight="1">
-      <c r="A899" s="19"/>
-      <c r="B899" s="19"/>
-      <c r="C899" s="19"/>
-      <c r="D899" s="19"/>
-      <c r="E899" s="19"/>
-      <c r="F899" s="19"/>
-      <c r="G899" s="19"/>
-      <c r="H899" s="19"/>
-      <c r="I899" s="19"/>
+      <c r="A899" s="20"/>
+      <c r="B899" s="20"/>
+      <c r="C899" s="20"/>
+      <c r="D899" s="20"/>
+      <c r="E899" s="20"/>
+      <c r="F899" s="20"/>
+      <c r="G899" s="20"/>
+      <c r="H899" s="20"/>
+      <c r="I899" s="20"/>
     </row>
     <row r="900" ht="15.75" customHeight="1">
-      <c r="A900" s="19"/>
-      <c r="B900" s="19"/>
-      <c r="C900" s="19"/>
-      <c r="D900" s="19"/>
-      <c r="E900" s="19"/>
-      <c r="F900" s="19"/>
-      <c r="G900" s="19"/>
-      <c r="H900" s="19"/>
-      <c r="I900" s="19"/>
+      <c r="A900" s="20"/>
+      <c r="B900" s="20"/>
+      <c r="C900" s="20"/>
+      <c r="D900" s="20"/>
+      <c r="E900" s="20"/>
+      <c r="F900" s="20"/>
+      <c r="G900" s="20"/>
+      <c r="H900" s="20"/>
+      <c r="I900" s="20"/>
     </row>
     <row r="901" ht="15.75" customHeight="1">
-      <c r="A901" s="19"/>
-      <c r="B901" s="19"/>
-      <c r="C901" s="19"/>
-      <c r="D901" s="19"/>
-      <c r="E901" s="19"/>
-      <c r="F901" s="19"/>
-      <c r="G901" s="19"/>
-      <c r="H901" s="19"/>
-      <c r="I901" s="19"/>
+      <c r="A901" s="20"/>
+      <c r="B901" s="20"/>
+      <c r="C901" s="20"/>
+      <c r="D901" s="20"/>
+      <c r="E901" s="20"/>
+      <c r="F901" s="20"/>
+      <c r="G901" s="20"/>
+      <c r="H901" s="20"/>
+      <c r="I901" s="20"/>
     </row>
     <row r="902" ht="15.75" customHeight="1">
-      <c r="A902" s="19"/>
-      <c r="B902" s="19"/>
-      <c r="C902" s="19"/>
-      <c r="D902" s="19"/>
-      <c r="E902" s="19"/>
-      <c r="F902" s="19"/>
-      <c r="G902" s="19"/>
-      <c r="H902" s="19"/>
-      <c r="I902" s="19"/>
+      <c r="A902" s="20"/>
+      <c r="B902" s="20"/>
+      <c r="C902" s="20"/>
+      <c r="D902" s="20"/>
+      <c r="E902" s="20"/>
+      <c r="F902" s="20"/>
+      <c r="G902" s="20"/>
+      <c r="H902" s="20"/>
+      <c r="I902" s="20"/>
     </row>
     <row r="903" ht="15.75" customHeight="1">
-      <c r="A903" s="19"/>
-      <c r="B903" s="19"/>
-      <c r="C903" s="19"/>
-      <c r="D903" s="19"/>
-      <c r="E903" s="19"/>
-      <c r="F903" s="19"/>
-      <c r="G903" s="19"/>
-      <c r="H903" s="19"/>
-      <c r="I903" s="19"/>
+      <c r="A903" s="20"/>
+      <c r="B903" s="20"/>
+      <c r="C903" s="20"/>
+      <c r="D903" s="20"/>
+      <c r="E903" s="20"/>
+      <c r="F903" s="20"/>
+      <c r="G903" s="20"/>
+      <c r="H903" s="20"/>
+      <c r="I903" s="20"/>
     </row>
     <row r="904" ht="15.75" customHeight="1">
-      <c r="A904" s="19"/>
-      <c r="B904" s="19"/>
-      <c r="C904" s="19"/>
-      <c r="D904" s="19"/>
-      <c r="E904" s="19"/>
-      <c r="F904" s="19"/>
-      <c r="G904" s="19"/>
-      <c r="H904" s="19"/>
-      <c r="I904" s="19"/>
+      <c r="A904" s="20"/>
+      <c r="B904" s="20"/>
+      <c r="C904" s="20"/>
+      <c r="D904" s="20"/>
+      <c r="E904" s="20"/>
+      <c r="F904" s="20"/>
+      <c r="G904" s="20"/>
+      <c r="H904" s="20"/>
+      <c r="I904" s="20"/>
     </row>
     <row r="905" ht="15.75" customHeight="1">
-      <c r="A905" s="19"/>
-      <c r="B905" s="19"/>
-      <c r="C905" s="19"/>
-      <c r="D905" s="19"/>
-      <c r="E905" s="19"/>
-      <c r="F905" s="19"/>
-      <c r="G905" s="19"/>
-      <c r="H905" s="19"/>
-      <c r="I905" s="19"/>
+      <c r="A905" s="20"/>
+      <c r="B905" s="20"/>
+      <c r="C905" s="20"/>
+      <c r="D905" s="20"/>
+      <c r="E905" s="20"/>
+      <c r="F905" s="20"/>
+      <c r="G905" s="20"/>
+      <c r="H905" s="20"/>
+      <c r="I905" s="20"/>
     </row>
     <row r="906" ht="15.75" customHeight="1">
-      <c r="A906" s="19"/>
-      <c r="B906" s="19"/>
-      <c r="C906" s="19"/>
-      <c r="D906" s="19"/>
-      <c r="E906" s="19"/>
-      <c r="F906" s="19"/>
-      <c r="G906" s="19"/>
-      <c r="H906" s="19"/>
-      <c r="I906" s="19"/>
+      <c r="A906" s="20"/>
+      <c r="B906" s="20"/>
+      <c r="C906" s="20"/>
+      <c r="D906" s="20"/>
+      <c r="E906" s="20"/>
+      <c r="F906" s="20"/>
+      <c r="G906" s="20"/>
+      <c r="H906" s="20"/>
+      <c r="I906" s="20"/>
     </row>
     <row r="907" ht="15.75" customHeight="1">
-      <c r="A907" s="19"/>
-      <c r="B907" s="19"/>
-      <c r="C907" s="19"/>
-      <c r="D907" s="19"/>
-      <c r="E907" s="19"/>
-      <c r="F907" s="19"/>
-      <c r="G907" s="19"/>
-      <c r="H907" s="19"/>
-      <c r="I907" s="19"/>
+      <c r="A907" s="20"/>
+      <c r="B907" s="20"/>
+      <c r="C907" s="20"/>
+      <c r="D907" s="20"/>
+      <c r="E907" s="20"/>
+      <c r="F907" s="20"/>
+      <c r="G907" s="20"/>
+      <c r="H907" s="20"/>
+      <c r="I907" s="20"/>
     </row>
     <row r="908" ht="15.75" customHeight="1">
-      <c r="A908" s="19"/>
-      <c r="B908" s="19"/>
-      <c r="C908" s="19"/>
-      <c r="D908" s="19"/>
-      <c r="E908" s="19"/>
-      <c r="F908" s="19"/>
-      <c r="G908" s="19"/>
-      <c r="H908" s="19"/>
-      <c r="I908" s="19"/>
+      <c r="A908" s="20"/>
+      <c r="B908" s="20"/>
+      <c r="C908" s="20"/>
+      <c r="D908" s="20"/>
+      <c r="E908" s="20"/>
+      <c r="F908" s="20"/>
+      <c r="G908" s="20"/>
+      <c r="H908" s="20"/>
+      <c r="I908" s="20"/>
     </row>
     <row r="909" ht="15.75" customHeight="1">
-      <c r="A909" s="19"/>
-      <c r="B909" s="19"/>
-      <c r="C909" s="19"/>
-      <c r="D909" s="19"/>
-      <c r="E909" s="19"/>
-      <c r="F909" s="19"/>
-      <c r="G909" s="19"/>
-      <c r="H909" s="19"/>
-      <c r="I909" s="19"/>
+      <c r="A909" s="20"/>
+      <c r="B909" s="20"/>
+      <c r="C909" s="20"/>
+      <c r="D909" s="20"/>
+      <c r="E909" s="20"/>
+      <c r="F909" s="20"/>
+      <c r="G909" s="20"/>
+      <c r="H909" s="20"/>
+      <c r="I909" s="20"/>
     </row>
     <row r="910" ht="15.75" customHeight="1">
-      <c r="A910" s="19"/>
-      <c r="B910" s="19"/>
-      <c r="C910" s="19"/>
-      <c r="D910" s="19"/>
-      <c r="E910" s="19"/>
-      <c r="F910" s="19"/>
-      <c r="G910" s="19"/>
-      <c r="H910" s="19"/>
-      <c r="I910" s="19"/>
+      <c r="A910" s="20"/>
+      <c r="B910" s="20"/>
+      <c r="C910" s="20"/>
+      <c r="D910" s="20"/>
+      <c r="E910" s="20"/>
+      <c r="F910" s="20"/>
+      <c r="G910" s="20"/>
+      <c r="H910" s="20"/>
+      <c r="I910" s="20"/>
     </row>
     <row r="911" ht="15.75" customHeight="1">
-      <c r="A911" s="19"/>
-      <c r="B911" s="19"/>
-      <c r="C911" s="19"/>
-      <c r="D911" s="19"/>
-      <c r="E911" s="19"/>
-      <c r="F911" s="19"/>
-      <c r="G911" s="19"/>
-      <c r="H911" s="19"/>
-      <c r="I911" s="19"/>
+      <c r="A911" s="20"/>
+      <c r="B911" s="20"/>
+      <c r="C911" s="20"/>
+      <c r="D911" s="20"/>
+      <c r="E911" s="20"/>
+      <c r="F911" s="20"/>
+      <c r="G911" s="20"/>
+      <c r="H911" s="20"/>
+      <c r="I911" s="20"/>
     </row>
     <row r="912" ht="15.75" customHeight="1">
-      <c r="A912" s="19"/>
-      <c r="B912" s="19"/>
-      <c r="C912" s="19"/>
-      <c r="D912" s="19"/>
-      <c r="E912" s="19"/>
-      <c r="F912" s="19"/>
-      <c r="G912" s="19"/>
-      <c r="H912" s="19"/>
-      <c r="I912" s="19"/>
+      <c r="A912" s="20"/>
+      <c r="B912" s="20"/>
+      <c r="C912" s="20"/>
+      <c r="D912" s="20"/>
+      <c r="E912" s="20"/>
+      <c r="F912" s="20"/>
+      <c r="G912" s="20"/>
+      <c r="H912" s="20"/>
+      <c r="I912" s="20"/>
     </row>
     <row r="913" ht="15.75" customHeight="1">
-      <c r="A913" s="19"/>
-      <c r="B913" s="19"/>
-      <c r="C913" s="19"/>
-      <c r="D913" s="19"/>
-      <c r="E913" s="19"/>
-      <c r="F913" s="19"/>
-      <c r="G913" s="19"/>
-      <c r="H913" s="19"/>
-      <c r="I913" s="19"/>
+      <c r="A913" s="20"/>
+      <c r="B913" s="20"/>
+      <c r="C913" s="20"/>
+      <c r="D913" s="20"/>
+      <c r="E913" s="20"/>
+      <c r="F913" s="20"/>
+      <c r="G913" s="20"/>
+      <c r="H913" s="20"/>
+      <c r="I913" s="20"/>
     </row>
     <row r="914" ht="15.75" customHeight="1">
-      <c r="A914" s="19"/>
-      <c r="B914" s="19"/>
-      <c r="C914" s="19"/>
-      <c r="D914" s="19"/>
-      <c r="E914" s="19"/>
-      <c r="F914" s="19"/>
-      <c r="G914" s="19"/>
-      <c r="H914" s="19"/>
-      <c r="I914" s="19"/>
+      <c r="A914" s="20"/>
+      <c r="B914" s="20"/>
+      <c r="C914" s="20"/>
+      <c r="D914" s="20"/>
+      <c r="E914" s="20"/>
+      <c r="F914" s="20"/>
+      <c r="G914" s="20"/>
+      <c r="H914" s="20"/>
+      <c r="I914" s="20"/>
     </row>
     <row r="915" ht="15.75" customHeight="1">
-      <c r="A915" s="19"/>
-      <c r="B915" s="19"/>
-      <c r="C915" s="19"/>
-      <c r="D915" s="19"/>
-      <c r="E915" s="19"/>
-      <c r="F915" s="19"/>
-      <c r="G915" s="19"/>
-      <c r="H915" s="19"/>
-      <c r="I915" s="19"/>
+      <c r="A915" s="20"/>
+      <c r="B915" s="20"/>
+      <c r="C915" s="20"/>
+      <c r="D915" s="20"/>
+      <c r="E915" s="20"/>
+      <c r="F915" s="20"/>
+      <c r="G915" s="20"/>
+      <c r="H915" s="20"/>
+      <c r="I915" s="20"/>
     </row>
     <row r="916" ht="15.75" customHeight="1">
-      <c r="A916" s="19"/>
-      <c r="B916" s="19"/>
-      <c r="C916" s="19"/>
-      <c r="D916" s="19"/>
-      <c r="E916" s="19"/>
-      <c r="F916" s="19"/>
-      <c r="G916" s="19"/>
-      <c r="H916" s="19"/>
-      <c r="I916" s="19"/>
+      <c r="A916" s="20"/>
+      <c r="B916" s="20"/>
+      <c r="C916" s="20"/>
+      <c r="D916" s="20"/>
+      <c r="E916" s="20"/>
+      <c r="F916" s="20"/>
+      <c r="G916" s="20"/>
+      <c r="H916" s="20"/>
+      <c r="I916" s="20"/>
     </row>
     <row r="917" ht="15.75" customHeight="1">
-      <c r="A917" s="19"/>
-      <c r="B917" s="19"/>
-      <c r="C917" s="19"/>
-      <c r="D917" s="19"/>
-      <c r="E917" s="19"/>
-      <c r="F917" s="19"/>
-      <c r="G917" s="19"/>
-      <c r="H917" s="19"/>
-      <c r="I917" s="19"/>
+      <c r="A917" s="20"/>
+      <c r="B917" s="20"/>
+      <c r="C917" s="20"/>
+      <c r="D917" s="20"/>
+      <c r="E917" s="20"/>
+      <c r="F917" s="20"/>
+      <c r="G917" s="20"/>
+      <c r="H917" s="20"/>
+      <c r="I917" s="20"/>
     </row>
     <row r="918" ht="15.75" customHeight="1">
-      <c r="A918" s="19"/>
-      <c r="B918" s="19"/>
-      <c r="C918" s="19"/>
-      <c r="D918" s="19"/>
-      <c r="E918" s="19"/>
-      <c r="F918" s="19"/>
-      <c r="G918" s="19"/>
-      <c r="H918" s="19"/>
-      <c r="I918" s="19"/>
+      <c r="A918" s="20"/>
+      <c r="B918" s="20"/>
+      <c r="C918" s="20"/>
+      <c r="D918" s="20"/>
+      <c r="E918" s="20"/>
+      <c r="F918" s="20"/>
+      <c r="G918" s="20"/>
+      <c r="H918" s="20"/>
+      <c r="I918" s="20"/>
     </row>
     <row r="919" ht="15.75" customHeight="1">
-      <c r="A919" s="19"/>
-      <c r="B919" s="19"/>
-      <c r="C919" s="19"/>
-      <c r="D919" s="19"/>
-      <c r="E919" s="19"/>
-      <c r="F919" s="19"/>
-      <c r="G919" s="19"/>
-      <c r="H919" s="19"/>
-      <c r="I919" s="19"/>
+      <c r="A919" s="20"/>
+      <c r="B919" s="20"/>
+      <c r="C919" s="20"/>
+      <c r="D919" s="20"/>
+      <c r="E919" s="20"/>
+      <c r="F919" s="20"/>
+      <c r="G919" s="20"/>
+      <c r="H919" s="20"/>
+      <c r="I919" s="20"/>
     </row>
     <row r="920" ht="15.75" customHeight="1">
-      <c r="A920" s="19"/>
-      <c r="B920" s="19"/>
-      <c r="C920" s="19"/>
-      <c r="D920" s="19"/>
-      <c r="E920" s="19"/>
-      <c r="F920" s="19"/>
-      <c r="G920" s="19"/>
-      <c r="H920" s="19"/>
-      <c r="I920" s="19"/>
+      <c r="A920" s="20"/>
+      <c r="B920" s="20"/>
+      <c r="C920" s="20"/>
+      <c r="D920" s="20"/>
+      <c r="E920" s="20"/>
+      <c r="F920" s="20"/>
+      <c r="G920" s="20"/>
+      <c r="H920" s="20"/>
+      <c r="I920" s="20"/>
     </row>
     <row r="921" ht="15.75" customHeight="1">
-      <c r="A921" s="19"/>
-      <c r="B921" s="19"/>
-      <c r="C921" s="19"/>
-      <c r="D921" s="19"/>
-      <c r="E921" s="19"/>
-      <c r="F921" s="19"/>
-      <c r="G921" s="19"/>
-      <c r="H921" s="19"/>
-      <c r="I921" s="19"/>
+      <c r="A921" s="20"/>
+      <c r="B921" s="20"/>
+      <c r="C921" s="20"/>
+      <c r="D921" s="20"/>
+      <c r="E921" s="20"/>
+      <c r="F921" s="20"/>
+      <c r="G921" s="20"/>
+      <c r="H921" s="20"/>
+      <c r="I921" s="20"/>
     </row>
     <row r="922" ht="15.75" customHeight="1">
-      <c r="A922" s="19"/>
-      <c r="B922" s="19"/>
-      <c r="C922" s="19"/>
-      <c r="D922" s="19"/>
-      <c r="E922" s="19"/>
-      <c r="F922" s="19"/>
-      <c r="G922" s="19"/>
-      <c r="H922" s="19"/>
-      <c r="I922" s="19"/>
+      <c r="A922" s="20"/>
+      <c r="B922" s="20"/>
+      <c r="C922" s="20"/>
+      <c r="D922" s="20"/>
+      <c r="E922" s="20"/>
+      <c r="F922" s="20"/>
+      <c r="G922" s="20"/>
+      <c r="H922" s="20"/>
+      <c r="I922" s="20"/>
     </row>
     <row r="923" ht="15.75" customHeight="1">
-      <c r="A923" s="19"/>
-      <c r="B923" s="19"/>
-      <c r="C923" s="19"/>
-      <c r="D923" s="19"/>
-      <c r="E923" s="19"/>
-      <c r="F923" s="19"/>
-      <c r="G923" s="19"/>
-      <c r="H923" s="19"/>
-      <c r="I923" s="19"/>
+      <c r="A923" s="20"/>
+      <c r="B923" s="20"/>
+      <c r="C923" s="20"/>
+      <c r="D923" s="20"/>
+      <c r="E923" s="20"/>
+      <c r="F923" s="20"/>
+      <c r="G923" s="20"/>
+      <c r="H923" s="20"/>
+      <c r="I923" s="20"/>
     </row>
     <row r="924" ht="15.75" customHeight="1">
-      <c r="A924" s="19"/>
-      <c r="B924" s="19"/>
-      <c r="C924" s="19"/>
-      <c r="D924" s="19"/>
-      <c r="E924" s="19"/>
-      <c r="F924" s="19"/>
-      <c r="G924" s="19"/>
-      <c r="H924" s="19"/>
-      <c r="I924" s="19"/>
+      <c r="A924" s="20"/>
+      <c r="B924" s="20"/>
+      <c r="C924" s="20"/>
+      <c r="D924" s="20"/>
+      <c r="E924" s="20"/>
+      <c r="F924" s="20"/>
+      <c r="G924" s="20"/>
+      <c r="H924" s="20"/>
+      <c r="I924" s="20"/>
     </row>
     <row r="925" ht="15.75" customHeight="1">
-      <c r="A925" s="19"/>
-      <c r="B925" s="19"/>
-      <c r="C925" s="19"/>
-      <c r="D925" s="19"/>
-      <c r="E925" s="19"/>
-      <c r="F925" s="19"/>
-      <c r="G925" s="19"/>
-      <c r="H925" s="19"/>
-      <c r="I925" s="19"/>
+      <c r="A925" s="20"/>
+      <c r="B925" s="20"/>
+      <c r="C925" s="20"/>
+      <c r="D925" s="20"/>
+      <c r="E925" s="20"/>
+      <c r="F925" s="20"/>
+      <c r="G925" s="20"/>
+      <c r="H925" s="20"/>
+      <c r="I925" s="20"/>
     </row>
     <row r="926" ht="15.75" customHeight="1">
-      <c r="A926" s="19"/>
-      <c r="B926" s="19"/>
-      <c r="C926" s="19"/>
-      <c r="D926" s="19"/>
-      <c r="E926" s="19"/>
-      <c r="F926" s="19"/>
-      <c r="G926" s="19"/>
-      <c r="H926" s="19"/>
-      <c r="I926" s="19"/>
+      <c r="A926" s="20"/>
+      <c r="B926" s="20"/>
+      <c r="C926" s="20"/>
+      <c r="D926" s="20"/>
+      <c r="E926" s="20"/>
+      <c r="F926" s="20"/>
+      <c r="G926" s="20"/>
+      <c r="H926" s="20"/>
+      <c r="I926" s="20"/>
     </row>
     <row r="927" ht="15.75" customHeight="1">
-      <c r="A927" s="19"/>
-      <c r="B927" s="19"/>
-      <c r="C927" s="19"/>
-      <c r="D927" s="19"/>
-      <c r="E927" s="19"/>
-      <c r="F927" s="19"/>
-      <c r="G927" s="19"/>
-      <c r="H927" s="19"/>
-      <c r="I927" s="19"/>
+      <c r="A927" s="20"/>
+      <c r="B927" s="20"/>
+      <c r="C927" s="20"/>
+      <c r="D927" s="20"/>
+      <c r="E927" s="20"/>
+      <c r="F927" s="20"/>
+      <c r="G927" s="20"/>
+      <c r="H927" s="20"/>
+      <c r="I927" s="20"/>
     </row>
     <row r="928" ht="15.75" customHeight="1">
-      <c r="A928" s="19"/>
-      <c r="B928" s="19"/>
-      <c r="C928" s="19"/>
-      <c r="D928" s="19"/>
-      <c r="E928" s="19"/>
-      <c r="F928" s="19"/>
-      <c r="G928" s="19"/>
-      <c r="H928" s="19"/>
-      <c r="I928" s="19"/>
+      <c r="A928" s="20"/>
+      <c r="B928" s="20"/>
+      <c r="C928" s="20"/>
+      <c r="D928" s="20"/>
+      <c r="E928" s="20"/>
+      <c r="F928" s="20"/>
+      <c r="G928" s="20"/>
+      <c r="H928" s="20"/>
+      <c r="I928" s="20"/>
     </row>
     <row r="929" ht="15.75" customHeight="1">
-      <c r="A929" s="19"/>
-      <c r="B929" s="19"/>
-      <c r="C929" s="19"/>
-      <c r="D929" s="19"/>
-      <c r="E929" s="19"/>
-      <c r="F929" s="19"/>
-      <c r="G929" s="19"/>
-      <c r="H929" s="19"/>
-      <c r="I929" s="19"/>
+      <c r="A929" s="20"/>
+      <c r="B929" s="20"/>
+      <c r="C929" s="20"/>
+      <c r="D929" s="20"/>
+      <c r="E929" s="20"/>
+      <c r="F929" s="20"/>
+      <c r="G929" s="20"/>
+      <c r="H929" s="20"/>
+      <c r="I929" s="20"/>
     </row>
     <row r="930" ht="15.75" customHeight="1">
-      <c r="A930" s="19"/>
-      <c r="B930" s="19"/>
-      <c r="C930" s="19"/>
-      <c r="D930" s="19"/>
-      <c r="E930" s="19"/>
-      <c r="F930" s="19"/>
-      <c r="G930" s="19"/>
-      <c r="H930" s="19"/>
-      <c r="I930" s="19"/>
+      <c r="A930" s="20"/>
+      <c r="B930" s="20"/>
+      <c r="C930" s="20"/>
+      <c r="D930" s="20"/>
+      <c r="E930" s="20"/>
+      <c r="F930" s="20"/>
+      <c r="G930" s="20"/>
+      <c r="H930" s="20"/>
+      <c r="I930" s="20"/>
     </row>
     <row r="931" ht="15.75" customHeight="1">
-      <c r="A931" s="19"/>
-      <c r="B931" s="19"/>
-      <c r="C931" s="19"/>
-      <c r="D931" s="19"/>
-      <c r="E931" s="19"/>
-      <c r="F931" s="19"/>
-      <c r="G931" s="19"/>
-      <c r="H931" s="19"/>
-      <c r="I931" s="19"/>
+      <c r="A931" s="20"/>
+      <c r="B931" s="20"/>
+      <c r="C931" s="20"/>
+      <c r="D931" s="20"/>
+      <c r="E931" s="20"/>
+      <c r="F931" s="20"/>
+      <c r="G931" s="20"/>
+      <c r="H931" s="20"/>
+      <c r="I931" s="20"/>
     </row>
     <row r="932" ht="15.75" customHeight="1">
-      <c r="A932" s="19"/>
-      <c r="B932" s="19"/>
-      <c r="C932" s="19"/>
-      <c r="D932" s="19"/>
-      <c r="E932" s="19"/>
-      <c r="F932" s="19"/>
-      <c r="G932" s="19"/>
-      <c r="H932" s="19"/>
-      <c r="I932" s="19"/>
+      <c r="A932" s="20"/>
+      <c r="B932" s="20"/>
+      <c r="C932" s="20"/>
+      <c r="D932" s="20"/>
+      <c r="E932" s="20"/>
+      <c r="F932" s="20"/>
+      <c r="G932" s="20"/>
+      <c r="H932" s="20"/>
+      <c r="I932" s="20"/>
     </row>
     <row r="933" ht="15.75" customHeight="1">
-      <c r="A933" s="19"/>
-      <c r="B933" s="19"/>
-      <c r="C933" s="19"/>
-      <c r="D933" s="19"/>
-      <c r="E933" s="19"/>
-      <c r="F933" s="19"/>
-      <c r="G933" s="19"/>
-      <c r="H933" s="19"/>
-      <c r="I933" s="19"/>
+      <c r="A933" s="20"/>
+      <c r="B933" s="20"/>
+      <c r="C933" s="20"/>
+      <c r="D933" s="20"/>
+      <c r="E933" s="20"/>
+      <c r="F933" s="20"/>
+      <c r="G933" s="20"/>
+      <c r="H933" s="20"/>
+      <c r="I933" s="20"/>
     </row>
     <row r="934" ht="15.75" customHeight="1">
-      <c r="A934" s="19"/>
-      <c r="B934" s="19"/>
-      <c r="C934" s="19"/>
-      <c r="D934" s="19"/>
-      <c r="E934" s="19"/>
-      <c r="F934" s="19"/>
-      <c r="G934" s="19"/>
-      <c r="H934" s="19"/>
-      <c r="I934" s="19"/>
+      <c r="A934" s="20"/>
+      <c r="B934" s="20"/>
+      <c r="C934" s="20"/>
+      <c r="D934" s="20"/>
+      <c r="E934" s="20"/>
+      <c r="F934" s="20"/>
+      <c r="G934" s="20"/>
+      <c r="H934" s="20"/>
+      <c r="I934" s="20"/>
     </row>
     <row r="935" ht="15.75" customHeight="1">
-      <c r="A935" s="19"/>
-      <c r="B935" s="19"/>
-      <c r="C935" s="19"/>
-      <c r="D935" s="19"/>
-      <c r="E935" s="19"/>
-      <c r="F935" s="19"/>
-      <c r="G935" s="19"/>
-      <c r="H935" s="19"/>
-      <c r="I935" s="19"/>
+      <c r="A935" s="20"/>
+      <c r="B935" s="20"/>
+      <c r="C935" s="20"/>
+      <c r="D935" s="20"/>
+      <c r="E935" s="20"/>
+      <c r="F935" s="20"/>
+      <c r="G935" s="20"/>
+      <c r="H935" s="20"/>
+      <c r="I935" s="20"/>
     </row>
     <row r="936" ht="15.75" customHeight="1">
-      <c r="A936" s="19"/>
-      <c r="B936" s="19"/>
-      <c r="C936" s="19"/>
-      <c r="D936" s="19"/>
-      <c r="E936" s="19"/>
-      <c r="F936" s="19"/>
-      <c r="G936" s="19"/>
-      <c r="H936" s="19"/>
-      <c r="I936" s="19"/>
+      <c r="A936" s="20"/>
+      <c r="B936" s="20"/>
+      <c r="C936" s="20"/>
+      <c r="D936" s="20"/>
+      <c r="E936" s="20"/>
+      <c r="F936" s="20"/>
+      <c r="G936" s="20"/>
+      <c r="H936" s="20"/>
+      <c r="I936" s="20"/>
     </row>
     <row r="937" ht="15.75" customHeight="1">
-      <c r="A937" s="19"/>
-      <c r="B937" s="19"/>
-      <c r="C937" s="19"/>
-      <c r="D937" s="19"/>
-      <c r="E937" s="19"/>
-      <c r="F937" s="19"/>
-      <c r="G937" s="19"/>
-      <c r="H937" s="19"/>
-      <c r="I937" s="19"/>
+      <c r="A937" s="20"/>
+      <c r="B937" s="20"/>
+      <c r="C937" s="20"/>
+      <c r="D937" s="20"/>
+      <c r="E937" s="20"/>
+      <c r="F937" s="20"/>
+      <c r="G937" s="20"/>
+      <c r="H937" s="20"/>
+      <c r="I937" s="20"/>
     </row>
     <row r="938" ht="15.75" customHeight="1">
-      <c r="A938" s="19"/>
-      <c r="B938" s="19"/>
-      <c r="C938" s="19"/>
-      <c r="D938" s="19"/>
-      <c r="E938" s="19"/>
-      <c r="F938" s="19"/>
-      <c r="G938" s="19"/>
-      <c r="H938" s="19"/>
-      <c r="I938" s="19"/>
+      <c r="A938" s="20"/>
+      <c r="B938" s="20"/>
+      <c r="C938" s="20"/>
+      <c r="D938" s="20"/>
+      <c r="E938" s="20"/>
+      <c r="F938" s="20"/>
+      <c r="G938" s="20"/>
+      <c r="H938" s="20"/>
+      <c r="I938" s="20"/>
     </row>
     <row r="939" ht="15.75" customHeight="1">
-      <c r="A939" s="19"/>
-      <c r="B939" s="19"/>
-      <c r="C939" s="19"/>
-      <c r="D939" s="19"/>
-      <c r="E939" s="19"/>
-      <c r="F939" s="19"/>
-      <c r="G939" s="19"/>
-      <c r="H939" s="19"/>
-      <c r="I939" s="19"/>
+      <c r="A939" s="20"/>
+      <c r="B939" s="20"/>
+      <c r="C939" s="20"/>
+      <c r="D939" s="20"/>
+      <c r="E939" s="20"/>
+      <c r="F939" s="20"/>
+      <c r="G939" s="20"/>
+      <c r="H939" s="20"/>
+      <c r="I939" s="20"/>
     </row>
     <row r="940" ht="15.75" customHeight="1">
-      <c r="A940" s="19"/>
-      <c r="B940" s="19"/>
-      <c r="C940" s="19"/>
-      <c r="D940" s="19"/>
-      <c r="E940" s="19"/>
-      <c r="F940" s="19"/>
-      <c r="G940" s="19"/>
-      <c r="H940" s="19"/>
-      <c r="I940" s="19"/>
+      <c r="A940" s="20"/>
+      <c r="B940" s="20"/>
+      <c r="C940" s="20"/>
+      <c r="D940" s="20"/>
+      <c r="E940" s="20"/>
+      <c r="F940" s="20"/>
+      <c r="G940" s="20"/>
+      <c r="H940" s="20"/>
+      <c r="I940" s="20"/>
     </row>
     <row r="941" ht="15.75" customHeight="1">
-      <c r="A941" s="19"/>
-      <c r="B941" s="19"/>
-      <c r="C941" s="19"/>
-      <c r="D941" s="19"/>
-      <c r="E941" s="19"/>
-      <c r="F941" s="19"/>
-      <c r="G941" s="19"/>
-      <c r="H941" s="19"/>
-      <c r="I941" s="19"/>
+      <c r="A941" s="20"/>
+      <c r="B941" s="20"/>
+      <c r="C941" s="20"/>
+      <c r="D941" s="20"/>
+      <c r="E941" s="20"/>
+      <c r="F941" s="20"/>
+      <c r="G941" s="20"/>
+      <c r="H941" s="20"/>
+      <c r="I941" s="20"/>
     </row>
     <row r="942" ht="15.75" customHeight="1">
-      <c r="A942" s="19"/>
-      <c r="B942" s="19"/>
-      <c r="C942" s="19"/>
-      <c r="D942" s="19"/>
-      <c r="E942" s="19"/>
-      <c r="F942" s="19"/>
-      <c r="G942" s="19"/>
-      <c r="H942" s="19"/>
-      <c r="I942" s="19"/>
+      <c r="A942" s="20"/>
+      <c r="B942" s="20"/>
+      <c r="C942" s="20"/>
+      <c r="D942" s="20"/>
+      <c r="E942" s="20"/>
+      <c r="F942" s="20"/>
+      <c r="G942" s="20"/>
+      <c r="H942" s="20"/>
+      <c r="I942" s="20"/>
     </row>
     <row r="943" ht="15.75" customHeight="1">
-      <c r="A943" s="19"/>
-      <c r="B943" s="19"/>
-      <c r="C943" s="19"/>
-      <c r="D943" s="19"/>
-      <c r="E943" s="19"/>
-      <c r="F943" s="19"/>
-      <c r="G943" s="19"/>
-      <c r="H943" s="19"/>
-      <c r="I943" s="19"/>
+      <c r="A943" s="20"/>
+      <c r="B943" s="20"/>
+      <c r="C943" s="20"/>
+      <c r="D943" s="20"/>
+      <c r="E943" s="20"/>
+      <c r="F943" s="20"/>
+      <c r="G943" s="20"/>
+      <c r="H943" s="20"/>
+      <c r="I943" s="20"/>
     </row>
     <row r="944" ht="15.75" customHeight="1">
-      <c r="A944" s="19"/>
-      <c r="B944" s="19"/>
-      <c r="C944" s="19"/>
-      <c r="D944" s="19"/>
-      <c r="E944" s="19"/>
-      <c r="F944" s="19"/>
-      <c r="G944" s="19"/>
-      <c r="H944" s="19"/>
-      <c r="I944" s="19"/>
+      <c r="A944" s="20"/>
+      <c r="B944" s="20"/>
+      <c r="C944" s="20"/>
+      <c r="D944" s="20"/>
+      <c r="E944" s="20"/>
+      <c r="F944" s="20"/>
+      <c r="G944" s="20"/>
+      <c r="H944" s="20"/>
+      <c r="I944" s="20"/>
     </row>
     <row r="945" ht="15.75" customHeight="1">
-      <c r="A945" s="19"/>
-      <c r="B945" s="19"/>
-      <c r="C945" s="19"/>
-      <c r="D945" s="19"/>
-      <c r="E945" s="19"/>
-      <c r="F945" s="19"/>
-      <c r="G945" s="19"/>
-      <c r="H945" s="19"/>
-      <c r="I945" s="19"/>
+      <c r="A945" s="20"/>
+      <c r="B945" s="20"/>
+      <c r="C945" s="20"/>
+      <c r="D945" s="20"/>
+      <c r="E945" s="20"/>
+      <c r="F945" s="20"/>
+      <c r="G945" s="20"/>
+      <c r="H945" s="20"/>
+      <c r="I945" s="20"/>
     </row>
     <row r="946" ht="15.75" customHeight="1">
-      <c r="A946" s="19"/>
-      <c r="B946" s="19"/>
-      <c r="C946" s="19"/>
-      <c r="D946" s="19"/>
-      <c r="E946" s="19"/>
-      <c r="F946" s="19"/>
-      <c r="G946" s="19"/>
-      <c r="H946" s="19"/>
-      <c r="I946" s="19"/>
+      <c r="A946" s="20"/>
+      <c r="B946" s="20"/>
+      <c r="C946" s="20"/>
+      <c r="D946" s="20"/>
+      <c r="E946" s="20"/>
+      <c r="F946" s="20"/>
+      <c r="G946" s="20"/>
+      <c r="H946" s="20"/>
+      <c r="I946" s="20"/>
     </row>
     <row r="947" ht="15.75" customHeight="1">
-      <c r="A947" s="19"/>
-      <c r="B947" s="19"/>
-      <c r="C947" s="19"/>
-      <c r="D947" s="19"/>
-      <c r="E947" s="19"/>
-      <c r="F947" s="19"/>
-      <c r="G947" s="19"/>
-      <c r="H947" s="19"/>
-      <c r="I947" s="19"/>
+      <c r="A947" s="20"/>
+      <c r="B947" s="20"/>
+      <c r="C947" s="20"/>
+      <c r="D947" s="20"/>
+      <c r="E947" s="20"/>
+      <c r="F947" s="20"/>
+      <c r="G947" s="20"/>
+      <c r="H947" s="20"/>
+      <c r="I947" s="20"/>
     </row>
     <row r="948" ht="15.75" customHeight="1">
-      <c r="A948" s="19"/>
-      <c r="B948" s="19"/>
-      <c r="C948" s="19"/>
-      <c r="D948" s="19"/>
-      <c r="E948" s="19"/>
-      <c r="F948" s="19"/>
-      <c r="G948" s="19"/>
-      <c r="H948" s="19"/>
-      <c r="I948" s="19"/>
+      <c r="A948" s="20"/>
+      <c r="B948" s="20"/>
+      <c r="C948" s="20"/>
+      <c r="D948" s="20"/>
+      <c r="E948" s="20"/>
+      <c r="F948" s="20"/>
+      <c r="G948" s="20"/>
+      <c r="H948" s="20"/>
+      <c r="I948" s="20"/>
     </row>
     <row r="949" ht="15.75" customHeight="1">
-      <c r="A949" s="19"/>
-      <c r="B949" s="19"/>
-      <c r="C949" s="19"/>
-      <c r="D949" s="19"/>
-      <c r="E949" s="19"/>
-      <c r="F949" s="19"/>
-      <c r="G949" s="19"/>
-      <c r="H949" s="19"/>
-      <c r="I949" s="19"/>
+      <c r="A949" s="20"/>
+      <c r="B949" s="20"/>
+      <c r="C949" s="20"/>
+      <c r="D949" s="20"/>
+      <c r="E949" s="20"/>
+      <c r="F949" s="20"/>
+      <c r="G949" s="20"/>
+      <c r="H949" s="20"/>
+      <c r="I949" s="20"/>
     </row>
     <row r="950" ht="15.75" customHeight="1">
-      <c r="A950" s="19"/>
-      <c r="B950" s="19"/>
-      <c r="C950" s="19"/>
-      <c r="D950" s="19"/>
-      <c r="E950" s="19"/>
-      <c r="F950" s="19"/>
-      <c r="G950" s="19"/>
-      <c r="H950" s="19"/>
-      <c r="I950" s="19"/>
+      <c r="A950" s="20"/>
+      <c r="B950" s="20"/>
+      <c r="C950" s="20"/>
+      <c r="D950" s="20"/>
+      <c r="E950" s="20"/>
+      <c r="F950" s="20"/>
+      <c r="G950" s="20"/>
+      <c r="H950" s="20"/>
+      <c r="I950" s="20"/>
     </row>
     <row r="951" ht="15.75" customHeight="1">
-      <c r="A951" s="19"/>
-      <c r="B951" s="19"/>
-      <c r="C951" s="19"/>
-      <c r="D951" s="19"/>
-      <c r="E951" s="19"/>
-      <c r="F951" s="19"/>
-      <c r="G951" s="19"/>
-      <c r="H951" s="19"/>
-      <c r="I951" s="19"/>
+      <c r="A951" s="20"/>
+      <c r="B951" s="20"/>
+      <c r="C951" s="20"/>
+      <c r="D951" s="20"/>
+      <c r="E951" s="20"/>
+      <c r="F951" s="20"/>
+      <c r="G951" s="20"/>
+      <c r="H951" s="20"/>
+      <c r="I951" s="20"/>
     </row>
     <row r="952" ht="15.75" customHeight="1">
-      <c r="A952" s="19"/>
-      <c r="B952" s="19"/>
-      <c r="C952" s="19"/>
-      <c r="D952" s="19"/>
-      <c r="E952" s="19"/>
-      <c r="F952" s="19"/>
-      <c r="G952" s="19"/>
-      <c r="H952" s="19"/>
-      <c r="I952" s="19"/>
+      <c r="A952" s="20"/>
+      <c r="B952" s="20"/>
+      <c r="C952" s="20"/>
+      <c r="D952" s="20"/>
+      <c r="E952" s="20"/>
+      <c r="F952" s="20"/>
+      <c r="G952" s="20"/>
+      <c r="H952" s="20"/>
+      <c r="I952" s="20"/>
     </row>
     <row r="953" ht="15.75" customHeight="1">
-      <c r="A953" s="19"/>
-      <c r="B953" s="19"/>
-      <c r="C953" s="19"/>
-      <c r="D953" s="19"/>
-      <c r="E953" s="19"/>
-      <c r="F953" s="19"/>
-      <c r="G953" s="19"/>
-      <c r="H953" s="19"/>
-      <c r="I953" s="19"/>
+      <c r="A953" s="20"/>
+      <c r="B953" s="20"/>
+      <c r="C953" s="20"/>
+      <c r="D953" s="20"/>
+      <c r="E953" s="20"/>
+      <c r="F953" s="20"/>
+      <c r="G953" s="20"/>
+      <c r="H953" s="20"/>
+      <c r="I953" s="20"/>
     </row>
     <row r="954" ht="15.75" customHeight="1">
-      <c r="A954" s="19"/>
-      <c r="B954" s="19"/>
-      <c r="C954" s="19"/>
-      <c r="D954" s="19"/>
-      <c r="E954" s="19"/>
-      <c r="F954" s="19"/>
-      <c r="G954" s="19"/>
-      <c r="H954" s="19"/>
-      <c r="I954" s="19"/>
+      <c r="A954" s="20"/>
+      <c r="B954" s="20"/>
+      <c r="C954" s="20"/>
+      <c r="D954" s="20"/>
+      <c r="E954" s="20"/>
+      <c r="F954" s="20"/>
+      <c r="G954" s="20"/>
+      <c r="H954" s="20"/>
+      <c r="I954" s="20"/>
     </row>
     <row r="955" ht="15.75" customHeight="1">
-      <c r="A955" s="19"/>
-      <c r="B955" s="19"/>
-      <c r="C955" s="19"/>
-      <c r="D955" s="19"/>
-      <c r="E955" s="19"/>
-      <c r="F955" s="19"/>
-      <c r="G955" s="19"/>
-      <c r="H955" s="19"/>
-      <c r="I955" s="19"/>
+      <c r="A955" s="20"/>
+      <c r="B955" s="20"/>
+      <c r="C955" s="20"/>
+      <c r="D955" s="20"/>
+      <c r="E955" s="20"/>
+      <c r="F955" s="20"/>
+      <c r="G955" s="20"/>
+      <c r="H955" s="20"/>
+      <c r="I955" s="20"/>
     </row>
     <row r="956" ht="15.75" customHeight="1">
-      <c r="A956" s="19"/>
-      <c r="B956" s="19"/>
-      <c r="C956" s="19"/>
-      <c r="D956" s="19"/>
-      <c r="E956" s="19"/>
-      <c r="F956" s="19"/>
-      <c r="G956" s="19"/>
-      <c r="H956" s="19"/>
-      <c r="I956" s="19"/>
+      <c r="A956" s="20"/>
+      <c r="B956" s="20"/>
+      <c r="C956" s="20"/>
+      <c r="D956" s="20"/>
+      <c r="E956" s="20"/>
+      <c r="F956" s="20"/>
+      <c r="G956" s="20"/>
+      <c r="H956" s="20"/>
+      <c r="I956" s="20"/>
     </row>
     <row r="957" ht="15.75" customHeight="1">
-      <c r="A957" s="19"/>
-      <c r="B957" s="19"/>
-      <c r="C957" s="19"/>
-      <c r="D957" s="19"/>
-      <c r="E957" s="19"/>
-      <c r="F957" s="19"/>
-      <c r="G957" s="19"/>
-      <c r="H957" s="19"/>
-      <c r="I957" s="19"/>
+      <c r="A957" s="20"/>
+      <c r="B957" s="20"/>
+      <c r="C957" s="20"/>
+      <c r="D957" s="20"/>
+      <c r="E957" s="20"/>
+      <c r="F957" s="20"/>
+      <c r="G957" s="20"/>
+      <c r="H957" s="20"/>
+      <c r="I957" s="20"/>
     </row>
     <row r="958" ht="15.75" customHeight="1">
-      <c r="A958" s="19"/>
-      <c r="B958" s="19"/>
-      <c r="C958" s="19"/>
-      <c r="D958" s="19"/>
-      <c r="E958" s="19"/>
-      <c r="F958" s="19"/>
-      <c r="G958" s="19"/>
-      <c r="H958" s="19"/>
-      <c r="I958" s="19"/>
+      <c r="A958" s="20"/>
+      <c r="B958" s="20"/>
+      <c r="C958" s="20"/>
+      <c r="D958" s="20"/>
+      <c r="E958" s="20"/>
+      <c r="F958" s="20"/>
+      <c r="G958" s="20"/>
+      <c r="H958" s="20"/>
+      <c r="I958" s="20"/>
     </row>
     <row r="959" ht="15.75" customHeight="1">
-      <c r="A959" s="19"/>
-      <c r="B959" s="19"/>
-      <c r="C959" s="19"/>
-      <c r="D959" s="19"/>
-      <c r="E959" s="19"/>
-      <c r="F959" s="19"/>
-      <c r="G959" s="19"/>
-      <c r="H959" s="19"/>
-      <c r="I959" s="19"/>
+      <c r="A959" s="20"/>
+      <c r="B959" s="20"/>
+      <c r="C959" s="20"/>
+      <c r="D959" s="20"/>
+      <c r="E959" s="20"/>
+      <c r="F959" s="20"/>
+      <c r="G959" s="20"/>
+      <c r="H959" s="20"/>
+      <c r="I959" s="20"/>
     </row>
     <row r="960" ht="15.75" customHeight="1">
-      <c r="A960" s="19"/>
-      <c r="B960" s="19"/>
-      <c r="C960" s="19"/>
-      <c r="D960" s="19"/>
-      <c r="E960" s="19"/>
-      <c r="F960" s="19"/>
-      <c r="G960" s="19"/>
-      <c r="H960" s="19"/>
-      <c r="I960" s="19"/>
+      <c r="A960" s="20"/>
+      <c r="B960" s="20"/>
+      <c r="C960" s="20"/>
+      <c r="D960" s="20"/>
+      <c r="E960" s="20"/>
+      <c r="F960" s="20"/>
+      <c r="G960" s="20"/>
+      <c r="H960" s="20"/>
+      <c r="I960" s="20"/>
     </row>
     <row r="961" ht="15.75" customHeight="1">
-      <c r="A961" s="19"/>
-      <c r="B961" s="19"/>
-      <c r="C961" s="19"/>
-      <c r="D961" s="19"/>
-      <c r="E961" s="19"/>
-      <c r="F961" s="19"/>
-      <c r="G961" s="19"/>
-      <c r="H961" s="19"/>
-      <c r="I961" s="19"/>
+      <c r="A961" s="20"/>
+      <c r="B961" s="20"/>
+      <c r="C961" s="20"/>
+      <c r="D961" s="20"/>
+      <c r="E961" s="20"/>
+      <c r="F961" s="20"/>
+      <c r="G961" s="20"/>
+      <c r="H961" s="20"/>
+      <c r="I961" s="20"/>
     </row>
     <row r="962" ht="15.75" customHeight="1">
-      <c r="A962" s="19"/>
-      <c r="B962" s="19"/>
-      <c r="C962" s="19"/>
-      <c r="D962" s="19"/>
-      <c r="E962" s="19"/>
-      <c r="F962" s="19"/>
-      <c r="G962" s="19"/>
-      <c r="H962" s="19"/>
-      <c r="I962" s="19"/>
+      <c r="A962" s="20"/>
+      <c r="B962" s="20"/>
+      <c r="C962" s="20"/>
+      <c r="D962" s="20"/>
+      <c r="E962" s="20"/>
+      <c r="F962" s="20"/>
+      <c r="G962" s="20"/>
+      <c r="H962" s="20"/>
+      <c r="I962" s="20"/>
     </row>
     <row r="963" ht="15.75" customHeight="1">
-      <c r="A963" s="19"/>
-      <c r="B963" s="19"/>
-      <c r="C963" s="19"/>
-      <c r="D963" s="19"/>
-      <c r="E963" s="19"/>
-      <c r="F963" s="19"/>
-      <c r="G963" s="19"/>
-      <c r="H963" s="19"/>
-      <c r="I963" s="19"/>
+      <c r="A963" s="20"/>
+      <c r="B963" s="20"/>
+      <c r="C963" s="20"/>
+      <c r="D963" s="20"/>
+      <c r="E963" s="20"/>
+      <c r="F963" s="20"/>
+      <c r="G963" s="20"/>
+      <c r="H963" s="20"/>
+      <c r="I963" s="20"/>
     </row>
     <row r="964" ht="15.75" customHeight="1">
-      <c r="A964" s="19"/>
-      <c r="B964" s="19"/>
-      <c r="C964" s="19"/>
-      <c r="D964" s="19"/>
-      <c r="E964" s="19"/>
-      <c r="F964" s="19"/>
-      <c r="G964" s="19"/>
-      <c r="H964" s="19"/>
-      <c r="I964" s="19"/>
+      <c r="A964" s="20"/>
+      <c r="B964" s="20"/>
+      <c r="C964" s="20"/>
+      <c r="D964" s="20"/>
+      <c r="E964" s="20"/>
+      <c r="F964" s="20"/>
+      <c r="G964" s="20"/>
+      <c r="H964" s="20"/>
+      <c r="I964" s="20"/>
     </row>
     <row r="965" ht="15.75" customHeight="1">
-      <c r="A965" s="19"/>
-      <c r="B965" s="19"/>
-      <c r="C965" s="19"/>
-      <c r="D965" s="19"/>
-      <c r="E965" s="19"/>
-      <c r="F965" s="19"/>
-      <c r="G965" s="19"/>
-      <c r="H965" s="19"/>
-      <c r="I965" s="19"/>
+      <c r="A965" s="20"/>
+      <c r="B965" s="20"/>
+      <c r="C965" s="20"/>
+      <c r="D965" s="20"/>
+      <c r="E965" s="20"/>
+      <c r="F965" s="20"/>
+      <c r="G965" s="20"/>
+      <c r="H965" s="20"/>
+      <c r="I965" s="20"/>
     </row>
     <row r="966" ht="15.75" customHeight="1">
-      <c r="A966" s="19"/>
-      <c r="B966" s="19"/>
-      <c r="C966" s="19"/>
-      <c r="D966" s="19"/>
-      <c r="E966" s="19"/>
-      <c r="F966" s="19"/>
-      <c r="G966" s="19"/>
-      <c r="H966" s="19"/>
-      <c r="I966" s="19"/>
+      <c r="A966" s="20"/>
+      <c r="B966" s="20"/>
+      <c r="C966" s="20"/>
+      <c r="D966" s="20"/>
+      <c r="E966" s="20"/>
+      <c r="F966" s="20"/>
+      <c r="G966" s="20"/>
+      <c r="H966" s="20"/>
+      <c r="I966" s="20"/>
     </row>
     <row r="967" ht="15.75" customHeight="1">
-      <c r="A967" s="19"/>
-      <c r="B967" s="19"/>
-      <c r="C967" s="19"/>
-      <c r="D967" s="19"/>
-      <c r="E967" s="19"/>
-      <c r="F967" s="19"/>
-      <c r="G967" s="19"/>
-      <c r="H967" s="19"/>
-      <c r="I967" s="19"/>
+      <c r="A967" s="20"/>
+      <c r="B967" s="20"/>
+      <c r="C967" s="20"/>
+      <c r="D967" s="20"/>
+      <c r="E967" s="20"/>
+      <c r="F967" s="20"/>
+      <c r="G967" s="20"/>
+      <c r="H967" s="20"/>
+      <c r="I967" s="20"/>
     </row>
     <row r="968" ht="15.75" customHeight="1">
-      <c r="A968" s="19"/>
-      <c r="B968" s="19"/>
-      <c r="C968" s="19"/>
-      <c r="D968" s="19"/>
-      <c r="E968" s="19"/>
-      <c r="F968" s="19"/>
-      <c r="G968" s="19"/>
-      <c r="H968" s="19"/>
-      <c r="I968" s="19"/>
+      <c r="A968" s="20"/>
+      <c r="B968" s="20"/>
+      <c r="C968" s="20"/>
+      <c r="D968" s="20"/>
+      <c r="E968" s="20"/>
+      <c r="F968" s="20"/>
+      <c r="G968" s="20"/>
+      <c r="H968" s="20"/>
+      <c r="I968" s="20"/>
     </row>
     <row r="969" ht="15.75" customHeight="1">
-      <c r="A969" s="19"/>
-      <c r="B969" s="19"/>
-      <c r="C969" s="19"/>
-      <c r="D969" s="19"/>
-      <c r="E969" s="19"/>
-      <c r="F969" s="19"/>
-      <c r="G969" s="19"/>
-      <c r="H969" s="19"/>
-      <c r="I969" s="19"/>
+      <c r="A969" s="20"/>
+      <c r="B969" s="20"/>
+      <c r="C969" s="20"/>
+      <c r="D969" s="20"/>
+      <c r="E969" s="20"/>
+      <c r="F969" s="20"/>
+      <c r="G969" s="20"/>
+      <c r="H969" s="20"/>
+      <c r="I969" s="20"/>
     </row>
     <row r="970" ht="15.75" customHeight="1">
-      <c r="A970" s="19"/>
-      <c r="B970" s="19"/>
-      <c r="C970" s="19"/>
-      <c r="D970" s="19"/>
-      <c r="E970" s="19"/>
-      <c r="F970" s="19"/>
-      <c r="G970" s="19"/>
-      <c r="H970" s="19"/>
-      <c r="I970" s="19"/>
+      <c r="A970" s="20"/>
+      <c r="B970" s="20"/>
+      <c r="C970" s="20"/>
+      <c r="D970" s="20"/>
+      <c r="E970" s="20"/>
+      <c r="F970" s="20"/>
+      <c r="G970" s="20"/>
+      <c r="H970" s="20"/>
+      <c r="I970" s="20"/>
     </row>
     <row r="971" ht="15.75" customHeight="1">
-      <c r="A971" s="19"/>
-      <c r="B971" s="19"/>
-      <c r="C971" s="19"/>
-      <c r="D971" s="19"/>
-      <c r="E971" s="19"/>
-      <c r="F971" s="19"/>
-      <c r="G971" s="19"/>
-      <c r="H971" s="19"/>
-      <c r="I971" s="19"/>
+      <c r="A971" s="20"/>
+      <c r="B971" s="20"/>
+      <c r="C971" s="20"/>
+      <c r="D971" s="20"/>
+      <c r="E971" s="20"/>
+      <c r="F971" s="20"/>
+      <c r="G971" s="20"/>
+      <c r="H971" s="20"/>
+      <c r="I971" s="20"/>
     </row>
     <row r="972" ht="15.75" customHeight="1">
-      <c r="A972" s="19"/>
-      <c r="B972" s="19"/>
-      <c r="C972" s="19"/>
-      <c r="D972" s="19"/>
-      <c r="E972" s="19"/>
-      <c r="F972" s="19"/>
-      <c r="G972" s="19"/>
-      <c r="H972" s="19"/>
-      <c r="I972" s="19"/>
+      <c r="A972" s="20"/>
+      <c r="B972" s="20"/>
+      <c r="C972" s="20"/>
+      <c r="D972" s="20"/>
+      <c r="E972" s="20"/>
+      <c r="F972" s="20"/>
+      <c r="G972" s="20"/>
+      <c r="H972" s="20"/>
+      <c r="I972" s="20"/>
     </row>
     <row r="973" ht="15.75" customHeight="1">
-      <c r="A973" s="19"/>
-      <c r="B973" s="19"/>
-      <c r="C973" s="19"/>
-      <c r="D973" s="19"/>
-      <c r="E973" s="19"/>
-      <c r="F973" s="19"/>
-      <c r="G973" s="19"/>
-      <c r="H973" s="19"/>
-      <c r="I973" s="19"/>
+      <c r="A973" s="20"/>
+      <c r="B973" s="20"/>
+      <c r="C973" s="20"/>
+      <c r="D973" s="20"/>
+      <c r="E973" s="20"/>
+      <c r="F973" s="20"/>
+      <c r="G973" s="20"/>
+      <c r="H973" s="20"/>
+      <c r="I973" s="20"/>
     </row>
     <row r="974" ht="15.75" customHeight="1">
-      <c r="A974" s="19"/>
-      <c r="B974" s="19"/>
-      <c r="C974" s="19"/>
-      <c r="D974" s="19"/>
-      <c r="E974" s="19"/>
-      <c r="F974" s="19"/>
-      <c r="G974" s="19"/>
-      <c r="H974" s="19"/>
-      <c r="I974" s="19"/>
+      <c r="A974" s="20"/>
+      <c r="B974" s="20"/>
+      <c r="C974" s="20"/>
+      <c r="D974" s="20"/>
+      <c r="E974" s="20"/>
+      <c r="F974" s="20"/>
+      <c r="G974" s="20"/>
+      <c r="H974" s="20"/>
+      <c r="I974" s="20"/>
     </row>
     <row r="975" ht="15.75" customHeight="1">
-      <c r="A975" s="19"/>
-      <c r="B975" s="19"/>
-      <c r="C975" s="19"/>
-      <c r="D975" s="19"/>
-      <c r="E975" s="19"/>
-      <c r="F975" s="19"/>
-      <c r="G975" s="19"/>
-      <c r="H975" s="19"/>
-      <c r="I975" s="19"/>
+      <c r="A975" s="20"/>
+      <c r="B975" s="20"/>
+      <c r="C975" s="20"/>
+      <c r="D975" s="20"/>
+      <c r="E975" s="20"/>
+      <c r="F975" s="20"/>
+      <c r="G975" s="20"/>
+      <c r="H975" s="20"/>
+      <c r="I975" s="20"/>
     </row>
     <row r="976" ht="15.75" customHeight="1">
-      <c r="A976" s="19"/>
-      <c r="B976" s="19"/>
-      <c r="C976" s="19"/>
-      <c r="D976" s="19"/>
-      <c r="E976" s="19"/>
-      <c r="F976" s="19"/>
-      <c r="G976" s="19"/>
-      <c r="H976" s="19"/>
-      <c r="I976" s="19"/>
+      <c r="A976" s="20"/>
+      <c r="B976" s="20"/>
+      <c r="C976" s="20"/>
+      <c r="D976" s="20"/>
+      <c r="E976" s="20"/>
+      <c r="F976" s="20"/>
+      <c r="G976" s="20"/>
+      <c r="H976" s="20"/>
+      <c r="I976" s="20"/>
     </row>
     <row r="977" ht="15.75" customHeight="1">
-      <c r="A977" s="19"/>
-      <c r="B977" s="19"/>
-      <c r="C977" s="19"/>
-      <c r="D977" s="19"/>
-      <c r="E977" s="19"/>
-      <c r="F977" s="19"/>
-      <c r="G977" s="19"/>
-      <c r="H977" s="19"/>
-      <c r="I977" s="19"/>
+      <c r="A977" s="20"/>
+      <c r="B977" s="20"/>
+      <c r="C977" s="20"/>
+      <c r="D977" s="20"/>
+      <c r="E977" s="20"/>
+      <c r="F977" s="20"/>
+      <c r="G977" s="20"/>
+      <c r="H977" s="20"/>
+      <c r="I977" s="20"/>
     </row>
     <row r="978" ht="15.75" customHeight="1">
-      <c r="A978" s="19"/>
-      <c r="B978" s="19"/>
-      <c r="C978" s="19"/>
-      <c r="D978" s="19"/>
-      <c r="E978" s="19"/>
-      <c r="F978" s="19"/>
-      <c r="G978" s="19"/>
-      <c r="H978" s="19"/>
-      <c r="I978" s="19"/>
+      <c r="A978" s="20"/>
+      <c r="B978" s="20"/>
+      <c r="C978" s="20"/>
+      <c r="D978" s="20"/>
+      <c r="E978" s="20"/>
+      <c r="F978" s="20"/>
+      <c r="G978" s="20"/>
+      <c r="H978" s="20"/>
+      <c r="I978" s="20"/>
     </row>
     <row r="979" ht="15.75" customHeight="1">
-      <c r="A979" s="19"/>
-      <c r="B979" s="19"/>
-      <c r="C979" s="19"/>
-      <c r="D979" s="19"/>
-      <c r="E979" s="19"/>
-      <c r="F979" s="19"/>
-      <c r="G979" s="19"/>
-      <c r="H979" s="19"/>
-      <c r="I979" s="19"/>
+      <c r="A979" s="20"/>
+      <c r="B979" s="20"/>
+      <c r="C979" s="20"/>
+      <c r="D979" s="20"/>
+      <c r="E979" s="20"/>
+      <c r="F979" s="20"/>
+      <c r="G979" s="20"/>
+      <c r="H979" s="20"/>
+      <c r="I979" s="20"/>
     </row>
     <row r="980" ht="15.75" customHeight="1">
-      <c r="A980" s="19"/>
-      <c r="B980" s="19"/>
-      <c r="C980" s="19"/>
-      <c r="D980" s="19"/>
-      <c r="E980" s="19"/>
-      <c r="F980" s="19"/>
-      <c r="G980" s="19"/>
-      <c r="H980" s="19"/>
-      <c r="I980" s="19"/>
+      <c r="A980" s="20"/>
+      <c r="B980" s="20"/>
+      <c r="C980" s="20"/>
+      <c r="D980" s="20"/>
+      <c r="E980" s="20"/>
+      <c r="F980" s="20"/>
+      <c r="G980" s="20"/>
+      <c r="H980" s="20"/>
+      <c r="I980" s="20"/>
     </row>
     <row r="981" ht="15.75" customHeight="1">
-      <c r="A981" s="19"/>
-      <c r="B981" s="19"/>
-      <c r="C981" s="19"/>
-      <c r="D981" s="19"/>
-      <c r="E981" s="19"/>
-      <c r="F981" s="19"/>
-      <c r="G981" s="19"/>
-      <c r="H981" s="19"/>
-      <c r="I981" s="19"/>
+      <c r="A981" s="20"/>
+      <c r="B981" s="20"/>
+      <c r="C981" s="20"/>
+      <c r="D981" s="20"/>
+      <c r="E981" s="20"/>
+      <c r="F981" s="20"/>
+      <c r="G981" s="20"/>
+      <c r="H981" s="20"/>
+      <c r="I981" s="20"/>
     </row>
     <row r="982" ht="15.75" customHeight="1">
-      <c r="A982" s="19"/>
-      <c r="B982" s="19"/>
-      <c r="C982" s="19"/>
-      <c r="D982" s="19"/>
-      <c r="E982" s="19"/>
-      <c r="F982" s="19"/>
-      <c r="G982" s="19"/>
-      <c r="H982" s="19"/>
-      <c r="I982" s="19"/>
+      <c r="A982" s="20"/>
+      <c r="B982" s="20"/>
+      <c r="C982" s="20"/>
+      <c r="D982" s="20"/>
+      <c r="E982" s="20"/>
+      <c r="F982" s="20"/>
+      <c r="G982" s="20"/>
+      <c r="H982" s="20"/>
+      <c r="I982" s="20"/>
     </row>
     <row r="983" ht="15.75" customHeight="1">
-      <c r="A983" s="19"/>
-      <c r="B983" s="19"/>
-      <c r="C983" s="19"/>
-      <c r="D983" s="19"/>
-      <c r="E983" s="19"/>
-      <c r="F983" s="19"/>
-      <c r="G983" s="19"/>
-      <c r="H983" s="19"/>
-      <c r="I983" s="19"/>
+      <c r="A983" s="20"/>
+      <c r="B983" s="20"/>
+      <c r="C983" s="20"/>
+      <c r="D983" s="20"/>
+      <c r="E983" s="20"/>
+      <c r="F983" s="20"/>
+      <c r="G983" s="20"/>
+      <c r="H983" s="20"/>
+      <c r="I983" s="20"/>
     </row>
     <row r="984" ht="15.75" customHeight="1">
-      <c r="A984" s="19"/>
-      <c r="B984" s="19"/>
-      <c r="C984" s="19"/>
-      <c r="D984" s="19"/>
-      <c r="E984" s="19"/>
-      <c r="F984" s="19"/>
-      <c r="G984" s="19"/>
-      <c r="H984" s="19"/>
-      <c r="I984" s="19"/>
+      <c r="A984" s="20"/>
+      <c r="B984" s="20"/>
+      <c r="C984" s="20"/>
+      <c r="D984" s="20"/>
+      <c r="E984" s="20"/>
+      <c r="F984" s="20"/>
+      <c r="G984" s="20"/>
+      <c r="H984" s="20"/>
+      <c r="I984" s="20"/>
     </row>
     <row r="985" ht="15.75" customHeight="1">
-      <c r="A985" s="19"/>
-      <c r="B985" s="19"/>
-      <c r="C985" s="19"/>
-      <c r="D985" s="19"/>
-      <c r="E985" s="19"/>
-      <c r="F985" s="19"/>
-      <c r="G985" s="19"/>
-      <c r="H985" s="19"/>
-      <c r="I985" s="19"/>
+      <c r="A985" s="20"/>
+      <c r="B985" s="20"/>
+      <c r="C985" s="20"/>
+      <c r="D985" s="20"/>
+      <c r="E985" s="20"/>
+      <c r="F985" s="20"/>
+      <c r="G985" s="20"/>
+      <c r="H985" s="20"/>
+      <c r="I985" s="20"/>
     </row>
     <row r="986" ht="15.75" customHeight="1">
-      <c r="A986" s="19"/>
-      <c r="B986" s="19"/>
-      <c r="C986" s="19"/>
-      <c r="D986" s="19"/>
-      <c r="E986" s="19"/>
-      <c r="F986" s="19"/>
-      <c r="G986" s="19"/>
-      <c r="H986" s="19"/>
-      <c r="I986" s="19"/>
+      <c r="A986" s="20"/>
+      <c r="B986" s="20"/>
+      <c r="C986" s="20"/>
+      <c r="D986" s="20"/>
+      <c r="E986" s="20"/>
+      <c r="F986" s="20"/>
+      <c r="G986" s="20"/>
+      <c r="H986" s="20"/>
+      <c r="I986" s="20"/>
     </row>
     <row r="987" ht="15.75" customHeight="1">
-      <c r="A987" s="19"/>
-      <c r="B987" s="19"/>
-      <c r="C987" s="19"/>
-      <c r="D987" s="19"/>
-      <c r="E987" s="19"/>
-      <c r="F987" s="19"/>
-      <c r="G987" s="19"/>
-      <c r="H987" s="19"/>
-      <c r="I987" s="19"/>
+      <c r="A987" s="20"/>
+      <c r="B987" s="20"/>
+      <c r="C987" s="20"/>
+      <c r="D987" s="20"/>
+      <c r="E987" s="20"/>
+      <c r="F987" s="20"/>
+      <c r="G987" s="20"/>
+      <c r="H987" s="20"/>
+      <c r="I987" s="20"/>
     </row>
     <row r="988" ht="15.75" customHeight="1">
-      <c r="A988" s="19"/>
-      <c r="B988" s="19"/>
-      <c r="C988" s="19"/>
-      <c r="D988" s="19"/>
-      <c r="E988" s="19"/>
-      <c r="F988" s="19"/>
-      <c r="G988" s="19"/>
-      <c r="H988" s="19"/>
-      <c r="I988" s="19"/>
+      <c r="A988" s="20"/>
+      <c r="B988" s="20"/>
+      <c r="C988" s="20"/>
+      <c r="D988" s="20"/>
+      <c r="E988" s="20"/>
+      <c r="F988" s="20"/>
+      <c r="G988" s="20"/>
+      <c r="H988" s="20"/>
+      <c r="I988" s="20"/>
     </row>
     <row r="989" ht="15.75" customHeight="1">
-      <c r="A989" s="19"/>
-      <c r="B989" s="19"/>
-      <c r="C989" s="19"/>
-      <c r="D989" s="19"/>
-      <c r="E989" s="19"/>
-      <c r="F989" s="19"/>
-      <c r="G989" s="19"/>
-      <c r="H989" s="19"/>
-      <c r="I989" s="19"/>
+      <c r="A989" s="20"/>
+      <c r="B989" s="20"/>
+      <c r="C989" s="20"/>
+      <c r="D989" s="20"/>
+      <c r="E989" s="20"/>
+      <c r="F989" s="20"/>
+      <c r="G989" s="20"/>
+      <c r="H989" s="20"/>
+      <c r="I989" s="20"/>
     </row>
     <row r="990" ht="15.75" customHeight="1">
-      <c r="A990" s="19"/>
-      <c r="B990" s="19"/>
-      <c r="C990" s="19"/>
-      <c r="D990" s="19"/>
-      <c r="E990" s="19"/>
-      <c r="F990" s="19"/>
-      <c r="G990" s="19"/>
-      <c r="H990" s="19"/>
-      <c r="I990" s="19"/>
+      <c r="A990" s="20"/>
+      <c r="B990" s="20"/>
+      <c r="C990" s="20"/>
+      <c r="D990" s="20"/>
+      <c r="E990" s="20"/>
+      <c r="F990" s="20"/>
+      <c r="G990" s="20"/>
+      <c r="H990" s="20"/>
+      <c r="I990" s="20"/>
     </row>
     <row r="991" ht="15.75" customHeight="1">
-      <c r="A991" s="19"/>
-      <c r="B991" s="19"/>
-      <c r="C991" s="19"/>
-      <c r="D991" s="19"/>
-      <c r="E991" s="19"/>
-      <c r="F991" s="19"/>
-      <c r="G991" s="19"/>
-      <c r="H991" s="19"/>
-      <c r="I991" s="19"/>
+      <c r="A991" s="20"/>
+      <c r="B991" s="20"/>
+      <c r="C991" s="20"/>
+      <c r="D991" s="20"/>
+      <c r="E991" s="20"/>
+      <c r="F991" s="20"/>
+      <c r="G991" s="20"/>
+      <c r="H991" s="20"/>
+      <c r="I991" s="20"/>
     </row>
     <row r="992" ht="15.75" customHeight="1">
-      <c r="A992" s="19"/>
-      <c r="B992" s="19"/>
-      <c r="C992" s="19"/>
-      <c r="D992" s="19"/>
-      <c r="E992" s="19"/>
-      <c r="F992" s="19"/>
-      <c r="G992" s="19"/>
-      <c r="H992" s="19"/>
-      <c r="I992" s="19"/>
+      <c r="A992" s="20"/>
+      <c r="B992" s="20"/>
+      <c r="C992" s="20"/>
+      <c r="D992" s="20"/>
+      <c r="E992" s="20"/>
+      <c r="F992" s="20"/>
+      <c r="G992" s="20"/>
+      <c r="H992" s="20"/>
+      <c r="I992" s="20"/>
     </row>
     <row r="993" ht="15.75" customHeight="1">
-      <c r="A993" s="19"/>
-      <c r="B993" s="19"/>
-      <c r="C993" s="19"/>
-      <c r="D993" s="19"/>
-      <c r="E993" s="19"/>
-      <c r="F993" s="19"/>
-      <c r="G993" s="19"/>
-      <c r="H993" s="19"/>
-      <c r="I993" s="19"/>
+      <c r="A993" s="20"/>
+      <c r="B993" s="20"/>
+      <c r="C993" s="20"/>
+      <c r="D993" s="20"/>
+      <c r="E993" s="20"/>
+      <c r="F993" s="20"/>
+      <c r="G993" s="20"/>
+      <c r="H993" s="20"/>
+      <c r="I993" s="20"/>
     </row>
     <row r="994" ht="15.75" customHeight="1">
-      <c r="A994" s="19"/>
-      <c r="B994" s="19"/>
-      <c r="C994" s="19"/>
-      <c r="D994" s="19"/>
-      <c r="E994" s="19"/>
-      <c r="F994" s="19"/>
-      <c r="G994" s="19"/>
-      <c r="H994" s="19"/>
-      <c r="I994" s="19"/>
+      <c r="A994" s="20"/>
+      <c r="B994" s="20"/>
+      <c r="C994" s="20"/>
+      <c r="D994" s="20"/>
+      <c r="E994" s="20"/>
+      <c r="F994" s="20"/>
+      <c r="G994" s="20"/>
+      <c r="H994" s="20"/>
+      <c r="I994" s="20"/>
     </row>
     <row r="995" ht="15.75" customHeight="1">
-      <c r="A995" s="19"/>
-      <c r="B995" s="19"/>
-      <c r="C995" s="19"/>
-      <c r="D995" s="19"/>
-      <c r="E995" s="19"/>
-      <c r="F995" s="19"/>
-      <c r="G995" s="19"/>
-      <c r="H995" s="19"/>
-      <c r="I995" s="19"/>
+      <c r="A995" s="20"/>
+      <c r="B995" s="20"/>
+      <c r="C995" s="20"/>
+      <c r="D995" s="20"/>
+      <c r="E995" s="20"/>
+      <c r="F995" s="20"/>
+      <c r="G995" s="20"/>
+      <c r="H995" s="20"/>
+      <c r="I995" s="20"/>
     </row>
     <row r="996" ht="15.75" customHeight="1">
-      <c r="A996" s="19"/>
-      <c r="B996" s="19"/>
-      <c r="C996" s="19"/>
-      <c r="D996" s="19"/>
-      <c r="E996" s="19"/>
-      <c r="F996" s="19"/>
-      <c r="G996" s="19"/>
-      <c r="H996" s="19"/>
-      <c r="I996" s="19"/>
+      <c r="A996" s="20"/>
+      <c r="B996" s="20"/>
+      <c r="C996" s="20"/>
+      <c r="D996" s="20"/>
+      <c r="E996" s="20"/>
+      <c r="F996" s="20"/>
+      <c r="G996" s="20"/>
+      <c r="H996" s="20"/>
+      <c r="I996" s="20"/>
     </row>
     <row r="997" ht="15.75" customHeight="1">
-      <c r="A997" s="19"/>
-      <c r="B997" s="19"/>
-      <c r="C997" s="19"/>
-      <c r="D997" s="19"/>
-      <c r="E997" s="19"/>
-      <c r="F997" s="19"/>
-      <c r="G997" s="19"/>
-      <c r="H997" s="19"/>
-      <c r="I997" s="19"/>
+      <c r="A997" s="20"/>
+      <c r="B997" s="20"/>
+      <c r="C997" s="20"/>
+      <c r="D997" s="20"/>
+      <c r="E997" s="20"/>
+      <c r="F997" s="20"/>
+      <c r="G997" s="20"/>
+      <c r="H997" s="20"/>
+      <c r="I997" s="20"/>
     </row>
     <row r="998" ht="15.75" customHeight="1">
-      <c r="A998" s="19"/>
-      <c r="B998" s="19"/>
-      <c r="C998" s="19"/>
-      <c r="D998" s="19"/>
-      <c r="E998" s="19"/>
-      <c r="F998" s="19"/>
-      <c r="G998" s="19"/>
-      <c r="H998" s="19"/>
-      <c r="I998" s="19"/>
+      <c r="A998" s="20"/>
+      <c r="B998" s="20"/>
+      <c r="C998" s="20"/>
+      <c r="D998" s="20"/>
+      <c r="E998" s="20"/>
+      <c r="F998" s="20"/>
+      <c r="G998" s="20"/>
+      <c r="H998" s="20"/>
+      <c r="I998" s="20"/>
     </row>
     <row r="999" ht="15.75" customHeight="1">
-      <c r="A999" s="19"/>
-      <c r="B999" s="19"/>
-      <c r="C999" s="19"/>
-      <c r="D999" s="19"/>
-      <c r="E999" s="19"/>
-      <c r="F999" s="19"/>
-      <c r="G999" s="19"/>
-      <c r="H999" s="19"/>
-      <c r="I999" s="19"/>
+      <c r="A999" s="20"/>
+      <c r="B999" s="20"/>
+      <c r="C999" s="20"/>
+      <c r="D999" s="20"/>
+      <c r="E999" s="20"/>
+      <c r="F999" s="20"/>
+      <c r="G999" s="20"/>
+      <c r="H999" s="20"/>
+      <c r="I999" s="20"/>
     </row>
     <row r="1000" ht="15.75" customHeight="1">
-      <c r="A1000" s="19"/>
-      <c r="B1000" s="19"/>
-      <c r="C1000" s="19"/>
-      <c r="D1000" s="19"/>
-      <c r="E1000" s="19"/>
-      <c r="F1000" s="19"/>
-      <c r="G1000" s="19"/>
-      <c r="H1000" s="19"/>
-      <c r="I1000" s="19"/>
+      <c r="A1000" s="20"/>
+      <c r="B1000" s="20"/>
+      <c r="C1000" s="20"/>
+      <c r="D1000" s="20"/>
+      <c r="E1000" s="20"/>
+      <c r="F1000" s="20"/>
+      <c r="G1000" s="20"/>
+      <c r="H1000" s="20"/>
+      <c r="I1000" s="20"/>
     </row>
   </sheetData>
   <dataValidations>

</xml_diff>

<commit_message>
última actualización dashboard con implementación de script que actualiza NB1 y NB2
</commit_message>
<xml_diff>
--- a/data/raw/io_data_bimbo.xlsx
+++ b/data/raw/io_data_bimbo.xlsx
@@ -23952,587 +23952,1541 @@
       </c>
     </row>
     <row r="812" ht="15.75" customHeight="1">
-      <c r="A812" s="3"/>
-      <c r="B812" s="4"/>
-      <c r="C812" s="8"/>
-      <c r="D812" s="8"/>
-      <c r="E812" s="5"/>
-      <c r="F812" s="5"/>
-      <c r="G812" s="20"/>
-      <c r="H812" s="12"/>
-      <c r="I812" s="20"/>
+      <c r="A812" s="13">
+        <v>46240.0</v>
+      </c>
+      <c r="B812" s="14">
+        <v>8256.0</v>
+      </c>
+      <c r="C812" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D812" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E812" s="16">
+        <v>0.6532175925925926</v>
+      </c>
+      <c r="F812" s="16">
+        <v>0.6552314814814815</v>
+      </c>
+      <c r="G812" s="19">
+        <v>0.24584490740740605</v>
+      </c>
+      <c r="H812" s="17">
+        <v>130.0</v>
+      </c>
+      <c r="I812" s="11">
+        <v>1224210.0</v>
+      </c>
     </row>
     <row r="813" ht="15.75" customHeight="1">
-      <c r="A813" s="3"/>
-      <c r="B813" s="4"/>
-      <c r="C813" s="8"/>
-      <c r="D813" s="8"/>
-      <c r="E813" s="5"/>
-      <c r="F813" s="5"/>
-      <c r="G813" s="20"/>
-      <c r="H813" s="12"/>
-      <c r="I813" s="20"/>
+      <c r="A813" s="13">
+        <v>46240.0</v>
+      </c>
+      <c r="B813" s="14">
+        <v>8263.0</v>
+      </c>
+      <c r="C813" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D813" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E813" s="16">
+        <v>0.6569097222222222</v>
+      </c>
+      <c r="F813" s="16">
+        <v>0.7088310185185185</v>
+      </c>
+      <c r="G813" s="19">
+        <v>0.24584490740740605</v>
+      </c>
+      <c r="H813" s="17">
+        <v>5230.0</v>
+      </c>
+      <c r="I813" s="11">
+        <v>2.2303442E7</v>
+      </c>
     </row>
     <row r="814" ht="15.75" customHeight="1">
-      <c r="A814" s="3"/>
-      <c r="B814" s="4"/>
-      <c r="C814" s="8"/>
-      <c r="D814" s="8"/>
-      <c r="E814" s="5"/>
-      <c r="F814" s="5"/>
-      <c r="G814" s="20"/>
-      <c r="H814" s="12"/>
-      <c r="I814" s="20"/>
+      <c r="A814" s="13">
+        <v>46240.0</v>
+      </c>
+      <c r="B814" s="14">
+        <v>9305.0</v>
+      </c>
+      <c r="C814" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D814" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E814" s="16">
+        <v>0.7248958333333333</v>
+      </c>
+      <c r="F814" s="16">
+        <v>0.7285532407407408</v>
+      </c>
+      <c r="G814" s="19">
+        <v>0.24584490740740605</v>
+      </c>
+      <c r="H814" s="17">
+        <v>165.0</v>
+      </c>
+      <c r="I814" s="11">
+        <v>938436.0</v>
+      </c>
     </row>
     <row r="815" ht="15.75" customHeight="1">
-      <c r="A815" s="3"/>
-      <c r="B815" s="4"/>
-      <c r="C815" s="8"/>
-      <c r="D815" s="8"/>
-      <c r="E815" s="5"/>
-      <c r="F815" s="5"/>
-      <c r="G815" s="20"/>
-      <c r="H815" s="12"/>
-      <c r="I815" s="20"/>
+      <c r="A815" s="13">
+        <v>46240.0</v>
+      </c>
+      <c r="B815" s="14">
+        <v>9310.0</v>
+      </c>
+      <c r="C815" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D815" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E815" s="16">
+        <v>0.729375</v>
+      </c>
+      <c r="F815" s="16">
+        <v>0.7378125</v>
+      </c>
+      <c r="G815" s="19">
+        <v>0.24584490740740605</v>
+      </c>
+      <c r="H815" s="17">
+        <v>457.0</v>
+      </c>
+      <c r="I815" s="11">
+        <v>3973390.0</v>
+      </c>
     </row>
     <row r="816" ht="15.75" customHeight="1">
-      <c r="A816" s="3"/>
-      <c r="B816" s="4"/>
-      <c r="C816" s="8"/>
-      <c r="D816" s="8"/>
-      <c r="E816" s="5"/>
-      <c r="F816" s="5"/>
-      <c r="G816" s="20"/>
-      <c r="H816" s="12"/>
-      <c r="I816" s="20"/>
+      <c r="A816" s="13">
+        <v>46240.0</v>
+      </c>
+      <c r="B816" s="14">
+        <v>9311.0</v>
+      </c>
+      <c r="C816" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D816" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E816" s="16">
+        <v>0.7421875</v>
+      </c>
+      <c r="F816" s="16">
+        <v>0.7479745370370371</v>
+      </c>
+      <c r="G816" s="19">
+        <v>0.24584490740740605</v>
+      </c>
+      <c r="H816" s="17">
+        <v>20.0</v>
+      </c>
+      <c r="I816" s="11">
+        <v>190186.0</v>
+      </c>
     </row>
     <row r="817" ht="15.75" customHeight="1">
-      <c r="A817" s="3"/>
-      <c r="B817" s="4"/>
-      <c r="C817" s="8"/>
-      <c r="D817" s="8"/>
-      <c r="E817" s="5"/>
-      <c r="F817" s="5"/>
-      <c r="G817" s="20"/>
-      <c r="H817" s="12"/>
-      <c r="I817" s="20"/>
+      <c r="A817" s="13">
+        <v>46240.0</v>
+      </c>
+      <c r="B817" s="14">
+        <v>9320.0</v>
+      </c>
+      <c r="C817" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D817" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E817" s="16">
+        <v>0.748912037037037</v>
+      </c>
+      <c r="F817" s="16">
+        <v>0.7544560185185185</v>
+      </c>
+      <c r="G817" s="19">
+        <v>0.24584490740740605</v>
+      </c>
+      <c r="H817" s="17">
+        <v>96.0</v>
+      </c>
+      <c r="I817" s="11">
+        <v>835396.0</v>
+      </c>
     </row>
     <row r="818" ht="15.75" customHeight="1">
-      <c r="A818" s="3"/>
-      <c r="B818" s="4"/>
-      <c r="C818" s="8"/>
-      <c r="D818" s="8"/>
-      <c r="E818" s="5"/>
-      <c r="F818" s="5"/>
-      <c r="G818" s="20"/>
-      <c r="H818" s="12"/>
-      <c r="I818" s="20"/>
+      <c r="A818" s="13">
+        <v>46240.0</v>
+      </c>
+      <c r="B818" s="14">
+        <v>9326.0</v>
+      </c>
+      <c r="C818" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D818" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E818" s="16">
+        <v>0.7558564814814814</v>
+      </c>
+      <c r="F818" s="16">
+        <v>0.7613657407407407</v>
+      </c>
+      <c r="G818" s="19">
+        <v>0.24584490740740605</v>
+      </c>
+      <c r="H818" s="17">
+        <v>191.0</v>
+      </c>
+      <c r="I818" s="11">
+        <v>1801978.0</v>
+      </c>
     </row>
     <row r="819" ht="15.75" customHeight="1">
-      <c r="A819" s="3"/>
-      <c r="B819" s="4"/>
-      <c r="C819" s="8"/>
-      <c r="D819" s="8"/>
-      <c r="E819" s="5"/>
-      <c r="F819" s="5"/>
-      <c r="G819" s="20"/>
-      <c r="H819" s="12"/>
-      <c r="I819" s="20"/>
+      <c r="A819" s="13">
+        <v>46240.0</v>
+      </c>
+      <c r="B819" s="14">
+        <v>9337.0</v>
+      </c>
+      <c r="C819" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D819" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E819" s="16">
+        <v>0.7633680555555555</v>
+      </c>
+      <c r="F819" s="16">
+        <v>0.7657407407407407</v>
+      </c>
+      <c r="G819" s="19">
+        <v>0.24584490740740605</v>
+      </c>
+      <c r="H819" s="17">
+        <v>42.0</v>
+      </c>
+      <c r="I819" s="11">
+        <v>368790.0</v>
+      </c>
     </row>
     <row r="820" ht="15.75" customHeight="1">
-      <c r="A820" s="3"/>
-      <c r="B820" s="4"/>
-      <c r="C820" s="8"/>
-      <c r="D820" s="8"/>
-      <c r="E820" s="5"/>
-      <c r="F820" s="5"/>
-      <c r="G820" s="20"/>
-      <c r="H820" s="12"/>
-      <c r="I820" s="20"/>
+      <c r="A820" s="13">
+        <v>46240.0</v>
+      </c>
+      <c r="B820" s="14">
+        <v>9339.0</v>
+      </c>
+      <c r="C820" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D820" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E820" s="16">
+        <v>0.7669097222222222</v>
+      </c>
+      <c r="F820" s="16">
+        <v>0.7686921296296296</v>
+      </c>
+      <c r="G820" s="19">
+        <v>0.24584490740740605</v>
+      </c>
+      <c r="H820" s="17">
+        <v>30.0</v>
+      </c>
+      <c r="I820" s="11">
+        <v>147510.0</v>
+      </c>
     </row>
     <row r="821" ht="15.75" customHeight="1">
-      <c r="A821" s="3"/>
-      <c r="B821" s="4"/>
-      <c r="C821" s="8"/>
-      <c r="D821" s="8"/>
-      <c r="E821" s="5"/>
-      <c r="F821" s="5"/>
-      <c r="G821" s="20"/>
-      <c r="H821" s="12"/>
-      <c r="I821" s="20"/>
+      <c r="A821" s="13">
+        <v>46240.0</v>
+      </c>
+      <c r="B821" s="14">
+        <v>9340.0</v>
+      </c>
+      <c r="C821" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D821" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E821" s="16">
+        <v>0.7694791666666667</v>
+      </c>
+      <c r="F821" s="16">
+        <v>0.7746296296296297</v>
+      </c>
+      <c r="G821" s="19">
+        <v>0.24584490740740605</v>
+      </c>
+      <c r="H821" s="17">
+        <v>101.0</v>
+      </c>
+      <c r="I821" s="11">
+        <v>905360.0</v>
+      </c>
     </row>
     <row r="822" ht="15.75" customHeight="1">
-      <c r="A822" s="3"/>
-      <c r="B822" s="4"/>
-      <c r="C822" s="8"/>
-      <c r="D822" s="8"/>
-      <c r="E822" s="5"/>
-      <c r="F822" s="5"/>
-      <c r="G822" s="20"/>
-      <c r="H822" s="12"/>
-      <c r="I822" s="20"/>
+      <c r="A822" s="13">
+        <v>46240.0</v>
+      </c>
+      <c r="B822" s="14">
+        <v>9345.0</v>
+      </c>
+      <c r="C822" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D822" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E822" s="16">
+        <v>0.7762731481481482</v>
+      </c>
+      <c r="F822" s="16">
+        <v>0.7788657407407408</v>
+      </c>
+      <c r="G822" s="19">
+        <v>0.24584490740740605</v>
+      </c>
+      <c r="H822" s="17">
+        <v>57.0</v>
+      </c>
+      <c r="I822" s="11">
+        <v>518426.0</v>
+      </c>
     </row>
     <row r="823" ht="15.75" customHeight="1">
-      <c r="A823" s="3"/>
-      <c r="B823" s="4"/>
-      <c r="C823" s="8"/>
-      <c r="D823" s="8"/>
-      <c r="E823" s="5"/>
-      <c r="F823" s="5"/>
-      <c r="G823" s="20"/>
-      <c r="H823" s="12"/>
-      <c r="I823" s="20"/>
+      <c r="A823" s="13">
+        <v>46240.0</v>
+      </c>
+      <c r="B823" s="14">
+        <v>9353.0</v>
+      </c>
+      <c r="C823" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D823" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E823" s="16">
+        <v>0.7797106481481482</v>
+      </c>
+      <c r="F823" s="16">
+        <v>0.7823842592592593</v>
+      </c>
+      <c r="G823" s="19">
+        <v>0.24584490740740605</v>
+      </c>
+      <c r="H823" s="17">
+        <v>190.0</v>
+      </c>
+      <c r="I823" s="11">
+        <v>1225000.0</v>
+      </c>
     </row>
     <row r="824" ht="15.75" customHeight="1">
-      <c r="A824" s="3"/>
-      <c r="B824" s="4"/>
-      <c r="C824" s="8"/>
-      <c r="D824" s="8"/>
-      <c r="E824" s="5"/>
-      <c r="F824" s="5"/>
-      <c r="G824" s="20"/>
-      <c r="H824" s="12"/>
-      <c r="I824" s="20"/>
+      <c r="A824" s="13">
+        <v>46240.0</v>
+      </c>
+      <c r="B824" s="14">
+        <v>9355.0</v>
+      </c>
+      <c r="C824" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D824" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E824" s="16">
+        <v>0.7833217592592593</v>
+      </c>
+      <c r="F824" s="16">
+        <v>0.7850694444444445</v>
+      </c>
+      <c r="G824" s="19">
+        <v>0.24584490740740605</v>
+      </c>
+      <c r="H824" s="17">
+        <v>32.0</v>
+      </c>
+      <c r="I824" s="11">
+        <v>197500.0</v>
+      </c>
     </row>
     <row r="825" ht="15.75" customHeight="1">
-      <c r="A825" s="3"/>
-      <c r="B825" s="4"/>
-      <c r="C825" s="8"/>
-      <c r="D825" s="8"/>
-      <c r="E825" s="5"/>
-      <c r="F825" s="5"/>
-      <c r="G825" s="20"/>
-      <c r="H825" s="12"/>
-      <c r="I825" s="20"/>
+      <c r="A825" s="13">
+        <v>46240.0</v>
+      </c>
+      <c r="B825" s="14">
+        <v>9390.0</v>
+      </c>
+      <c r="C825" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D825" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E825" s="16">
+        <v>0.7858333333333334</v>
+      </c>
+      <c r="F825" s="16">
+        <v>0.7872453703703703</v>
+      </c>
+      <c r="G825" s="19">
+        <v>0.24584490740740605</v>
+      </c>
+      <c r="H825" s="17">
+        <v>18.0</v>
+      </c>
+      <c r="I825" s="11">
+        <v>88506.0</v>
+      </c>
     </row>
     <row r="826" ht="15.75" customHeight="1">
-      <c r="A826" s="3"/>
-      <c r="B826" s="4"/>
-      <c r="C826" s="8"/>
-      <c r="D826" s="8"/>
-      <c r="E826" s="5"/>
-      <c r="F826" s="5"/>
-      <c r="G826" s="20"/>
-      <c r="H826" s="12"/>
-      <c r="I826" s="20"/>
+      <c r="A826" s="13">
+        <v>46240.0</v>
+      </c>
+      <c r="B826" s="14">
+        <v>9420.0</v>
+      </c>
+      <c r="C826" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D826" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E826" s="16">
+        <v>0.7879513888888889</v>
+      </c>
+      <c r="F826" s="16">
+        <v>0.7899884259259259</v>
+      </c>
+      <c r="G826" s="19">
+        <v>0.24584490740740605</v>
+      </c>
+      <c r="H826" s="17">
+        <v>35.0</v>
+      </c>
+      <c r="I826" s="11">
+        <v>339330.0</v>
+      </c>
     </row>
     <row r="827" ht="15.75" customHeight="1">
-      <c r="A827" s="3"/>
-      <c r="B827" s="4"/>
-      <c r="C827" s="8"/>
-      <c r="D827" s="8"/>
-      <c r="E827" s="5"/>
-      <c r="F827" s="5"/>
-      <c r="G827" s="20"/>
-      <c r="H827" s="12"/>
-      <c r="I827" s="20"/>
+      <c r="A827" s="13">
+        <v>46240.0</v>
+      </c>
+      <c r="B827" s="14">
+        <v>9422.0</v>
+      </c>
+      <c r="C827" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D827" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E827" s="16">
+        <v>0.7909027777777777</v>
+      </c>
+      <c r="F827" s="16">
+        <v>0.7929861111111111</v>
+      </c>
+      <c r="G827" s="19">
+        <v>0.24584490740740605</v>
+      </c>
+      <c r="H827" s="17">
+        <v>35.0</v>
+      </c>
+      <c r="I827" s="11">
+        <v>367185.0</v>
+      </c>
     </row>
     <row r="828" ht="15.75" customHeight="1">
-      <c r="A828" s="3"/>
-      <c r="B828" s="4"/>
-      <c r="C828" s="8"/>
-      <c r="D828" s="8"/>
-      <c r="E828" s="5"/>
-      <c r="F828" s="5"/>
-      <c r="G828" s="20"/>
-      <c r="H828" s="12"/>
-      <c r="I828" s="20"/>
+      <c r="A828" s="13">
+        <v>46240.0</v>
+      </c>
+      <c r="B828" s="14">
+        <v>9426.0</v>
+      </c>
+      <c r="C828" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D828" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E828" s="16">
+        <v>0.7938773148148148</v>
+      </c>
+      <c r="F828" s="16">
+        <v>0.7962268518518518</v>
+      </c>
+      <c r="G828" s="19">
+        <v>0.24584490740740605</v>
+      </c>
+      <c r="H828" s="17">
+        <v>80.0</v>
+      </c>
+      <c r="I828" s="11">
+        <v>783570.0</v>
+      </c>
     </row>
     <row r="829" ht="15.75" customHeight="1">
-      <c r="A829" s="3"/>
-      <c r="B829" s="4"/>
-      <c r="C829" s="8"/>
-      <c r="D829" s="8"/>
-      <c r="E829" s="5"/>
-      <c r="F829" s="5"/>
-      <c r="G829" s="20"/>
-      <c r="H829" s="12"/>
-      <c r="I829" s="20"/>
+      <c r="A829" s="13">
+        <v>46240.0</v>
+      </c>
+      <c r="B829" s="14">
+        <v>9424.0</v>
+      </c>
+      <c r="C829" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D829" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E829" s="16">
+        <v>0.7972453703703704</v>
+      </c>
+      <c r="F829" s="16">
+        <v>0.7997222222222222</v>
+      </c>
+      <c r="G829" s="19">
+        <v>0.24584490740740605</v>
+      </c>
+      <c r="H829" s="17">
+        <v>45.0</v>
+      </c>
+      <c r="I829" s="11">
+        <v>416385.0</v>
+      </c>
     </row>
     <row r="830" ht="15.75" customHeight="1">
-      <c r="A830" s="3"/>
-      <c r="B830" s="4"/>
-      <c r="C830" s="8"/>
-      <c r="D830" s="8"/>
-      <c r="E830" s="5"/>
-      <c r="F830" s="5"/>
-      <c r="G830" s="20"/>
-      <c r="H830" s="12"/>
-      <c r="I830" s="20"/>
+      <c r="A830" s="13">
+        <v>46240.0</v>
+      </c>
+      <c r="B830" s="14">
+        <v>9425.0</v>
+      </c>
+      <c r="C830" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D830" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E830" s="16">
+        <v>0.8010532407407407</v>
+      </c>
+      <c r="F830" s="16">
+        <v>0.8028356481481481</v>
+      </c>
+      <c r="G830" s="19">
+        <v>0.24584490740740605</v>
+      </c>
+      <c r="H830" s="17">
+        <v>43.0</v>
+      </c>
+      <c r="I830" s="11">
+        <v>444240.0</v>
+      </c>
     </row>
     <row r="831" ht="15.75" customHeight="1">
-      <c r="A831" s="3"/>
-      <c r="B831" s="4"/>
-      <c r="C831" s="8"/>
-      <c r="D831" s="8"/>
-      <c r="E831" s="5"/>
-      <c r="F831" s="5"/>
-      <c r="G831" s="20"/>
-      <c r="H831" s="12"/>
-      <c r="I831" s="20"/>
+      <c r="A831" s="13">
+        <v>46240.0</v>
+      </c>
+      <c r="B831" s="14">
+        <v>9434.0</v>
+      </c>
+      <c r="C831" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D831" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E831" s="16">
+        <v>0.8037152777777777</v>
+      </c>
+      <c r="F831" s="16">
+        <v>0.8063425925925926</v>
+      </c>
+      <c r="G831" s="19">
+        <v>0.24584490740740605</v>
+      </c>
+      <c r="H831" s="17">
+        <v>61.0</v>
+      </c>
+      <c r="I831" s="11">
+        <v>574270.0</v>
+      </c>
     </row>
     <row r="832" ht="15.75" customHeight="1">
-      <c r="A832" s="3"/>
-      <c r="B832" s="4"/>
-      <c r="C832" s="8"/>
-      <c r="D832" s="8"/>
-      <c r="E832" s="5"/>
-      <c r="F832" s="5"/>
-      <c r="G832" s="20"/>
-      <c r="H832" s="12"/>
-      <c r="I832" s="20"/>
+      <c r="A832" s="13">
+        <v>46240.0</v>
+      </c>
+      <c r="B832" s="14">
+        <v>9435.0</v>
+      </c>
+      <c r="C832" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D832" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E832" s="16">
+        <v>0.8071990740740741</v>
+      </c>
+      <c r="F832" s="16">
+        <v>0.8098958333333334</v>
+      </c>
+      <c r="G832" s="19">
+        <v>0.24584490740740605</v>
+      </c>
+      <c r="H832" s="17">
+        <v>46.0</v>
+      </c>
+      <c r="I832" s="11">
+        <v>951426.0</v>
+      </c>
     </row>
     <row r="833" ht="15.75" customHeight="1">
-      <c r="A833" s="3"/>
-      <c r="B833" s="4"/>
-      <c r="C833" s="8"/>
-      <c r="D833" s="8"/>
-      <c r="E833" s="5"/>
-      <c r="F833" s="5"/>
-      <c r="G833" s="20"/>
-      <c r="H833" s="12"/>
-      <c r="I833" s="20"/>
+      <c r="A833" s="13">
+        <v>46240.0</v>
+      </c>
+      <c r="B833" s="14">
+        <v>307.0</v>
+      </c>
+      <c r="C833" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D833" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E833" s="16">
+        <v>0.8359953703703704</v>
+      </c>
+      <c r="F833" s="16">
+        <v>0.8495949074074074</v>
+      </c>
+      <c r="G833" s="19">
+        <v>0.24584490740740605</v>
+      </c>
+      <c r="H833" s="17">
+        <v>710.0</v>
+      </c>
+      <c r="I833" s="11">
+        <v>1554984.0</v>
+      </c>
     </row>
     <row r="834" ht="15.75" customHeight="1">
-      <c r="A834" s="3"/>
-      <c r="B834" s="4"/>
-      <c r="C834" s="8"/>
-      <c r="D834" s="8"/>
-      <c r="E834" s="5"/>
-      <c r="F834" s="5"/>
-      <c r="G834" s="20"/>
-      <c r="H834" s="12"/>
-      <c r="I834" s="20"/>
+      <c r="A834" s="13">
+        <v>46240.0</v>
+      </c>
+      <c r="B834" s="14">
+        <v>311.0</v>
+      </c>
+      <c r="C834" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D834" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E834" s="16">
+        <v>0.8505787037037037</v>
+      </c>
+      <c r="F834" s="16">
+        <v>0.875462962962963</v>
+      </c>
+      <c r="G834" s="19">
+        <v>0.24584490740740605</v>
+      </c>
+      <c r="H834" s="17">
+        <v>1429.0</v>
+      </c>
+      <c r="I834" s="11">
+        <v>4535549.0</v>
+      </c>
     </row>
     <row r="835" ht="15.75" customHeight="1">
-      <c r="A835" s="3"/>
-      <c r="B835" s="4"/>
-      <c r="C835" s="8"/>
-      <c r="D835" s="8"/>
-      <c r="E835" s="5"/>
-      <c r="F835" s="5"/>
-      <c r="G835" s="20"/>
-      <c r="H835" s="12"/>
-      <c r="I835" s="20"/>
+      <c r="A835" s="13">
+        <v>46240.0</v>
+      </c>
+      <c r="B835" s="14">
+        <v>207.0</v>
+      </c>
+      <c r="C835" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D835" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E835" s="16">
+        <v>0.8772106481481482</v>
+      </c>
+      <c r="F835" s="16">
+        <v>0.8990162037037037</v>
+      </c>
+      <c r="G835" s="19">
+        <v>0.24584490740740605</v>
+      </c>
+      <c r="H835" s="17">
+        <v>1004.0</v>
+      </c>
+      <c r="I835" s="11">
+        <v>2744851.0</v>
+      </c>
     </row>
     <row r="836" ht="15.75" customHeight="1">
-      <c r="A836" s="3"/>
-      <c r="B836" s="4"/>
-      <c r="C836" s="8"/>
-      <c r="D836" s="8"/>
-      <c r="E836" s="5"/>
-      <c r="F836" s="5"/>
-      <c r="G836" s="20"/>
-      <c r="H836" s="12"/>
-      <c r="I836" s="20"/>
+      <c r="A836" s="13">
+        <v>46240.0</v>
+      </c>
+      <c r="B836" s="14">
+        <v>211.0</v>
+      </c>
+      <c r="C836" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D836" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E836" s="16">
+        <v>0.901087962962963</v>
+      </c>
+      <c r="F836" s="16">
+        <v>0.9228356481481481</v>
+      </c>
+      <c r="G836" s="19">
+        <v>0.24584490740740605</v>
+      </c>
+      <c r="H836" s="17">
+        <v>1268.0</v>
+      </c>
+      <c r="I836" s="11">
+        <v>3535892.0</v>
+      </c>
     </row>
     <row r="837" ht="15.75" customHeight="1">
-      <c r="A837" s="3"/>
-      <c r="B837" s="4"/>
-      <c r="C837" s="8"/>
-      <c r="D837" s="8"/>
-      <c r="E837" s="5"/>
-      <c r="F837" s="5"/>
-      <c r="G837" s="20"/>
-      <c r="H837" s="12"/>
-      <c r="I837" s="20"/>
+      <c r="A837" s="13">
+        <v>46240.0</v>
+      </c>
+      <c r="B837" s="14">
+        <v>253.0</v>
+      </c>
+      <c r="C837" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D837" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E837" s="16">
+        <v>0.9247453703703704</v>
+      </c>
+      <c r="F837" s="16">
+        <v>0.9409259259259259</v>
+      </c>
+      <c r="G837" s="19">
+        <v>0.24584490740740605</v>
+      </c>
+      <c r="H837" s="17">
+        <v>851.0</v>
+      </c>
+      <c r="I837" s="11">
+        <v>1994637.0</v>
+      </c>
     </row>
     <row r="838" ht="15.75" customHeight="1">
-      <c r="A838" s="3"/>
-      <c r="B838" s="4"/>
-      <c r="C838" s="8"/>
-      <c r="D838" s="8"/>
-      <c r="E838" s="5"/>
-      <c r="F838" s="5"/>
-      <c r="G838" s="20"/>
-      <c r="H838" s="12"/>
-      <c r="I838" s="20"/>
+      <c r="A838" s="13">
+        <v>46240.0</v>
+      </c>
+      <c r="B838" s="14">
+        <v>258.0</v>
+      </c>
+      <c r="C838" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D838" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E838" s="16">
+        <v>0.9420949074074074</v>
+      </c>
+      <c r="F838" s="16">
+        <v>0.9560763888888889</v>
+      </c>
+      <c r="G838" s="19">
+        <v>0.24584490740740605</v>
+      </c>
+      <c r="H838" s="17">
+        <v>1038.0</v>
+      </c>
+      <c r="I838" s="11">
+        <v>2143189.0</v>
+      </c>
     </row>
     <row r="839" ht="15.75" customHeight="1">
-      <c r="A839" s="3"/>
-      <c r="B839" s="4"/>
-      <c r="C839" s="8"/>
-      <c r="D839" s="8"/>
-      <c r="E839" s="5"/>
-      <c r="F839" s="5"/>
-      <c r="G839" s="20"/>
-      <c r="H839" s="12"/>
-      <c r="I839" s="20"/>
+      <c r="A839" s="13">
+        <v>46240.0</v>
+      </c>
+      <c r="B839" s="14">
+        <v>264.0</v>
+      </c>
+      <c r="C839" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D839" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E839" s="16">
+        <v>0.9575694444444445</v>
+      </c>
+      <c r="F839" s="16">
+        <v>0.9745601851851852</v>
+      </c>
+      <c r="G839" s="19">
+        <v>0.24584490740740605</v>
+      </c>
+      <c r="H839" s="17">
+        <v>1085.0</v>
+      </c>
+      <c r="I839" s="11">
+        <v>2176026.0</v>
+      </c>
     </row>
     <row r="840" ht="15.75" customHeight="1">
-      <c r="A840" s="3"/>
-      <c r="B840" s="4"/>
-      <c r="C840" s="8"/>
-      <c r="D840" s="8"/>
-      <c r="E840" s="5"/>
-      <c r="F840" s="5"/>
-      <c r="G840" s="20"/>
-      <c r="H840" s="12"/>
-      <c r="I840" s="20"/>
+      <c r="A840" s="13">
+        <v>46242.0</v>
+      </c>
+      <c r="B840" s="14">
+        <v>9376.0</v>
+      </c>
+      <c r="C840" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D840" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E840" s="16">
+        <v>0.6288888888888889</v>
+      </c>
+      <c r="F840" s="16">
+        <v>0.6337384259259259</v>
+      </c>
+      <c r="G840" s="19">
+        <v>0.27596064814814625</v>
+      </c>
+      <c r="H840" s="17">
+        <v>98.0</v>
+      </c>
+      <c r="I840" s="11">
+        <v>297340.0</v>
+      </c>
     </row>
     <row r="841" ht="15.75" customHeight="1">
-      <c r="A841" s="3"/>
-      <c r="B841" s="4"/>
-      <c r="C841" s="8"/>
-      <c r="D841" s="8"/>
-      <c r="E841" s="5"/>
-      <c r="F841" s="5"/>
-      <c r="G841" s="20"/>
-      <c r="H841" s="12"/>
-      <c r="I841" s="20"/>
+      <c r="A841" s="13">
+        <v>46242.0</v>
+      </c>
+      <c r="B841" s="14">
+        <v>9375.0</v>
+      </c>
+      <c r="C841" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D841" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E841" s="16">
+        <v>0.6347916666666666</v>
+      </c>
+      <c r="F841" s="16">
+        <v>0.6397337962962963</v>
+      </c>
+      <c r="G841" s="19">
+        <v>0.27596064814814625</v>
+      </c>
+      <c r="H841" s="17">
+        <v>93.0</v>
+      </c>
+      <c r="I841" s="11">
+        <v>318179.0</v>
+      </c>
     </row>
     <row r="842" ht="15.75" customHeight="1">
-      <c r="A842" s="3"/>
-      <c r="B842" s="4"/>
-      <c r="C842" s="8"/>
-      <c r="D842" s="8"/>
-      <c r="E842" s="5"/>
-      <c r="F842" s="5"/>
-      <c r="G842" s="20"/>
-      <c r="H842" s="12"/>
-      <c r="I842" s="20"/>
+      <c r="A842" s="13">
+        <v>46242.0</v>
+      </c>
+      <c r="B842" s="14">
+        <v>8002.0</v>
+      </c>
+      <c r="C842" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D842" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E842" s="16">
+        <v>0.6413657407407407</v>
+      </c>
+      <c r="F842" s="16">
+        <v>0.6565509259259259</v>
+      </c>
+      <c r="G842" s="19">
+        <v>0.27596064814814625</v>
+      </c>
+      <c r="H842" s="17">
+        <v>861.0</v>
+      </c>
+      <c r="I842" s="11">
+        <v>2831325.0</v>
+      </c>
     </row>
     <row r="843" ht="15.75" customHeight="1">
-      <c r="A843" s="3"/>
-      <c r="B843" s="4"/>
-      <c r="C843" s="8"/>
-      <c r="D843" s="8"/>
-      <c r="E843" s="5"/>
-      <c r="F843" s="5"/>
-      <c r="G843" s="20"/>
-      <c r="H843" s="12"/>
-      <c r="I843" s="20"/>
+      <c r="A843" s="13">
+        <v>46242.0</v>
+      </c>
+      <c r="B843" s="14">
+        <v>9378.0</v>
+      </c>
+      <c r="C843" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D843" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E843" s="16">
+        <v>0.659212962962963</v>
+      </c>
+      <c r="F843" s="16">
+        <v>0.6634027777777778</v>
+      </c>
+      <c r="G843" s="19">
+        <v>0.27596064814814625</v>
+      </c>
+      <c r="H843" s="17">
+        <v>128.0</v>
+      </c>
+      <c r="I843" s="11">
+        <v>321824.0</v>
+      </c>
     </row>
     <row r="844" ht="15.75" customHeight="1">
-      <c r="A844" s="3"/>
-      <c r="B844" s="4"/>
-      <c r="C844" s="8"/>
-      <c r="D844" s="8"/>
-      <c r="E844" s="5"/>
-      <c r="F844" s="5"/>
-      <c r="G844" s="20"/>
-      <c r="H844" s="12"/>
-      <c r="I844" s="20"/>
+      <c r="A844" s="13">
+        <v>46242.0</v>
+      </c>
+      <c r="B844" s="14">
+        <v>9379.0</v>
+      </c>
+      <c r="C844" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D844" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E844" s="16">
+        <v>0.6646296296296297</v>
+      </c>
+      <c r="F844" s="16">
+        <v>0.6700694444444445</v>
+      </c>
+      <c r="G844" s="19">
+        <v>0.27596064814814625</v>
+      </c>
+      <c r="H844" s="17">
+        <v>185.0</v>
+      </c>
+      <c r="I844" s="11">
+        <v>378608.0</v>
+      </c>
     </row>
     <row r="845" ht="15.75" customHeight="1">
-      <c r="A845" s="3"/>
-      <c r="B845" s="4"/>
-      <c r="C845" s="8"/>
-      <c r="D845" s="8"/>
-      <c r="E845" s="5"/>
-      <c r="F845" s="5"/>
-      <c r="G845" s="20"/>
-      <c r="H845" s="12"/>
-      <c r="I845" s="20"/>
+      <c r="A845" s="13">
+        <v>46242.0</v>
+      </c>
+      <c r="B845" s="14">
+        <v>9384.0</v>
+      </c>
+      <c r="C845" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D845" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E845" s="16">
+        <v>0.6709837962962963</v>
+      </c>
+      <c r="F845" s="16">
+        <v>0.6753587962962962</v>
+      </c>
+      <c r="G845" s="19">
+        <v>0.27596064814814625</v>
+      </c>
+      <c r="H845" s="17">
+        <v>85.0</v>
+      </c>
+      <c r="I845" s="11">
+        <v>295625.0</v>
+      </c>
     </row>
     <row r="846" ht="15.75" customHeight="1">
-      <c r="A846" s="3"/>
-      <c r="B846" s="4"/>
-      <c r="C846" s="8"/>
-      <c r="D846" s="8"/>
-      <c r="E846" s="5"/>
-      <c r="F846" s="5"/>
-      <c r="G846" s="20"/>
-      <c r="H846" s="12"/>
-      <c r="I846" s="20"/>
+      <c r="A846" s="13">
+        <v>46242.0</v>
+      </c>
+      <c r="B846" s="14">
+        <v>9386.0</v>
+      </c>
+      <c r="C846" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D846" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E846" s="16">
+        <v>0.6761805555555556</v>
+      </c>
+      <c r="F846" s="16">
+        <v>0.6809490740740741</v>
+      </c>
+      <c r="G846" s="19">
+        <v>0.27596064814814625</v>
+      </c>
+      <c r="H846" s="17">
+        <v>116.0</v>
+      </c>
+      <c r="I846" s="11">
+        <v>372609.0</v>
+      </c>
     </row>
     <row r="847" ht="15.75" customHeight="1">
-      <c r="A847" s="3"/>
-      <c r="B847" s="4"/>
-      <c r="C847" s="8"/>
-      <c r="D847" s="8"/>
-      <c r="E847" s="5"/>
-      <c r="F847" s="5"/>
-      <c r="G847" s="20"/>
-      <c r="H847" s="12"/>
-      <c r="I847" s="20"/>
+      <c r="A847" s="13">
+        <v>46242.0</v>
+      </c>
+      <c r="B847" s="14">
+        <v>9390.0</v>
+      </c>
+      <c r="C847" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D847" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E847" s="16">
+        <v>0.6821180555555556</v>
+      </c>
+      <c r="F847" s="16">
+        <v>0.6859490740740741</v>
+      </c>
+      <c r="G847" s="19">
+        <v>0.27596064814814625</v>
+      </c>
+      <c r="H847" s="17">
+        <v>80.0</v>
+      </c>
+      <c r="I847" s="11">
+        <v>266768.0</v>
+      </c>
     </row>
     <row r="848" ht="15.75" customHeight="1">
-      <c r="A848" s="3"/>
-      <c r="B848" s="4"/>
-      <c r="C848" s="8"/>
-      <c r="D848" s="8"/>
-      <c r="E848" s="5"/>
-      <c r="F848" s="5"/>
-      <c r="G848" s="20"/>
-      <c r="H848" s="12"/>
-      <c r="I848" s="20"/>
+      <c r="A848" s="13">
+        <v>46242.0</v>
+      </c>
+      <c r="B848" s="14">
+        <v>7603.0</v>
+      </c>
+      <c r="C848" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D848" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E848" s="16">
+        <v>0.6869791666666667</v>
+      </c>
+      <c r="F848" s="16">
+        <v>0.7018402777777778</v>
+      </c>
+      <c r="G848" s="19">
+        <v>0.27596064814814625</v>
+      </c>
+      <c r="H848" s="17">
+        <v>364.0</v>
+      </c>
+      <c r="I848" s="11">
+        <v>2256276.0</v>
+      </c>
     </row>
     <row r="849" ht="15.75" customHeight="1">
-      <c r="A849" s="3"/>
-      <c r="B849" s="4"/>
-      <c r="C849" s="8"/>
-      <c r="D849" s="8"/>
-      <c r="E849" s="5"/>
-      <c r="F849" s="5"/>
-      <c r="G849" s="20"/>
-      <c r="H849" s="12"/>
-      <c r="I849" s="20"/>
+      <c r="A849" s="13">
+        <v>46242.0</v>
+      </c>
+      <c r="B849" s="14">
+        <v>7606.0</v>
+      </c>
+      <c r="C849" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D849" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E849" s="16">
+        <v>0.7039930555555556</v>
+      </c>
+      <c r="F849" s="16">
+        <v>0.7129166666666666</v>
+      </c>
+      <c r="G849" s="19">
+        <v>0.27596064814814625</v>
+      </c>
+      <c r="H849" s="17">
+        <v>211.0</v>
+      </c>
+      <c r="I849" s="11">
+        <v>1192705.0</v>
+      </c>
     </row>
     <row r="850" ht="15.75" customHeight="1">
-      <c r="A850" s="3"/>
-      <c r="B850" s="4"/>
-      <c r="C850" s="8"/>
-      <c r="D850" s="8"/>
-      <c r="E850" s="5"/>
-      <c r="F850" s="5"/>
-      <c r="G850" s="20"/>
-      <c r="H850" s="12"/>
-      <c r="I850" s="20"/>
+      <c r="A850" s="13">
+        <v>46242.0</v>
+      </c>
+      <c r="B850" s="14">
+        <v>7613.0</v>
+      </c>
+      <c r="C850" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D850" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E850" s="16">
+        <v>0.713912037037037</v>
+      </c>
+      <c r="F850" s="16">
+        <v>0.7344444444444445</v>
+      </c>
+      <c r="G850" s="19">
+        <v>0.27596064814814625</v>
+      </c>
+      <c r="H850" s="17">
+        <v>967.0</v>
+      </c>
+      <c r="I850" s="11">
+        <v>4808405.0</v>
+      </c>
     </row>
     <row r="851" ht="15.75" customHeight="1">
-      <c r="A851" s="3"/>
-      <c r="B851" s="4"/>
-      <c r="C851" s="8"/>
-      <c r="D851" s="8"/>
-      <c r="E851" s="5"/>
-      <c r="F851" s="5"/>
-      <c r="G851" s="20"/>
-      <c r="H851" s="12"/>
-      <c r="I851" s="20"/>
+      <c r="A851" s="13">
+        <v>46242.0</v>
+      </c>
+      <c r="B851" s="14">
+        <v>7628.0</v>
+      </c>
+      <c r="C851" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D851" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E851" s="16">
+        <v>0.7373032407407407</v>
+      </c>
+      <c r="F851" s="16">
+        <v>0.7464814814814815</v>
+      </c>
+      <c r="G851" s="19">
+        <v>0.27596064814814625</v>
+      </c>
+      <c r="H851" s="17">
+        <v>238.0</v>
+      </c>
+      <c r="I851" s="11">
+        <v>1081393.0</v>
+      </c>
     </row>
     <row r="852" ht="15.75" customHeight="1">
-      <c r="A852" s="3"/>
-      <c r="B852" s="4"/>
-      <c r="C852" s="8"/>
-      <c r="D852" s="8"/>
-      <c r="E852" s="5"/>
-      <c r="F852" s="5"/>
-      <c r="G852" s="20"/>
-      <c r="H852" s="12"/>
-      <c r="I852" s="20"/>
+      <c r="A852" s="13">
+        <v>46242.0</v>
+      </c>
+      <c r="B852" s="14">
+        <v>7644.0</v>
+      </c>
+      <c r="C852" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D852" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E852" s="16">
+        <v>0.7485069444444444</v>
+      </c>
+      <c r="F852" s="16">
+        <v>0.7569791666666666</v>
+      </c>
+      <c r="G852" s="19">
+        <v>0.27596064814814625</v>
+      </c>
+      <c r="H852" s="17">
+        <v>218.0</v>
+      </c>
+      <c r="I852" s="11">
+        <v>890981.0</v>
+      </c>
     </row>
     <row r="853" ht="15.75" customHeight="1">
-      <c r="A853" s="3"/>
-      <c r="B853" s="4"/>
-      <c r="C853" s="8"/>
-      <c r="D853" s="8"/>
-      <c r="E853" s="5"/>
-      <c r="F853" s="5"/>
-      <c r="G853" s="20"/>
-      <c r="H853" s="12"/>
-      <c r="I853" s="20"/>
+      <c r="A853" s="13">
+        <v>46242.0</v>
+      </c>
+      <c r="B853" s="14">
+        <v>7648.0</v>
+      </c>
+      <c r="C853" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D853" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E853" s="18">
+        <v>0.7580787037037037</v>
+      </c>
+      <c r="F853" s="16">
+        <v>0.7652777777777777</v>
+      </c>
+      <c r="G853" s="19">
+        <v>0.27596064814814625</v>
+      </c>
+      <c r="H853" s="17">
+        <v>102.0</v>
+      </c>
+      <c r="I853" s="11">
+        <v>476669.0</v>
+      </c>
     </row>
     <row r="854" ht="15.75" customHeight="1">
-      <c r="A854" s="3"/>
-      <c r="B854" s="4"/>
-      <c r="C854" s="8"/>
-      <c r="D854" s="8"/>
-      <c r="E854" s="5"/>
-      <c r="F854" s="5"/>
-      <c r="G854" s="20"/>
-      <c r="H854" s="12"/>
-      <c r="I854" s="20"/>
+      <c r="A854" s="13">
+        <v>46242.0</v>
+      </c>
+      <c r="B854" s="14">
+        <v>7664.0</v>
+      </c>
+      <c r="C854" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D854" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E854" s="16">
+        <v>0.7663541666666667</v>
+      </c>
+      <c r="F854" s="16">
+        <v>0.7759143518518519</v>
+      </c>
+      <c r="G854" s="19">
+        <v>0.27596064814814625</v>
+      </c>
+      <c r="H854" s="17">
+        <v>222.0</v>
+      </c>
+      <c r="I854" s="11">
+        <v>857497.0</v>
+      </c>
     </row>
     <row r="855" ht="15.75" customHeight="1">
-      <c r="A855" s="3"/>
-      <c r="B855" s="4"/>
-      <c r="C855" s="8"/>
-      <c r="D855" s="8"/>
-      <c r="E855" s="5"/>
-      <c r="F855" s="5"/>
-      <c r="G855" s="20"/>
-      <c r="H855" s="12"/>
-      <c r="I855" s="20"/>
+      <c r="A855" s="13">
+        <v>46242.0</v>
+      </c>
+      <c r="B855" s="14">
+        <v>7656.0</v>
+      </c>
+      <c r="C855" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D855" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E855" s="16">
+        <v>0.7769212962962962</v>
+      </c>
+      <c r="F855" s="16">
+        <v>0.7824074074074074</v>
+      </c>
+      <c r="G855" s="19">
+        <v>0.27596064814814625</v>
+      </c>
+      <c r="H855" s="17">
+        <v>101.0</v>
+      </c>
+      <c r="I855" s="11">
+        <v>382900.0</v>
+      </c>
     </row>
     <row r="856" ht="15.75" customHeight="1">
-      <c r="A856" s="3"/>
-      <c r="B856" s="4"/>
-      <c r="C856" s="8"/>
-      <c r="D856" s="8"/>
-      <c r="E856" s="5"/>
-      <c r="F856" s="5"/>
-      <c r="G856" s="20"/>
-      <c r="H856" s="12"/>
-      <c r="I856" s="20"/>
+      <c r="A856" s="13">
+        <v>46242.0</v>
+      </c>
+      <c r="B856" s="14">
+        <v>7674.0</v>
+      </c>
+      <c r="C856" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D856" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E856" s="16">
+        <v>0.7850810185185185</v>
+      </c>
+      <c r="F856" s="16">
+        <v>0.7883796296296296</v>
+      </c>
+      <c r="G856" s="19">
+        <v>0.27596064814814625</v>
+      </c>
+      <c r="H856" s="17">
+        <v>286.0</v>
+      </c>
+      <c r="I856" s="11">
+        <v>3592668.0</v>
+      </c>
     </row>
     <row r="857" ht="15.75" customHeight="1">
-      <c r="A857" s="3"/>
-      <c r="B857" s="4"/>
-      <c r="C857" s="8"/>
-      <c r="D857" s="8"/>
-      <c r="E857" s="5"/>
-      <c r="F857" s="5"/>
-      <c r="G857" s="20"/>
-      <c r="H857" s="12"/>
-      <c r="I857" s="20"/>
+      <c r="A857" s="13">
+        <v>46242.0</v>
+      </c>
+      <c r="B857" s="14">
+        <v>7691.0</v>
+      </c>
+      <c r="C857" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D857" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E857" s="16">
+        <v>0.7934837962962963</v>
+      </c>
+      <c r="F857" s="16">
+        <v>0.804375</v>
+      </c>
+      <c r="G857" s="19">
+        <v>0.27596064814814625</v>
+      </c>
+      <c r="H857" s="17">
+        <v>332.0</v>
+      </c>
+      <c r="I857" s="11">
+        <v>1731497.0</v>
+      </c>
     </row>
     <row r="858" ht="15.75" customHeight="1">
-      <c r="A858" s="3"/>
-      <c r="B858" s="4"/>
-      <c r="C858" s="8"/>
-      <c r="D858" s="8"/>
-      <c r="E858" s="5"/>
-      <c r="F858" s="5"/>
-      <c r="G858" s="20"/>
-      <c r="H858" s="12"/>
-      <c r="I858" s="20"/>
+      <c r="A858" s="13">
+        <v>46242.0</v>
+      </c>
+      <c r="B858" s="14">
+        <v>7732.0</v>
+      </c>
+      <c r="C858" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D858" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E858" s="16">
+        <v>0.8058333333333333</v>
+      </c>
+      <c r="F858" s="16">
+        <v>0.8144097222222222</v>
+      </c>
+      <c r="G858" s="19">
+        <v>0.27596064814814625</v>
+      </c>
+      <c r="H858" s="17">
+        <v>162.0</v>
+      </c>
+      <c r="I858" s="11">
+        <v>752432.0</v>
+      </c>
     </row>
     <row r="859" ht="15.75" customHeight="1">
-      <c r="A859" s="3"/>
-      <c r="B859" s="4"/>
-      <c r="C859" s="8"/>
-      <c r="D859" s="8"/>
-      <c r="E859" s="5"/>
-      <c r="F859" s="5"/>
-      <c r="G859" s="20"/>
-      <c r="H859" s="12"/>
-      <c r="I859" s="20"/>
+      <c r="A859" s="13">
+        <v>46242.0</v>
+      </c>
+      <c r="B859" s="14">
+        <v>307.0</v>
+      </c>
+      <c r="C859" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D859" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E859" s="16">
+        <v>0.8418981481481481</v>
+      </c>
+      <c r="F859" s="16">
+        <v>0.856412037037037</v>
+      </c>
+      <c r="G859" s="19">
+        <v>0.27596064814814625</v>
+      </c>
+      <c r="H859" s="17">
+        <v>845.0</v>
+      </c>
+      <c r="I859" s="11">
+        <v>1942065.0</v>
+      </c>
     </row>
     <row r="860" ht="15.75" customHeight="1">
-      <c r="A860" s="3"/>
-      <c r="B860" s="4"/>
-      <c r="C860" s="8"/>
-      <c r="D860" s="8"/>
-      <c r="E860" s="5"/>
-      <c r="F860" s="5"/>
-      <c r="G860" s="20"/>
-      <c r="H860" s="12"/>
-      <c r="I860" s="20"/>
+      <c r="A860" s="13">
+        <v>46242.0</v>
+      </c>
+      <c r="B860" s="14">
+        <v>310.0</v>
+      </c>
+      <c r="C860" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D860" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E860" s="16">
+        <v>0.8577430555555555</v>
+      </c>
+      <c r="F860" s="16">
+        <v>0.8725694444444444</v>
+      </c>
+      <c r="G860" s="19">
+        <v>0.27596064814814625</v>
+      </c>
+      <c r="H860" s="17">
+        <v>1004.0</v>
+      </c>
+      <c r="I860" s="11">
+        <v>2212242.0</v>
+      </c>
     </row>
     <row r="861" ht="15.75" customHeight="1">
-      <c r="A861" s="3"/>
-      <c r="B861" s="4"/>
-      <c r="C861" s="8"/>
-      <c r="D861" s="8"/>
-      <c r="E861" s="5"/>
-      <c r="F861" s="5"/>
-      <c r="G861" s="20"/>
-      <c r="H861" s="12"/>
-      <c r="I861" s="20"/>
+      <c r="A861" s="13">
+        <v>46242.0</v>
+      </c>
+      <c r="B861" s="14">
+        <v>201.0</v>
+      </c>
+      <c r="C861" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D861" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E861" s="16">
+        <v>0.8745717592592592</v>
+      </c>
+      <c r="F861" s="16">
+        <v>0.8967361111111111</v>
+      </c>
+      <c r="G861" s="19">
+        <v>0.27596064814814625</v>
+      </c>
+      <c r="H861" s="17">
+        <v>1242.0</v>
+      </c>
+      <c r="I861" s="11">
+        <v>3158208.0</v>
+      </c>
     </row>
     <row r="862" ht="15.75" customHeight="1">
-      <c r="A862" s="3"/>
-      <c r="B862" s="4"/>
-      <c r="C862" s="8"/>
-      <c r="D862" s="8"/>
-      <c r="E862" s="5"/>
-      <c r="F862" s="5"/>
-      <c r="G862" s="20"/>
-      <c r="H862" s="12"/>
-      <c r="I862" s="20"/>
+      <c r="A862" s="13">
+        <v>46242.0</v>
+      </c>
+      <c r="B862" s="14">
+        <v>212.0</v>
+      </c>
+      <c r="C862" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D862" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E862" s="16">
+        <v>0.8990277777777778</v>
+      </c>
+      <c r="F862" s="16">
+        <v>0.9223263888888888</v>
+      </c>
+      <c r="G862" s="19">
+        <v>0.27596064814814625</v>
+      </c>
+      <c r="H862" s="17">
+        <v>933.0</v>
+      </c>
+      <c r="I862" s="11">
+        <v>3609963.0</v>
+      </c>
     </row>
     <row r="863" ht="15.75" customHeight="1">
-      <c r="A863" s="3"/>
-      <c r="B863" s="4"/>
-      <c r="C863" s="8"/>
-      <c r="D863" s="8"/>
-      <c r="E863" s="5"/>
-      <c r="F863" s="5"/>
-      <c r="G863" s="20"/>
-      <c r="H863" s="12"/>
-      <c r="I863" s="20"/>
+      <c r="A863" s="13">
+        <v>46242.0</v>
+      </c>
+      <c r="B863" s="14">
+        <v>256.0</v>
+      </c>
+      <c r="C863" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D863" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E863" s="16">
+        <v>0.9239583333333333</v>
+      </c>
+      <c r="F863" s="16">
+        <v>0.9430439814814815</v>
+      </c>
+      <c r="G863" s="19">
+        <v>0.27596064814814625</v>
+      </c>
+      <c r="H863" s="17">
+        <v>1135.0</v>
+      </c>
+      <c r="I863" s="11">
+        <v>2303576.0</v>
+      </c>
     </row>
     <row r="864" ht="15.75" customHeight="1">
-      <c r="A864" s="3"/>
-      <c r="B864" s="4"/>
-      <c r="C864" s="8"/>
-      <c r="D864" s="8"/>
-      <c r="E864" s="5"/>
-      <c r="F864" s="5"/>
-      <c r="G864" s="20"/>
-      <c r="H864" s="12"/>
-      <c r="I864" s="20"/>
+      <c r="A864" s="13">
+        <v>46242.0</v>
+      </c>
+      <c r="B864" s="14">
+        <v>264.0</v>
+      </c>
+      <c r="C864" s="15">
+        <v>0.625</v>
+      </c>
+      <c r="D864" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="E864" s="16">
+        <v>0.9458680555555555</v>
+      </c>
+      <c r="F864" s="16">
+        <v>0.9733796296296297</v>
+      </c>
+      <c r="G864" s="19">
+        <v>0.27596064814814625</v>
+      </c>
+      <c r="H864" s="17">
+        <v>1534.0</v>
+      </c>
+      <c r="I864" s="11">
+        <v>3636391.0</v>
+      </c>
     </row>
     <row r="865" ht="15.75" customHeight="1">
       <c r="A865" s="3"/>

</xml_diff>